<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 07:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B149A157-022E-4E4B-81A3-37871F4F5AB2}</x14:id>
+          <x14:id>{0CAD9C41-E70A-4439-BA2E-4FED744FE620}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{29B73502-BD12-4DCF-95C5-4FACF1A7692F}</x14:id>
+          <x14:id>{33019606-A41A-4833-84D9-FB077060EB19}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F596AE96-A317-4B49-966B-4F6610595532}</x14:id>
+          <x14:id>{9DB31D83-79D1-4AC2-A7F3-6F60F0C8B437}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F5E2829F-4841-4D90-AE42-CED76A283E31}</x14:id>
+          <x14:id>{AEF046B1-B313-4677-95AC-C0A53C24DB96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B149A157-022E-4E4B-81A3-37871F4F5AB2}">
+          <x14:cfRule type="dataBar" id="{0CAD9C41-E70A-4439-BA2E-4FED744FE620}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{29B73502-BD12-4DCF-95C5-4FACF1A7692F}">
+          <x14:cfRule type="dataBar" id="{33019606-A41A-4833-84D9-FB077060EB19}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F596AE96-A317-4B49-966B-4F6610595532}">
+          <x14:cfRule type="dataBar" id="{9DB31D83-79D1-4AC2-A7F3-6F60F0C8B437}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F5E2829F-4841-4D90-AE42-CED76A283E31}">
+          <x14:cfRule type="dataBar" id="{AEF046B1-B313-4677-95AC-C0A53C24DB96}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{43230FA6-A89C-46E7-8012-ABEF160D6711}</x14:id>
+          <x14:id>{5DA783FF-CA8B-4099-AECF-4BA4B335DDFC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A84A1B9B-6E50-4825-B4AB-E69323E472F7}</x14:id>
+          <x14:id>{9FC4415B-5CBB-4D59-9A47-6AFD9E72D3D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{638C3862-A680-4CC5-856B-F7E9F2A74487}</x14:id>
+          <x14:id>{5988289E-21F1-4DA7-9F4C-19B5323DCA17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7573640E-8C05-46B0-A41C-610A4B54BBFC}</x14:id>
+          <x14:id>{086CCAE2-3CEB-437A-9279-DD1841C054A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{43230FA6-A89C-46E7-8012-ABEF160D6711}">
+          <x14:cfRule type="dataBar" id="{5DA783FF-CA8B-4099-AECF-4BA4B335DDFC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A84A1B9B-6E50-4825-B4AB-E69323E472F7}">
+          <x14:cfRule type="dataBar" id="{9FC4415B-5CBB-4D59-9A47-6AFD9E72D3D1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{638C3862-A680-4CC5-856B-F7E9F2A74487}">
+          <x14:cfRule type="dataBar" id="{5988289E-21F1-4DA7-9F4C-19B5323DCA17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7573640E-8C05-46B0-A41C-610A4B54BBFC}">
+          <x14:cfRule type="dataBar" id="{086CCAE2-3CEB-437A-9279-DD1841C054A7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0CAD9C41-E70A-4439-BA2E-4FED744FE620}</x14:id>
+          <x14:id>{0ACD53B3-B761-4F4D-B015-1B6A15CD8631}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{33019606-A41A-4833-84D9-FB077060EB19}</x14:id>
+          <x14:id>{FC46523F-8CF8-4950-AF4E-F634BD4F1774}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9DB31D83-79D1-4AC2-A7F3-6F60F0C8B437}</x14:id>
+          <x14:id>{D085AD85-641C-40C7-9DD4-EE46E58E7BAD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AEF046B1-B313-4677-95AC-C0A53C24DB96}</x14:id>
+          <x14:id>{11C96272-FAC8-4FE8-AD84-E9B9547DD71B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0CAD9C41-E70A-4439-BA2E-4FED744FE620}">
+          <x14:cfRule type="dataBar" id="{0ACD53B3-B761-4F4D-B015-1B6A15CD8631}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{33019606-A41A-4833-84D9-FB077060EB19}">
+          <x14:cfRule type="dataBar" id="{FC46523F-8CF8-4950-AF4E-F634BD4F1774}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9DB31D83-79D1-4AC2-A7F3-6F60F0C8B437}">
+          <x14:cfRule type="dataBar" id="{D085AD85-641C-40C7-9DD4-EE46E58E7BAD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AEF046B1-B313-4677-95AC-C0A53C24DB96}">
+          <x14:cfRule type="dataBar" id="{11C96272-FAC8-4FE8-AD84-E9B9547DD71B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5DA783FF-CA8B-4099-AECF-4BA4B335DDFC}</x14:id>
+          <x14:id>{92EC6F82-9D83-4AB9-90AB-868B8519574A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FC4415B-5CBB-4D59-9A47-6AFD9E72D3D1}</x14:id>
+          <x14:id>{D170DB9C-DC3A-4164-BDCD-E8484130FC7B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5988289E-21F1-4DA7-9F4C-19B5323DCA17}</x14:id>
+          <x14:id>{0EF5CF08-78C6-4C1A-9DAC-11E2DB380684}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{086CCAE2-3CEB-437A-9279-DD1841C054A7}</x14:id>
+          <x14:id>{41D5AC1B-5540-49E9-A624-2911D653423C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5DA783FF-CA8B-4099-AECF-4BA4B335DDFC}">
+          <x14:cfRule type="dataBar" id="{92EC6F82-9D83-4AB9-90AB-868B8519574A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FC4415B-5CBB-4D59-9A47-6AFD9E72D3D1}">
+          <x14:cfRule type="dataBar" id="{D170DB9C-DC3A-4164-BDCD-E8484130FC7B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5988289E-21F1-4DA7-9F4C-19B5323DCA17}">
+          <x14:cfRule type="dataBar" id="{0EF5CF08-78C6-4C1A-9DAC-11E2DB380684}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{086CCAE2-3CEB-437A-9279-DD1841C054A7}">
+          <x14:cfRule type="dataBar" id="{41D5AC1B-5540-49E9-A624-2911D653423C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0ACD53B3-B761-4F4D-B015-1B6A15CD8631}</x14:id>
+          <x14:id>{FE899157-8EE3-4539-A70C-E36C02FE0CC2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FC46523F-8CF8-4950-AF4E-F634BD4F1774}</x14:id>
+          <x14:id>{7978FB87-581F-433F-BFDA-A91872B51347}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D085AD85-641C-40C7-9DD4-EE46E58E7BAD}</x14:id>
+          <x14:id>{0E382F96-E792-4267-9285-1E7915F971E1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11C96272-FAC8-4FE8-AD84-E9B9547DD71B}</x14:id>
+          <x14:id>{AE35FB0B-ED1B-469A-819D-16C3CE585BC6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0ACD53B3-B761-4F4D-B015-1B6A15CD8631}">
+          <x14:cfRule type="dataBar" id="{FE899157-8EE3-4539-A70C-E36C02FE0CC2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FC46523F-8CF8-4950-AF4E-F634BD4F1774}">
+          <x14:cfRule type="dataBar" id="{7978FB87-581F-433F-BFDA-A91872B51347}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D085AD85-641C-40C7-9DD4-EE46E58E7BAD}">
+          <x14:cfRule type="dataBar" id="{0E382F96-E792-4267-9285-1E7915F971E1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11C96272-FAC8-4FE8-AD84-E9B9547DD71B}">
+          <x14:cfRule type="dataBar" id="{AE35FB0B-ED1B-469A-819D-16C3CE585BC6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{92EC6F82-9D83-4AB9-90AB-868B8519574A}</x14:id>
+          <x14:id>{8E1FD8DA-2E9E-4500-932B-1E1FED259444}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D170DB9C-DC3A-4164-BDCD-E8484130FC7B}</x14:id>
+          <x14:id>{DB5E4302-4DB0-485A-B877-A62B34FB75F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0EF5CF08-78C6-4C1A-9DAC-11E2DB380684}</x14:id>
+          <x14:id>{C6196077-A152-46A2-8DD4-266D76E317CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{41D5AC1B-5540-49E9-A624-2911D653423C}</x14:id>
+          <x14:id>{759F8A91-B7A4-4B4A-A6FB-A52296FD2E08}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{92EC6F82-9D83-4AB9-90AB-868B8519574A}">
+          <x14:cfRule type="dataBar" id="{8E1FD8DA-2E9E-4500-932B-1E1FED259444}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D170DB9C-DC3A-4164-BDCD-E8484130FC7B}">
+          <x14:cfRule type="dataBar" id="{DB5E4302-4DB0-485A-B877-A62B34FB75F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0EF5CF08-78C6-4C1A-9DAC-11E2DB380684}">
+          <x14:cfRule type="dataBar" id="{C6196077-A152-46A2-8DD4-266D76E317CA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{41D5AC1B-5540-49E9-A624-2911D653423C}">
+          <x14:cfRule type="dataBar" id="{759F8A91-B7A4-4B4A-A6FB-A52296FD2E08}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE899157-8EE3-4539-A70C-E36C02FE0CC2}</x14:id>
+          <x14:id>{9A7615AF-9F28-4124-9980-CC5787C641CC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7978FB87-581F-433F-BFDA-A91872B51347}</x14:id>
+          <x14:id>{84225AA6-0559-40E6-8E03-900256017607}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0E382F96-E792-4267-9285-1E7915F971E1}</x14:id>
+          <x14:id>{F7CA045B-12A6-4029-B2AB-0F9E47C2D42F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AE35FB0B-ED1B-469A-819D-16C3CE585BC6}</x14:id>
+          <x14:id>{21C4C153-E9B7-409E-9F1B-26187C193211}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE899157-8EE3-4539-A70C-E36C02FE0CC2}">
+          <x14:cfRule type="dataBar" id="{9A7615AF-9F28-4124-9980-CC5787C641CC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7978FB87-581F-433F-BFDA-A91872B51347}">
+          <x14:cfRule type="dataBar" id="{84225AA6-0559-40E6-8E03-900256017607}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0E382F96-E792-4267-9285-1E7915F971E1}">
+          <x14:cfRule type="dataBar" id="{F7CA045B-12A6-4029-B2AB-0F9E47C2D42F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AE35FB0B-ED1B-469A-819D-16C3CE585BC6}">
+          <x14:cfRule type="dataBar" id="{21C4C153-E9B7-409E-9F1B-26187C193211}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8E1FD8DA-2E9E-4500-932B-1E1FED259444}</x14:id>
+          <x14:id>{8F502E5D-85F0-4CA3-B397-4B1477044CA7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DB5E4302-4DB0-485A-B877-A62B34FB75F5}</x14:id>
+          <x14:id>{C2FDD438-F1A2-4197-940C-BC739BA0F6EB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6196077-A152-46A2-8DD4-266D76E317CA}</x14:id>
+          <x14:id>{EE77BC88-A2F9-4460-B04F-0ECD4A95A7A3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{759F8A91-B7A4-4B4A-A6FB-A52296FD2E08}</x14:id>
+          <x14:id>{8581FDD0-F871-41C0-9794-E97C3059A4ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8E1FD8DA-2E9E-4500-932B-1E1FED259444}">
+          <x14:cfRule type="dataBar" id="{8F502E5D-85F0-4CA3-B397-4B1477044CA7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DB5E4302-4DB0-485A-B877-A62B34FB75F5}">
+          <x14:cfRule type="dataBar" id="{C2FDD438-F1A2-4197-940C-BC739BA0F6EB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6196077-A152-46A2-8DD4-266D76E317CA}">
+          <x14:cfRule type="dataBar" id="{EE77BC88-A2F9-4460-B04F-0ECD4A95A7A3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{759F8A91-B7A4-4B4A-A6FB-A52296FD2E08}">
+          <x14:cfRule type="dataBar" id="{8581FDD0-F871-41C0-9794-E97C3059A4ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9A7615AF-9F28-4124-9980-CC5787C641CC}</x14:id>
+          <x14:id>{68C2C6E8-B045-4AAD-B29D-A461BA3A845C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84225AA6-0559-40E6-8E03-900256017607}</x14:id>
+          <x14:id>{53B4A72D-6339-4034-90CC-8C0C240BC1CD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F7CA045B-12A6-4029-B2AB-0F9E47C2D42F}</x14:id>
+          <x14:id>{B2C5198F-7061-49A3-890D-3392127F26B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{21C4C153-E9B7-409E-9F1B-26187C193211}</x14:id>
+          <x14:id>{92954B10-EE41-4D81-BF72-F8507F76BBF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9A7615AF-9F28-4124-9980-CC5787C641CC}">
+          <x14:cfRule type="dataBar" id="{68C2C6E8-B045-4AAD-B29D-A461BA3A845C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84225AA6-0559-40E6-8E03-900256017607}">
+          <x14:cfRule type="dataBar" id="{53B4A72D-6339-4034-90CC-8C0C240BC1CD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F7CA045B-12A6-4029-B2AB-0F9E47C2D42F}">
+          <x14:cfRule type="dataBar" id="{B2C5198F-7061-49A3-890D-3392127F26B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{21C4C153-E9B7-409E-9F1B-26187C193211}">
+          <x14:cfRule type="dataBar" id="{92954B10-EE41-4D81-BF72-F8507F76BBF6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F502E5D-85F0-4CA3-B397-4B1477044CA7}</x14:id>
+          <x14:id>{244EE6BC-84AA-4616-8D6A-AB2AE508F1BD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C2FDD438-F1A2-4197-940C-BC739BA0F6EB}</x14:id>
+          <x14:id>{5D7ECBAA-00F2-46D8-BA25-26939A56F6DD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE77BC88-A2F9-4460-B04F-0ECD4A95A7A3}</x14:id>
+          <x14:id>{85AB7587-D989-4935-8C21-6A4576710656}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8581FDD0-F871-41C0-9794-E97C3059A4ED}</x14:id>
+          <x14:id>{2F042FC0-CA1C-40EE-B13A-AB9552A5D36F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F502E5D-85F0-4CA3-B397-4B1477044CA7}">
+          <x14:cfRule type="dataBar" id="{244EE6BC-84AA-4616-8D6A-AB2AE508F1BD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C2FDD438-F1A2-4197-940C-BC739BA0F6EB}">
+          <x14:cfRule type="dataBar" id="{5D7ECBAA-00F2-46D8-BA25-26939A56F6DD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE77BC88-A2F9-4460-B04F-0ECD4A95A7A3}">
+          <x14:cfRule type="dataBar" id="{85AB7587-D989-4935-8C21-6A4576710656}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8581FDD0-F871-41C0-9794-E97C3059A4ED}">
+          <x14:cfRule type="dataBar" id="{2F042FC0-CA1C-40EE-B13A-AB9552A5D36F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{68C2C6E8-B045-4AAD-B29D-A461BA3A845C}</x14:id>
+          <x14:id>{9FBE11BA-4D10-43DE-A7EE-9159EE36B7A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53B4A72D-6339-4034-90CC-8C0C240BC1CD}</x14:id>
+          <x14:id>{B7C8F4C2-4051-463A-AA5C-ADB7F53961C6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B2C5198F-7061-49A3-890D-3392127F26B5}</x14:id>
+          <x14:id>{BC9EF45F-45BF-447F-BAE7-E5D7471B9011}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{92954B10-EE41-4D81-BF72-F8507F76BBF6}</x14:id>
+          <x14:id>{B1B04FB5-506C-4A89-B05F-0B854FC730DF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{68C2C6E8-B045-4AAD-B29D-A461BA3A845C}">
+          <x14:cfRule type="dataBar" id="{9FBE11BA-4D10-43DE-A7EE-9159EE36B7A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53B4A72D-6339-4034-90CC-8C0C240BC1CD}">
+          <x14:cfRule type="dataBar" id="{B7C8F4C2-4051-463A-AA5C-ADB7F53961C6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B2C5198F-7061-49A3-890D-3392127F26B5}">
+          <x14:cfRule type="dataBar" id="{BC9EF45F-45BF-447F-BAE7-E5D7471B9011}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{92954B10-EE41-4D81-BF72-F8507F76BBF6}">
+          <x14:cfRule type="dataBar" id="{B1B04FB5-506C-4A89-B05F-0B854FC730DF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{244EE6BC-84AA-4616-8D6A-AB2AE508F1BD}</x14:id>
+          <x14:id>{AD24273D-1DAD-405E-9018-DEF4E6BE6C32}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5D7ECBAA-00F2-46D8-BA25-26939A56F6DD}</x14:id>
+          <x14:id>{B35BA881-7BB7-4F0A-A135-61D896DAE81E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{85AB7587-D989-4935-8C21-6A4576710656}</x14:id>
+          <x14:id>{761AFAF8-1BA8-499A-9F2C-73DB93224A74}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2F042FC0-CA1C-40EE-B13A-AB9552A5D36F}</x14:id>
+          <x14:id>{9AC8271D-45CB-4912-94A1-A3BF5A67AA31}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{244EE6BC-84AA-4616-8D6A-AB2AE508F1BD}">
+          <x14:cfRule type="dataBar" id="{AD24273D-1DAD-405E-9018-DEF4E6BE6C32}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5D7ECBAA-00F2-46D8-BA25-26939A56F6DD}">
+          <x14:cfRule type="dataBar" id="{B35BA881-7BB7-4F0A-A135-61D896DAE81E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{85AB7587-D989-4935-8C21-6A4576710656}">
+          <x14:cfRule type="dataBar" id="{761AFAF8-1BA8-499A-9F2C-73DB93224A74}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2F042FC0-CA1C-40EE-B13A-AB9552A5D36F}">
+          <x14:cfRule type="dataBar" id="{9AC8271D-45CB-4912-94A1-A3BF5A67AA31}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FBE11BA-4D10-43DE-A7EE-9159EE36B7A8}</x14:id>
+          <x14:id>{09BD0845-BEC5-4D7B-B651-6529CA5458B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B7C8F4C2-4051-463A-AA5C-ADB7F53961C6}</x14:id>
+          <x14:id>{0F99F2F5-683A-4211-9E2B-D92BDA099C9A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC9EF45F-45BF-447F-BAE7-E5D7471B9011}</x14:id>
+          <x14:id>{99862413-77F3-4185-BF16-5231954CA795}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B1B04FB5-506C-4A89-B05F-0B854FC730DF}</x14:id>
+          <x14:id>{0B9FAD38-F1CD-4589-A6CB-B038BB7B6105}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FBE11BA-4D10-43DE-A7EE-9159EE36B7A8}">
+          <x14:cfRule type="dataBar" id="{09BD0845-BEC5-4D7B-B651-6529CA5458B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B7C8F4C2-4051-463A-AA5C-ADB7F53961C6}">
+          <x14:cfRule type="dataBar" id="{0F99F2F5-683A-4211-9E2B-D92BDA099C9A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC9EF45F-45BF-447F-BAE7-E5D7471B9011}">
+          <x14:cfRule type="dataBar" id="{99862413-77F3-4185-BF16-5231954CA795}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B1B04FB5-506C-4A89-B05F-0B854FC730DF}">
+          <x14:cfRule type="dataBar" id="{0B9FAD38-F1CD-4589-A6CB-B038BB7B6105}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AD24273D-1DAD-405E-9018-DEF4E6BE6C32}</x14:id>
+          <x14:id>{65B5C461-DF90-4ED5-B648-7D0313AFD8F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B35BA881-7BB7-4F0A-A135-61D896DAE81E}</x14:id>
+          <x14:id>{2C97615E-A028-469A-A680-8877752224B9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{761AFAF8-1BA8-499A-9F2C-73DB93224A74}</x14:id>
+          <x14:id>{09C5BD6B-9D81-4BC0-AA0A-8748142E547E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9AC8271D-45CB-4912-94A1-A3BF5A67AA31}</x14:id>
+          <x14:id>{FE8B372F-BABC-4CC5-B1CB-BD8A949AF8F3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AD24273D-1DAD-405E-9018-DEF4E6BE6C32}">
+          <x14:cfRule type="dataBar" id="{65B5C461-DF90-4ED5-B648-7D0313AFD8F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B35BA881-7BB7-4F0A-A135-61D896DAE81E}">
+          <x14:cfRule type="dataBar" id="{2C97615E-A028-469A-A680-8877752224B9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{761AFAF8-1BA8-499A-9F2C-73DB93224A74}">
+          <x14:cfRule type="dataBar" id="{09C5BD6B-9D81-4BC0-AA0A-8748142E547E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9AC8271D-45CB-4912-94A1-A3BF5A67AA31}">
+          <x14:cfRule type="dataBar" id="{FE8B372F-BABC-4CC5-B1CB-BD8A949AF8F3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{09BD0845-BEC5-4D7B-B651-6529CA5458B5}</x14:id>
+          <x14:id>{939DA7EF-3FDB-49BD-8745-9222DA183469}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F99F2F5-683A-4211-9E2B-D92BDA099C9A}</x14:id>
+          <x14:id>{9D3B833A-2730-470C-B690-F3390CECAE73}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99862413-77F3-4185-BF16-5231954CA795}</x14:id>
+          <x14:id>{E2BA61AA-F509-47FF-8049-50F6F1270697}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B9FAD38-F1CD-4589-A6CB-B038BB7B6105}</x14:id>
+          <x14:id>{15CE0C39-5E68-4A70-940F-4D0228B1A22E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{09BD0845-BEC5-4D7B-B651-6529CA5458B5}">
+          <x14:cfRule type="dataBar" id="{939DA7EF-3FDB-49BD-8745-9222DA183469}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0F99F2F5-683A-4211-9E2B-D92BDA099C9A}">
+          <x14:cfRule type="dataBar" id="{9D3B833A-2730-470C-B690-F3390CECAE73}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99862413-77F3-4185-BF16-5231954CA795}">
+          <x14:cfRule type="dataBar" id="{E2BA61AA-F509-47FF-8049-50F6F1270697}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B9FAD38-F1CD-4589-A6CB-B038BB7B6105}">
+          <x14:cfRule type="dataBar" id="{15CE0C39-5E68-4A70-940F-4D0228B1A22E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{65B5C461-DF90-4ED5-B648-7D0313AFD8F5}</x14:id>
+          <x14:id>{C42550FE-1452-4AF2-B32E-27CA74E055B8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C97615E-A028-469A-A680-8877752224B9}</x14:id>
+          <x14:id>{A8905CDF-3857-4C0A-8338-0BEC6E26480E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{09C5BD6B-9D81-4BC0-AA0A-8748142E547E}</x14:id>
+          <x14:id>{D153B539-E3C1-4F42-86E8-A23A1831068C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE8B372F-BABC-4CC5-B1CB-BD8A949AF8F3}</x14:id>
+          <x14:id>{1CE4F3B7-7E89-4321-BB43-4EC8A245B9B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{65B5C461-DF90-4ED5-B648-7D0313AFD8F5}">
+          <x14:cfRule type="dataBar" id="{C42550FE-1452-4AF2-B32E-27CA74E055B8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C97615E-A028-469A-A680-8877752224B9}">
+          <x14:cfRule type="dataBar" id="{A8905CDF-3857-4C0A-8338-0BEC6E26480E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{09C5BD6B-9D81-4BC0-AA0A-8748142E547E}">
+          <x14:cfRule type="dataBar" id="{D153B539-E3C1-4F42-86E8-A23A1831068C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE8B372F-BABC-4CC5-B1CB-BD8A949AF8F3}">
+          <x14:cfRule type="dataBar" id="{1CE4F3B7-7E89-4321-BB43-4EC8A245B9B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:41Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{939DA7EF-3FDB-49BD-8745-9222DA183469}</x14:id>
+          <x14:id>{3F99C9C5-7E88-44FF-B1A5-C54FC7DD7B94}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9D3B833A-2730-470C-B690-F3390CECAE73}</x14:id>
+          <x14:id>{9FBA0817-4818-43DB-A4F7-A44D183BFBBE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E2BA61AA-F509-47FF-8049-50F6F1270697}</x14:id>
+          <x14:id>{62332EA6-77BC-4CC1-9059-50D62FA5BA22}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{15CE0C39-5E68-4A70-940F-4D0228B1A22E}</x14:id>
+          <x14:id>{25E0BDA6-B547-4D05-BAA7-E8FD7BFD49D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{939DA7EF-3FDB-49BD-8745-9222DA183469}">
+          <x14:cfRule type="dataBar" id="{3F99C9C5-7E88-44FF-B1A5-C54FC7DD7B94}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9D3B833A-2730-470C-B690-F3390CECAE73}">
+          <x14:cfRule type="dataBar" id="{9FBA0817-4818-43DB-A4F7-A44D183BFBBE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E2BA61AA-F509-47FF-8049-50F6F1270697}">
+          <x14:cfRule type="dataBar" id="{62332EA6-77BC-4CC1-9059-50D62FA5BA22}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{15CE0C39-5E68-4A70-940F-4D0228B1A22E}">
+          <x14:cfRule type="dataBar" id="{25E0BDA6-B547-4D05-BAA7-E8FD7BFD49D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C42550FE-1452-4AF2-B32E-27CA74E055B8}</x14:id>
+          <x14:id>{6281458B-7A6F-4C6E-B442-7E77D6FC5E50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A8905CDF-3857-4C0A-8338-0BEC6E26480E}</x14:id>
+          <x14:id>{0510702D-EFA0-46B0-AFCD-C29424A57DC9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D153B539-E3C1-4F42-86E8-A23A1831068C}</x14:id>
+          <x14:id>{D5F59C7C-20D3-4E7A-845B-AA85E0C93BE7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1CE4F3B7-7E89-4321-BB43-4EC8A245B9B7}</x14:id>
+          <x14:id>{11A165F3-13A1-45E6-AA25-ED35FE8AE0F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C42550FE-1452-4AF2-B32E-27CA74E055B8}">
+          <x14:cfRule type="dataBar" id="{6281458B-7A6F-4C6E-B442-7E77D6FC5E50}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A8905CDF-3857-4C0A-8338-0BEC6E26480E}">
+          <x14:cfRule type="dataBar" id="{0510702D-EFA0-46B0-AFCD-C29424A57DC9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D153B539-E3C1-4F42-86E8-A23A1831068C}">
+          <x14:cfRule type="dataBar" id="{D5F59C7C-20D3-4E7A-845B-AA85E0C93BE7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1CE4F3B7-7E89-4321-BB43-4EC8A245B9B7}">
+          <x14:cfRule type="dataBar" id="{11A165F3-13A1-45E6-AA25-ED35FE8AE0F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3F99C9C5-7E88-44FF-B1A5-C54FC7DD7B94}</x14:id>
+          <x14:id>{DA781858-9E50-475E-83C4-38C5F351E8FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FBA0817-4818-43DB-A4F7-A44D183BFBBE}</x14:id>
+          <x14:id>{7B910B81-B1A9-4324-811B-B20E7CB7FA74}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62332EA6-77BC-4CC1-9059-50D62FA5BA22}</x14:id>
+          <x14:id>{382E16F0-77F4-4146-AD20-A48824B69FFF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25E0BDA6-B547-4D05-BAA7-E8FD7BFD49D5}</x14:id>
+          <x14:id>{462B0333-152E-40FE-AFAF-170BF1763467}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3F99C9C5-7E88-44FF-B1A5-C54FC7DD7B94}">
+          <x14:cfRule type="dataBar" id="{DA781858-9E50-475E-83C4-38C5F351E8FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FBA0817-4818-43DB-A4F7-A44D183BFBBE}">
+          <x14:cfRule type="dataBar" id="{7B910B81-B1A9-4324-811B-B20E7CB7FA74}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62332EA6-77BC-4CC1-9059-50D62FA5BA22}">
+          <x14:cfRule type="dataBar" id="{382E16F0-77F4-4146-AD20-A48824B69FFF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25E0BDA6-B547-4D05-BAA7-E8FD7BFD49D5}">
+          <x14:cfRule type="dataBar" id="{462B0333-152E-40FE-AFAF-170BF1763467}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6281458B-7A6F-4C6E-B442-7E77D6FC5E50}</x14:id>
+          <x14:id>{56C24E3C-30CE-4885-B6B8-7A8B4A951763}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0510702D-EFA0-46B0-AFCD-C29424A57DC9}</x14:id>
+          <x14:id>{0A59FBF7-5DB0-4CB4-9831-DB67D8385DB8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D5F59C7C-20D3-4E7A-845B-AA85E0C93BE7}</x14:id>
+          <x14:id>{71B754F0-0FF8-4C7D-B843-6293D91B53D3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11A165F3-13A1-45E6-AA25-ED35FE8AE0F5}</x14:id>
+          <x14:id>{BF882B0E-CF36-403E-9BBF-244B35987566}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6281458B-7A6F-4C6E-B442-7E77D6FC5E50}">
+          <x14:cfRule type="dataBar" id="{56C24E3C-30CE-4885-B6B8-7A8B4A951763}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0510702D-EFA0-46B0-AFCD-C29424A57DC9}">
+          <x14:cfRule type="dataBar" id="{0A59FBF7-5DB0-4CB4-9831-DB67D8385DB8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D5F59C7C-20D3-4E7A-845B-AA85E0C93BE7}">
+          <x14:cfRule type="dataBar" id="{71B754F0-0FF8-4C7D-B843-6293D91B53D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11A165F3-13A1-45E6-AA25-ED35FE8AE0F5}">
+          <x14:cfRule type="dataBar" id="{BF882B0E-CF36-403E-9BBF-244B35987566}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA781858-9E50-475E-83C4-38C5F351E8FD}</x14:id>
+          <x14:id>{6A300533-E378-40E6-BC70-12C05D8DFA4B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7B910B81-B1A9-4324-811B-B20E7CB7FA74}</x14:id>
+          <x14:id>{1EE5EC0B-89DF-4ED2-BA8E-00BEE2EA6F0A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{382E16F0-77F4-4146-AD20-A48824B69FFF}</x14:id>
+          <x14:id>{ABC69D64-DE44-4D30-A20A-583E35B868CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{462B0333-152E-40FE-AFAF-170BF1763467}</x14:id>
+          <x14:id>{40A9E58D-37DB-4B85-88FE-9AD98F47678E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA781858-9E50-475E-83C4-38C5F351E8FD}">
+          <x14:cfRule type="dataBar" id="{6A300533-E378-40E6-BC70-12C05D8DFA4B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7B910B81-B1A9-4324-811B-B20E7CB7FA74}">
+          <x14:cfRule type="dataBar" id="{1EE5EC0B-89DF-4ED2-BA8E-00BEE2EA6F0A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{382E16F0-77F4-4146-AD20-A48824B69FFF}">
+          <x14:cfRule type="dataBar" id="{ABC69D64-DE44-4D30-A20A-583E35B868CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{462B0333-152E-40FE-AFAF-170BF1763467}">
+          <x14:cfRule type="dataBar" id="{40A9E58D-37DB-4B85-88FE-9AD98F47678E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{56C24E3C-30CE-4885-B6B8-7A8B4A951763}</x14:id>
+          <x14:id>{19C6879F-9C92-4D38-B593-5B579B84649D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0A59FBF7-5DB0-4CB4-9831-DB67D8385DB8}</x14:id>
+          <x14:id>{04F0ABEC-F65C-46F8-B099-ED17022461D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{71B754F0-0FF8-4C7D-B843-6293D91B53D3}</x14:id>
+          <x14:id>{C7BAEB43-8C6F-4399-8B00-4FE1542CBF6B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BF882B0E-CF36-403E-9BBF-244B35987566}</x14:id>
+          <x14:id>{ECA97B32-0067-44EE-B17E-B4620CEC5A68}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{56C24E3C-30CE-4885-B6B8-7A8B4A951763}">
+          <x14:cfRule type="dataBar" id="{19C6879F-9C92-4D38-B593-5B579B84649D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0A59FBF7-5DB0-4CB4-9831-DB67D8385DB8}">
+          <x14:cfRule type="dataBar" id="{04F0ABEC-F65C-46F8-B099-ED17022461D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{71B754F0-0FF8-4C7D-B843-6293D91B53D3}">
+          <x14:cfRule type="dataBar" id="{C7BAEB43-8C6F-4399-8B00-4FE1542CBF6B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BF882B0E-CF36-403E-9BBF-244B35987566}">
+          <x14:cfRule type="dataBar" id="{ECA97B32-0067-44EE-B17E-B4620CEC5A68}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6A300533-E378-40E6-BC70-12C05D8DFA4B}</x14:id>
+          <x14:id>{28E57BCD-567B-46F3-9235-012F7F5328A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1EE5EC0B-89DF-4ED2-BA8E-00BEE2EA6F0A}</x14:id>
+          <x14:id>{63CFED25-4369-4720-B757-DC878AE01BBE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ABC69D64-DE44-4D30-A20A-583E35B868CF}</x14:id>
+          <x14:id>{37C728DB-6853-4716-9B8F-BD1BBCA806FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{40A9E58D-37DB-4B85-88FE-9AD98F47678E}</x14:id>
+          <x14:id>{1567011C-4786-4A94-9ABA-67E791FF4C29}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6A300533-E378-40E6-BC70-12C05D8DFA4B}">
+          <x14:cfRule type="dataBar" id="{28E57BCD-567B-46F3-9235-012F7F5328A7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1EE5EC0B-89DF-4ED2-BA8E-00BEE2EA6F0A}">
+          <x14:cfRule type="dataBar" id="{63CFED25-4369-4720-B757-DC878AE01BBE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ABC69D64-DE44-4D30-A20A-583E35B868CF}">
+          <x14:cfRule type="dataBar" id="{37C728DB-6853-4716-9B8F-BD1BBCA806FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{40A9E58D-37DB-4B85-88FE-9AD98F47678E}">
+          <x14:cfRule type="dataBar" id="{1567011C-4786-4A94-9ABA-67E791FF4C29}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19C6879F-9C92-4D38-B593-5B579B84649D}</x14:id>
+          <x14:id>{F3C9C23B-0269-4536-A04E-E2473EA43170}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{04F0ABEC-F65C-46F8-B099-ED17022461D2}</x14:id>
+          <x14:id>{6D5ABFDB-0D20-4EC2-82BE-FF6B3CC22A72}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C7BAEB43-8C6F-4399-8B00-4FE1542CBF6B}</x14:id>
+          <x14:id>{44999278-2B40-4E33-8D64-9F4915FD7631}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ECA97B32-0067-44EE-B17E-B4620CEC5A68}</x14:id>
+          <x14:id>{38DC7E1B-1B64-419D-8279-9182DBD96ABF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19C6879F-9C92-4D38-B593-5B579B84649D}">
+          <x14:cfRule type="dataBar" id="{F3C9C23B-0269-4536-A04E-E2473EA43170}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{04F0ABEC-F65C-46F8-B099-ED17022461D2}">
+          <x14:cfRule type="dataBar" id="{6D5ABFDB-0D20-4EC2-82BE-FF6B3CC22A72}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C7BAEB43-8C6F-4399-8B00-4FE1542CBF6B}">
+          <x14:cfRule type="dataBar" id="{44999278-2B40-4E33-8D64-9F4915FD7631}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ECA97B32-0067-44EE-B17E-B4620CEC5A68}">
+          <x14:cfRule type="dataBar" id="{38DC7E1B-1B64-419D-8279-9182DBD96ABF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28E57BCD-567B-46F3-9235-012F7F5328A7}</x14:id>
+          <x14:id>{14189360-3901-4B47-A444-4736B67E9F4A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{63CFED25-4369-4720-B757-DC878AE01BBE}</x14:id>
+          <x14:id>{6331AFE6-10A1-4BBF-B857-030FD88FE108}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37C728DB-6853-4716-9B8F-BD1BBCA806FD}</x14:id>
+          <x14:id>{F91F5773-5399-4FC2-8285-21821CF644B1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1567011C-4786-4A94-9ABA-67E791FF4C29}</x14:id>
+          <x14:id>{96306A1E-0AFA-4BC4-8771-D4200790D410}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28E57BCD-567B-46F3-9235-012F7F5328A7}">
+          <x14:cfRule type="dataBar" id="{14189360-3901-4B47-A444-4736B67E9F4A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{63CFED25-4369-4720-B757-DC878AE01BBE}">
+          <x14:cfRule type="dataBar" id="{6331AFE6-10A1-4BBF-B857-030FD88FE108}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37C728DB-6853-4716-9B8F-BD1BBCA806FD}">
+          <x14:cfRule type="dataBar" id="{F91F5773-5399-4FC2-8285-21821CF644B1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1567011C-4786-4A94-9ABA-67E791FF4C29}">
+          <x14:cfRule type="dataBar" id="{96306A1E-0AFA-4BC4-8771-D4200790D410}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F3C9C23B-0269-4536-A04E-E2473EA43170}</x14:id>
+          <x14:id>{5A164E3A-C0A6-4CCB-8BD2-E2D561A62005}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D5ABFDB-0D20-4EC2-82BE-FF6B3CC22A72}</x14:id>
+          <x14:id>{B6CCB658-63D8-473D-8FCA-254DB4167779}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{44999278-2B40-4E33-8D64-9F4915FD7631}</x14:id>
+          <x14:id>{63E96497-C348-4A5B-A774-5033F4A0613F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38DC7E1B-1B64-419D-8279-9182DBD96ABF}</x14:id>
+          <x14:id>{7578C282-4EF6-4216-BD3E-808EDC81B6B8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F3C9C23B-0269-4536-A04E-E2473EA43170}">
+          <x14:cfRule type="dataBar" id="{5A164E3A-C0A6-4CCB-8BD2-E2D561A62005}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D5ABFDB-0D20-4EC2-82BE-FF6B3CC22A72}">
+          <x14:cfRule type="dataBar" id="{B6CCB658-63D8-473D-8FCA-254DB4167779}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{44999278-2B40-4E33-8D64-9F4915FD7631}">
+          <x14:cfRule type="dataBar" id="{63E96497-C348-4A5B-A774-5033F4A0613F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38DC7E1B-1B64-419D-8279-9182DBD96ABF}">
+          <x14:cfRule type="dataBar" id="{7578C282-4EF6-4216-BD3E-808EDC81B6B8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{14189360-3901-4B47-A444-4736B67E9F4A}</x14:id>
+          <x14:id>{90DC0FDC-B49A-42FF-B41E-D14ED6C56D13}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6331AFE6-10A1-4BBF-B857-030FD88FE108}</x14:id>
+          <x14:id>{0D72B1DA-5B32-4AE6-B27F-A4D5F4165701}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F91F5773-5399-4FC2-8285-21821CF644B1}</x14:id>
+          <x14:id>{F749179F-3D70-4ACF-876D-F047D8FE77AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{96306A1E-0AFA-4BC4-8771-D4200790D410}</x14:id>
+          <x14:id>{1CCA8AEE-245A-42F3-A809-B7108EE5EA27}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{14189360-3901-4B47-A444-4736B67E9F4A}">
+          <x14:cfRule type="dataBar" id="{90DC0FDC-B49A-42FF-B41E-D14ED6C56D13}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6331AFE6-10A1-4BBF-B857-030FD88FE108}">
+          <x14:cfRule type="dataBar" id="{0D72B1DA-5B32-4AE6-B27F-A4D5F4165701}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F91F5773-5399-4FC2-8285-21821CF644B1}">
+          <x14:cfRule type="dataBar" id="{F749179F-3D70-4ACF-876D-F047D8FE77AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{96306A1E-0AFA-4BC4-8771-D4200790D410}">
+          <x14:cfRule type="dataBar" id="{1CCA8AEE-245A-42F3-A809-B7108EE5EA27}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A164E3A-C0A6-4CCB-8BD2-E2D561A62005}</x14:id>
+          <x14:id>{87DDAAFA-6030-4378-856A-16C0619BB379}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B6CCB658-63D8-473D-8FCA-254DB4167779}</x14:id>
+          <x14:id>{BD18E125-9EE1-45E1-8BBC-7078EA9B07DE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{63E96497-C348-4A5B-A774-5033F4A0613F}</x14:id>
+          <x14:id>{26523BEB-F1D9-4975-9D77-8F0D0D59EFAA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7578C282-4EF6-4216-BD3E-808EDC81B6B8}</x14:id>
+          <x14:id>{6917975B-EC26-435A-91FA-AF1E974D3A6C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A164E3A-C0A6-4CCB-8BD2-E2D561A62005}">
+          <x14:cfRule type="dataBar" id="{87DDAAFA-6030-4378-856A-16C0619BB379}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B6CCB658-63D8-473D-8FCA-254DB4167779}">
+          <x14:cfRule type="dataBar" id="{BD18E125-9EE1-45E1-8BBC-7078EA9B07DE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{63E96497-C348-4A5B-A774-5033F4A0613F}">
+          <x14:cfRule type="dataBar" id="{26523BEB-F1D9-4975-9D77-8F0D0D59EFAA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7578C282-4EF6-4216-BD3E-808EDC81B6B8}">
+          <x14:cfRule type="dataBar" id="{6917975B-EC26-435A-91FA-AF1E974D3A6C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90DC0FDC-B49A-42FF-B41E-D14ED6C56D13}</x14:id>
+          <x14:id>{EBF454DE-9C1D-4CCF-89C9-21D78AAF83E5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D72B1DA-5B32-4AE6-B27F-A4D5F4165701}</x14:id>
+          <x14:id>{B52670D2-5BD4-4267-8937-02057E4CD34F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F749179F-3D70-4ACF-876D-F047D8FE77AF}</x14:id>
+          <x14:id>{DBE6E430-6770-4271-9823-AD3E51D75C97}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1CCA8AEE-245A-42F3-A809-B7108EE5EA27}</x14:id>
+          <x14:id>{BBE0FAB4-E48B-4081-939B-C6AA09A1AC83}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90DC0FDC-B49A-42FF-B41E-D14ED6C56D13}">
+          <x14:cfRule type="dataBar" id="{EBF454DE-9C1D-4CCF-89C9-21D78AAF83E5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D72B1DA-5B32-4AE6-B27F-A4D5F4165701}">
+          <x14:cfRule type="dataBar" id="{B52670D2-5BD4-4267-8937-02057E4CD34F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F749179F-3D70-4ACF-876D-F047D8FE77AF}">
+          <x14:cfRule type="dataBar" id="{DBE6E430-6770-4271-9823-AD3E51D75C97}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1CCA8AEE-245A-42F3-A809-B7108EE5EA27}">
+          <x14:cfRule type="dataBar" id="{BBE0FAB4-E48B-4081-939B-C6AA09A1AC83}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87DDAAFA-6030-4378-856A-16C0619BB379}</x14:id>
+          <x14:id>{658258C5-E4E5-4D76-80B4-22881D409F80}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BD18E125-9EE1-45E1-8BBC-7078EA9B07DE}</x14:id>
+          <x14:id>{F319EF93-F61D-4C0D-9229-E2DB2DAF19F3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26523BEB-F1D9-4975-9D77-8F0D0D59EFAA}</x14:id>
+          <x14:id>{48DB0EF4-9527-491C-85C2-CABDEB29FA43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6917975B-EC26-435A-91FA-AF1E974D3A6C}</x14:id>
+          <x14:id>{0B38E494-DFF6-490A-84AF-AF19F2777630}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87DDAAFA-6030-4378-856A-16C0619BB379}">
+          <x14:cfRule type="dataBar" id="{658258C5-E4E5-4D76-80B4-22881D409F80}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BD18E125-9EE1-45E1-8BBC-7078EA9B07DE}">
+          <x14:cfRule type="dataBar" id="{F319EF93-F61D-4C0D-9229-E2DB2DAF19F3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26523BEB-F1D9-4975-9D77-8F0D0D59EFAA}">
+          <x14:cfRule type="dataBar" id="{48DB0EF4-9527-491C-85C2-CABDEB29FA43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6917975B-EC26-435A-91FA-AF1E974D3A6C}">
+          <x14:cfRule type="dataBar" id="{0B38E494-DFF6-490A-84AF-AF19F2777630}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EBF454DE-9C1D-4CCF-89C9-21D78AAF83E5}</x14:id>
+          <x14:id>{ED1EB5D2-2CC6-479A-9E92-4A5B174124F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B52670D2-5BD4-4267-8937-02057E4CD34F}</x14:id>
+          <x14:id>{6B044868-E1C5-47F9-8671-3CFD495C6C18}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DBE6E430-6770-4271-9823-AD3E51D75C97}</x14:id>
+          <x14:id>{A80EA6FC-12E8-49F3-94E2-6A2757C9A7DC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BBE0FAB4-E48B-4081-939B-C6AA09A1AC83}</x14:id>
+          <x14:id>{FE4AFF5B-EEA7-497F-9A0B-0287F31EE59D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EBF454DE-9C1D-4CCF-89C9-21D78AAF83E5}">
+          <x14:cfRule type="dataBar" id="{ED1EB5D2-2CC6-479A-9E92-4A5B174124F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B52670D2-5BD4-4267-8937-02057E4CD34F}">
+          <x14:cfRule type="dataBar" id="{6B044868-E1C5-47F9-8671-3CFD495C6C18}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DBE6E430-6770-4271-9823-AD3E51D75C97}">
+          <x14:cfRule type="dataBar" id="{A80EA6FC-12E8-49F3-94E2-6A2757C9A7DC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BBE0FAB4-E48B-4081-939B-C6AA09A1AC83}">
+          <x14:cfRule type="dataBar" id="{FE4AFF5B-EEA7-497F-9A0B-0287F31EE59D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{658258C5-E4E5-4D76-80B4-22881D409F80}</x14:id>
+          <x14:id>{CEAA9E50-1C0D-4139-9BE9-C1A9EF585806}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F319EF93-F61D-4C0D-9229-E2DB2DAF19F3}</x14:id>
+          <x14:id>{2BB8030E-DD22-4681-981D-B9A08F890BC7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{48DB0EF4-9527-491C-85C2-CABDEB29FA43}</x14:id>
+          <x14:id>{BD41133E-FAF3-4DF1-919A-B1E0B4080B53}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B38E494-DFF6-490A-84AF-AF19F2777630}</x14:id>
+          <x14:id>{FD45B2C2-2224-4639-A7B2-7214FCE90CFC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{658258C5-E4E5-4D76-80B4-22881D409F80}">
+          <x14:cfRule type="dataBar" id="{CEAA9E50-1C0D-4139-9BE9-C1A9EF585806}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F319EF93-F61D-4C0D-9229-E2DB2DAF19F3}">
+          <x14:cfRule type="dataBar" id="{2BB8030E-DD22-4681-981D-B9A08F890BC7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{48DB0EF4-9527-491C-85C2-CABDEB29FA43}">
+          <x14:cfRule type="dataBar" id="{BD41133E-FAF3-4DF1-919A-B1E0B4080B53}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B38E494-DFF6-490A-84AF-AF19F2777630}">
+          <x14:cfRule type="dataBar" id="{FD45B2C2-2224-4639-A7B2-7214FCE90CFC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ED1EB5D2-2CC6-479A-9E92-4A5B174124F1}</x14:id>
+          <x14:id>{5A530807-9865-4422-9000-38D14E725BC2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B044868-E1C5-47F9-8671-3CFD495C6C18}</x14:id>
+          <x14:id>{880A927B-5828-4B3E-B37F-394EF02F3FF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A80EA6FC-12E8-49F3-94E2-6A2757C9A7DC}</x14:id>
+          <x14:id>{7E6385AE-B54D-4FAA-9F22-549019B388C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE4AFF5B-EEA7-497F-9A0B-0287F31EE59D}</x14:id>
+          <x14:id>{9D6CE0F4-A2AC-44DB-8811-1C56E46B1EDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ED1EB5D2-2CC6-479A-9E92-4A5B174124F1}">
+          <x14:cfRule type="dataBar" id="{5A530807-9865-4422-9000-38D14E725BC2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B044868-E1C5-47F9-8671-3CFD495C6C18}">
+          <x14:cfRule type="dataBar" id="{880A927B-5828-4B3E-B37F-394EF02F3FF6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A80EA6FC-12E8-49F3-94E2-6A2757C9A7DC}">
+          <x14:cfRule type="dataBar" id="{7E6385AE-B54D-4FAA-9F22-549019B388C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE4AFF5B-EEA7-497F-9A0B-0287F31EE59D}">
+          <x14:cfRule type="dataBar" id="{9D6CE0F4-A2AC-44DB-8811-1C56E46B1EDE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CEAA9E50-1C0D-4139-9BE9-C1A9EF585806}</x14:id>
+          <x14:id>{0D5D11D8-B192-4FAE-B881-D0D486C1A224}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2BB8030E-DD22-4681-981D-B9A08F890BC7}</x14:id>
+          <x14:id>{335731BE-9FD3-4681-89AD-F41A90CEF8CE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BD41133E-FAF3-4DF1-919A-B1E0B4080B53}</x14:id>
+          <x14:id>{F9505426-64E6-44DE-9B8D-2D723D5AA4CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD45B2C2-2224-4639-A7B2-7214FCE90CFC}</x14:id>
+          <x14:id>{07717B63-34C0-4346-8AC0-69F678EAB30B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CEAA9E50-1C0D-4139-9BE9-C1A9EF585806}">
+          <x14:cfRule type="dataBar" id="{0D5D11D8-B192-4FAE-B881-D0D486C1A224}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2BB8030E-DD22-4681-981D-B9A08F890BC7}">
+          <x14:cfRule type="dataBar" id="{335731BE-9FD3-4681-89AD-F41A90CEF8CE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BD41133E-FAF3-4DF1-919A-B1E0B4080B53}">
+          <x14:cfRule type="dataBar" id="{F9505426-64E6-44DE-9B8D-2D723D5AA4CA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD45B2C2-2224-4639-A7B2-7214FCE90CFC}">
+          <x14:cfRule type="dataBar" id="{07717B63-34C0-4346-8AC0-69F678EAB30B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-26 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -9342,7 +9342,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A530807-9865-4422-9000-38D14E725BC2}</x14:id>
+          <x14:id>{F6F02384-94B2-4E61-9007-5B409B486B43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9356,7 +9356,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{880A927B-5828-4B3E-B37F-394EF02F3FF6}</x14:id>
+          <x14:id>{BB741000-45CC-4F5C-A4C4-011892AA907F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9370,7 +9370,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E6385AE-B54D-4FAA-9F22-549019B388C0}</x14:id>
+          <x14:id>{97DE45FD-98A0-4578-A900-C33170039368}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9384,7 +9384,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9D6CE0F4-A2AC-44DB-8811-1C56E46B1EDE}</x14:id>
+          <x14:id>{E05346F7-7C39-4A39-8F96-223E4869CBAE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -9394,7 +9394,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A530807-9865-4422-9000-38D14E725BC2}">
+          <x14:cfRule type="dataBar" id="{F6F02384-94B2-4E61-9007-5B409B486B43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9407,7 +9407,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{880A927B-5828-4B3E-B37F-394EF02F3FF6}">
+          <x14:cfRule type="dataBar" id="{BB741000-45CC-4F5C-A4C4-011892AA907F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9420,7 +9420,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E6385AE-B54D-4FAA-9F22-549019B388C0}">
+          <x14:cfRule type="dataBar" id="{97DE45FD-98A0-4578-A900-C33170039368}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -9433,7 +9433,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9D6CE0F4-A2AC-44DB-8811-1C56E46B1EDE}">
+          <x14:cfRule type="dataBar" id="{E05346F7-7C39-4A39-8F96-223E4869CBAE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24733,7 +24733,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D5D11D8-B192-4FAE-B881-D0D486C1A224}</x14:id>
+          <x14:id>{1C41934E-C719-4D95-9C6E-099D69842FA4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24747,7 +24747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{335731BE-9FD3-4681-89AD-F41A90CEF8CE}</x14:id>
+          <x14:id>{A8E4B3E7-C1B2-4AAC-865A-A625EA665821}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24761,7 +24761,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F9505426-64E6-44DE-9B8D-2D723D5AA4CA}</x14:id>
+          <x14:id>{C5C97920-1FAC-446F-8C0F-08B4C6E95DE4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24775,7 +24775,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07717B63-34C0-4346-8AC0-69F678EAB30B}</x14:id>
+          <x14:id>{75882BBC-1EFF-434A-A6CB-2DD36101E466}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24785,7 +24785,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D5D11D8-B192-4FAE-B881-D0D486C1A224}">
+          <x14:cfRule type="dataBar" id="{1C41934E-C719-4D95-9C6E-099D69842FA4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24798,7 +24798,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{335731BE-9FD3-4681-89AD-F41A90CEF8CE}">
+          <x14:cfRule type="dataBar" id="{A8E4B3E7-C1B2-4AAC-865A-A625EA665821}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24811,7 +24811,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F9505426-64E6-44DE-9B8D-2D723D5AA4CA}">
+          <x14:cfRule type="dataBar" id="{C5C97920-1FAC-446F-8C0F-08B4C6E95DE4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -24824,7 +24824,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07717B63-34C0-4346-8AC0-69F678EAB30B}">
+          <x14:cfRule type="dataBar" id="{75882BBC-1EFF-434A-A6CB-2DD36101E466}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC93E8DF-E694-4916-B1E3-03FA3B24B409}</x14:id>
+          <x14:id>{2E46669A-62DC-4700-8137-858102B0F3D4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE95CCE7-0ECA-4478-81B7-0CA89248268E}</x14:id>
+          <x14:id>{E4F55C7F-EE76-46E0-AA50-F06D3B661BDA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D1D6EE73-816F-4F8E-B623-C8353595B7C6}</x14:id>
+          <x14:id>{553D7079-DD29-47D9-A54C-EBFE50E92B16}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5805542F-5621-4382-B46D-EF6ED7630116}</x14:id>
+          <x14:id>{0AC227CF-A5AB-42A9-A917-766D4B5B88DF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC93E8DF-E694-4916-B1E3-03FA3B24B409}">
+          <x14:cfRule type="dataBar" id="{2E46669A-62DC-4700-8137-858102B0F3D4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE95CCE7-0ECA-4478-81B7-0CA89248268E}">
+          <x14:cfRule type="dataBar" id="{E4F55C7F-EE76-46E0-AA50-F06D3B661BDA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D1D6EE73-816F-4F8E-B623-C8353595B7C6}">
+          <x14:cfRule type="dataBar" id="{553D7079-DD29-47D9-A54C-EBFE50E92B16}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5805542F-5621-4382-B46D-EF6ED7630116}">
+          <x14:cfRule type="dataBar" id="{0AC227CF-A5AB-42A9-A917-766D4B5B88DF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5CF11F49-A1FE-4FBC-89AE-661EBB9FEAD4}</x14:id>
+          <x14:id>{118D8608-4C36-4573-BCD2-1E0F3A3ABBC9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF6BF09D-B5DD-4F0F-9D71-71DF32BB9019}</x14:id>
+          <x14:id>{2F1B5E40-0DDC-4A2C-87F1-625D8B983138}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CA442B00-9330-4E45-9E93-178708996B5D}</x14:id>
+          <x14:id>{DFD0836E-8B7E-42E0-90A0-710C0928C742}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A510F62D-13A0-4B21-9EB9-28CB87DF7BB7}</x14:id>
+          <x14:id>{240C8D9B-E635-4462-8310-853838D8B9A4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5CF11F49-A1FE-4FBC-89AE-661EBB9FEAD4}">
+          <x14:cfRule type="dataBar" id="{118D8608-4C36-4573-BCD2-1E0F3A3ABBC9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF6BF09D-B5DD-4F0F-9D71-71DF32BB9019}">
+          <x14:cfRule type="dataBar" id="{2F1B5E40-0DDC-4A2C-87F1-625D8B983138}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CA442B00-9330-4E45-9E93-178708996B5D}">
+          <x14:cfRule type="dataBar" id="{DFD0836E-8B7E-42E0-90A0-710C0928C742}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A510F62D-13A0-4B21-9EB9-28CB87DF7BB7}">
+          <x14:cfRule type="dataBar" id="{240C8D9B-E635-4462-8310-853838D8B9A4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E46669A-62DC-4700-8137-858102B0F3D4}</x14:id>
+          <x14:id>{E02B30A7-8763-42D4-B9ED-DCDF5BDA9822}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4F55C7F-EE76-46E0-AA50-F06D3B661BDA}</x14:id>
+          <x14:id>{D573E603-B92C-4455-AC85-55A28CB76195}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{553D7079-DD29-47D9-A54C-EBFE50E92B16}</x14:id>
+          <x14:id>{026291C6-43CA-43EA-BE1D-35919E424E24}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0AC227CF-A5AB-42A9-A917-766D4B5B88DF}</x14:id>
+          <x14:id>{BECBA617-AE80-4E4B-B6CE-A45E9306F2B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E46669A-62DC-4700-8137-858102B0F3D4}">
+          <x14:cfRule type="dataBar" id="{E02B30A7-8763-42D4-B9ED-DCDF5BDA9822}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4F55C7F-EE76-46E0-AA50-F06D3B661BDA}">
+          <x14:cfRule type="dataBar" id="{D573E603-B92C-4455-AC85-55A28CB76195}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{553D7079-DD29-47D9-A54C-EBFE50E92B16}">
+          <x14:cfRule type="dataBar" id="{026291C6-43CA-43EA-BE1D-35919E424E24}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0AC227CF-A5AB-42A9-A917-766D4B5B88DF}">
+          <x14:cfRule type="dataBar" id="{BECBA617-AE80-4E4B-B6CE-A45E9306F2B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{118D8608-4C36-4573-BCD2-1E0F3A3ABBC9}</x14:id>
+          <x14:id>{AA911ABD-3D92-4FDD-87CB-E83B4558CAC5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2F1B5E40-0DDC-4A2C-87F1-625D8B983138}</x14:id>
+          <x14:id>{8D21B86C-DBF7-4EDF-B50A-D8A8E975708E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DFD0836E-8B7E-42E0-90A0-710C0928C742}</x14:id>
+          <x14:id>{0891BBEC-1883-492A-BB3F-104E4634B2DD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{240C8D9B-E635-4462-8310-853838D8B9A4}</x14:id>
+          <x14:id>{80FA0F6B-18E9-4C44-9565-7AF7F8D623BE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{118D8608-4C36-4573-BCD2-1E0F3A3ABBC9}">
+          <x14:cfRule type="dataBar" id="{AA911ABD-3D92-4FDD-87CB-E83B4558CAC5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2F1B5E40-0DDC-4A2C-87F1-625D8B983138}">
+          <x14:cfRule type="dataBar" id="{8D21B86C-DBF7-4EDF-B50A-D8A8E975708E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DFD0836E-8B7E-42E0-90A0-710C0928C742}">
+          <x14:cfRule type="dataBar" id="{0891BBEC-1883-492A-BB3F-104E4634B2DD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{240C8D9B-E635-4462-8310-853838D8B9A4}">
+          <x14:cfRule type="dataBar" id="{80FA0F6B-18E9-4C44-9565-7AF7F8D623BE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E02B30A7-8763-42D4-B9ED-DCDF5BDA9822}</x14:id>
+          <x14:id>{3D43DFD7-E7F9-4745-8CD4-D28A3DAD8EC3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D573E603-B92C-4455-AC85-55A28CB76195}</x14:id>
+          <x14:id>{6516F728-9C93-4209-A669-57F481A7FE93}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{026291C6-43CA-43EA-BE1D-35919E424E24}</x14:id>
+          <x14:id>{3962020B-484D-4EEB-B134-1D00716BFE97}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BECBA617-AE80-4E4B-B6CE-A45E9306F2B4}</x14:id>
+          <x14:id>{2CA982BA-7AED-43A3-9F00-258EFE611C57}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E02B30A7-8763-42D4-B9ED-DCDF5BDA9822}">
+          <x14:cfRule type="dataBar" id="{3D43DFD7-E7F9-4745-8CD4-D28A3DAD8EC3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D573E603-B92C-4455-AC85-55A28CB76195}">
+          <x14:cfRule type="dataBar" id="{6516F728-9C93-4209-A669-57F481A7FE93}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{026291C6-43CA-43EA-BE1D-35919E424E24}">
+          <x14:cfRule type="dataBar" id="{3962020B-484D-4EEB-B134-1D00716BFE97}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BECBA617-AE80-4E4B-B6CE-A45E9306F2B4}">
+          <x14:cfRule type="dataBar" id="{2CA982BA-7AED-43A3-9F00-258EFE611C57}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA911ABD-3D92-4FDD-87CB-E83B4558CAC5}</x14:id>
+          <x14:id>{CB3328FB-1D00-4845-AB6C-14624B5D3794}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8D21B86C-DBF7-4EDF-B50A-D8A8E975708E}</x14:id>
+          <x14:id>{C3F679B9-0FA2-499B-85FF-771A42D4B3A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0891BBEC-1883-492A-BB3F-104E4634B2DD}</x14:id>
+          <x14:id>{0891EA0B-9B06-4DF9-A7E9-B5368D4DE93E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{80FA0F6B-18E9-4C44-9565-7AF7F8D623BE}</x14:id>
+          <x14:id>{137D0D41-E464-4BF0-B221-A768FBE01E69}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA911ABD-3D92-4FDD-87CB-E83B4558CAC5}">
+          <x14:cfRule type="dataBar" id="{CB3328FB-1D00-4845-AB6C-14624B5D3794}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8D21B86C-DBF7-4EDF-B50A-D8A8E975708E}">
+          <x14:cfRule type="dataBar" id="{C3F679B9-0FA2-499B-85FF-771A42D4B3A7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0891BBEC-1883-492A-BB3F-104E4634B2DD}">
+          <x14:cfRule type="dataBar" id="{0891EA0B-9B06-4DF9-A7E9-B5368D4DE93E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{80FA0F6B-18E9-4C44-9565-7AF7F8D623BE}">
+          <x14:cfRule type="dataBar" id="{137D0D41-E464-4BF0-B221-A768FBE01E69}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D43DFD7-E7F9-4745-8CD4-D28A3DAD8EC3}</x14:id>
+          <x14:id>{EAA29757-39EE-496C-8D0C-E87406DB1EE9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6516F728-9C93-4209-A669-57F481A7FE93}</x14:id>
+          <x14:id>{DAD3E7EA-81E6-4683-A7AB-B70D145C8EA6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3962020B-484D-4EEB-B134-1D00716BFE97}</x14:id>
+          <x14:id>{7366D342-EFEF-486D-ABC7-50A1223103AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2CA982BA-7AED-43A3-9F00-258EFE611C57}</x14:id>
+          <x14:id>{9CD552B5-0191-49D0-8EFA-E1A0A4158C90}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D43DFD7-E7F9-4745-8CD4-D28A3DAD8EC3}">
+          <x14:cfRule type="dataBar" id="{EAA29757-39EE-496C-8D0C-E87406DB1EE9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6516F728-9C93-4209-A669-57F481A7FE93}">
+          <x14:cfRule type="dataBar" id="{DAD3E7EA-81E6-4683-A7AB-B70D145C8EA6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3962020B-484D-4EEB-B134-1D00716BFE97}">
+          <x14:cfRule type="dataBar" id="{7366D342-EFEF-486D-ABC7-50A1223103AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2CA982BA-7AED-43A3-9F00-258EFE611C57}">
+          <x14:cfRule type="dataBar" id="{9CD552B5-0191-49D0-8EFA-E1A0A4158C90}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CB3328FB-1D00-4845-AB6C-14624B5D3794}</x14:id>
+          <x14:id>{DF7A73A4-3A15-4D01-B326-4C5EE753E14B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C3F679B9-0FA2-499B-85FF-771A42D4B3A7}</x14:id>
+          <x14:id>{59C8A5EE-7F41-45DA-89A5-1609C9F9F083}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0891EA0B-9B06-4DF9-A7E9-B5368D4DE93E}</x14:id>
+          <x14:id>{D550E517-C0C8-4409-B10A-FAD7297C941A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{137D0D41-E464-4BF0-B221-A768FBE01E69}</x14:id>
+          <x14:id>{FFDD4F55-B7DA-4479-82D6-CC965E4E81F6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CB3328FB-1D00-4845-AB6C-14624B5D3794}">
+          <x14:cfRule type="dataBar" id="{DF7A73A4-3A15-4D01-B326-4C5EE753E14B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C3F679B9-0FA2-499B-85FF-771A42D4B3A7}">
+          <x14:cfRule type="dataBar" id="{59C8A5EE-7F41-45DA-89A5-1609C9F9F083}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0891EA0B-9B06-4DF9-A7E9-B5368D4DE93E}">
+          <x14:cfRule type="dataBar" id="{D550E517-C0C8-4409-B10A-FAD7297C941A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{137D0D41-E464-4BF0-B221-A768FBE01E69}">
+          <x14:cfRule type="dataBar" id="{FFDD4F55-B7DA-4479-82D6-CC965E4E81F6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EAA29757-39EE-496C-8D0C-E87406DB1EE9}</x14:id>
+          <x14:id>{2FD2A86E-541F-4444-BFE7-8B70D790A215}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DAD3E7EA-81E6-4683-A7AB-B70D145C8EA6}</x14:id>
+          <x14:id>{526E34E8-82D7-4862-98FF-417495D1EC01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7366D342-EFEF-486D-ABC7-50A1223103AB}</x14:id>
+          <x14:id>{1D938954-A429-4262-B9BF-E0CC33E3FD97}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9CD552B5-0191-49D0-8EFA-E1A0A4158C90}</x14:id>
+          <x14:id>{934CD0BF-67ED-4044-9417-63BBA08616D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EAA29757-39EE-496C-8D0C-E87406DB1EE9}">
+          <x14:cfRule type="dataBar" id="{2FD2A86E-541F-4444-BFE7-8B70D790A215}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DAD3E7EA-81E6-4683-A7AB-B70D145C8EA6}">
+          <x14:cfRule type="dataBar" id="{526E34E8-82D7-4862-98FF-417495D1EC01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7366D342-EFEF-486D-ABC7-50A1223103AB}">
+          <x14:cfRule type="dataBar" id="{1D938954-A429-4262-B9BF-E0CC33E3FD97}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9CD552B5-0191-49D0-8EFA-E1A0A4158C90}">
+          <x14:cfRule type="dataBar" id="{934CD0BF-67ED-4044-9417-63BBA08616D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DF7A73A4-3A15-4D01-B326-4C5EE753E14B}</x14:id>
+          <x14:id>{189FE16B-3C45-4ED1-AB74-1743FBFD26CD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{59C8A5EE-7F41-45DA-89A5-1609C9F9F083}</x14:id>
+          <x14:id>{C0303A87-0D95-46B3-B072-5255187D7CD8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D550E517-C0C8-4409-B10A-FAD7297C941A}</x14:id>
+          <x14:id>{D6FB19C9-FA9B-42C8-A690-0EF33CBBB311}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FFDD4F55-B7DA-4479-82D6-CC965E4E81F6}</x14:id>
+          <x14:id>{C54E5308-87FF-4C8B-AF5D-05F6CC3FC8F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DF7A73A4-3A15-4D01-B326-4C5EE753E14B}">
+          <x14:cfRule type="dataBar" id="{189FE16B-3C45-4ED1-AB74-1743FBFD26CD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{59C8A5EE-7F41-45DA-89A5-1609C9F9F083}">
+          <x14:cfRule type="dataBar" id="{C0303A87-0D95-46B3-B072-5255187D7CD8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D550E517-C0C8-4409-B10A-FAD7297C941A}">
+          <x14:cfRule type="dataBar" id="{D6FB19C9-FA9B-42C8-A690-0EF33CBBB311}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FFDD4F55-B7DA-4479-82D6-CC965E4E81F6}">
+          <x14:cfRule type="dataBar" id="{C54E5308-87FF-4C8B-AF5D-05F6CC3FC8F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2FD2A86E-541F-4444-BFE7-8B70D790A215}</x14:id>
+          <x14:id>{BDBEAD58-0142-4286-AE1A-9CF534495B01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{526E34E8-82D7-4862-98FF-417495D1EC01}</x14:id>
+          <x14:id>{D09AC923-DEC1-494F-A3CC-ABE181B01602}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1D938954-A429-4262-B9BF-E0CC33E3FD97}</x14:id>
+          <x14:id>{58C0BD30-2288-4427-8643-F3A161E068CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{934CD0BF-67ED-4044-9417-63BBA08616D0}</x14:id>
+          <x14:id>{049F3817-33DC-4DD2-B793-26272D793A56}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2FD2A86E-541F-4444-BFE7-8B70D790A215}">
+          <x14:cfRule type="dataBar" id="{BDBEAD58-0142-4286-AE1A-9CF534495B01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{526E34E8-82D7-4862-98FF-417495D1EC01}">
+          <x14:cfRule type="dataBar" id="{D09AC923-DEC1-494F-A3CC-ABE181B01602}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1D938954-A429-4262-B9BF-E0CC33E3FD97}">
+          <x14:cfRule type="dataBar" id="{58C0BD30-2288-4427-8643-F3A161E068CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{934CD0BF-67ED-4044-9417-63BBA08616D0}">
+          <x14:cfRule type="dataBar" id="{049F3817-33DC-4DD2-B793-26272D793A56}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{189FE16B-3C45-4ED1-AB74-1743FBFD26CD}</x14:id>
+          <x14:id>{4EC02170-73DC-434D-9A84-F8BA250DBC60}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C0303A87-0D95-46B3-B072-5255187D7CD8}</x14:id>
+          <x14:id>{52D55F30-454D-4441-842B-ADBD56BE2C01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D6FB19C9-FA9B-42C8-A690-0EF33CBBB311}</x14:id>
+          <x14:id>{D30F656D-98F1-4CC8-BE26-718ABE82AABD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C54E5308-87FF-4C8B-AF5D-05F6CC3FC8F2}</x14:id>
+          <x14:id>{487C563C-1CB1-4CA4-96F2-1C7F272AAC51}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{189FE16B-3C45-4ED1-AB74-1743FBFD26CD}">
+          <x14:cfRule type="dataBar" id="{4EC02170-73DC-434D-9A84-F8BA250DBC60}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C0303A87-0D95-46B3-B072-5255187D7CD8}">
+          <x14:cfRule type="dataBar" id="{52D55F30-454D-4441-842B-ADBD56BE2C01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D6FB19C9-FA9B-42C8-A690-0EF33CBBB311}">
+          <x14:cfRule type="dataBar" id="{D30F656D-98F1-4CC8-BE26-718ABE82AABD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C54E5308-87FF-4C8B-AF5D-05F6CC3FC8F2}">
+          <x14:cfRule type="dataBar" id="{487C563C-1CB1-4CA4-96F2-1C7F272AAC51}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BDBEAD58-0142-4286-AE1A-9CF534495B01}</x14:id>
+          <x14:id>{07AE2089-9754-4886-BC47-D30335DA97EC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D09AC923-DEC1-494F-A3CC-ABE181B01602}</x14:id>
+          <x14:id>{D39A41A8-67F0-4E66-976A-6E595358760B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58C0BD30-2288-4427-8643-F3A161E068CB}</x14:id>
+          <x14:id>{A4879A86-4D08-40D8-8A93-FC8539AD2B0F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{049F3817-33DC-4DD2-B793-26272D793A56}</x14:id>
+          <x14:id>{BC8106AE-C825-4BE1-8753-9F733727C893}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BDBEAD58-0142-4286-AE1A-9CF534495B01}">
+          <x14:cfRule type="dataBar" id="{07AE2089-9754-4886-BC47-D30335DA97EC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D09AC923-DEC1-494F-A3CC-ABE181B01602}">
+          <x14:cfRule type="dataBar" id="{D39A41A8-67F0-4E66-976A-6E595358760B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58C0BD30-2288-4427-8643-F3A161E068CB}">
+          <x14:cfRule type="dataBar" id="{A4879A86-4D08-40D8-8A93-FC8539AD2B0F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{049F3817-33DC-4DD2-B793-26272D793A56}">
+          <x14:cfRule type="dataBar" id="{BC8106AE-C825-4BE1-8753-9F733727C893}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4EC02170-73DC-434D-9A84-F8BA250DBC60}</x14:id>
+          <x14:id>{A99E49C9-82BB-4DBA-ABC4-AF1E3DC61D39}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{52D55F30-454D-4441-842B-ADBD56BE2C01}</x14:id>
+          <x14:id>{7DC85811-50C7-4C13-B403-945A9212E6F8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D30F656D-98F1-4CC8-BE26-718ABE82AABD}</x14:id>
+          <x14:id>{2EA09098-0B52-4513-983C-4F32544C9DCA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{487C563C-1CB1-4CA4-96F2-1C7F272AAC51}</x14:id>
+          <x14:id>{02D56062-0C7E-4B56-9E76-A142B9C3965F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4EC02170-73DC-434D-9A84-F8BA250DBC60}">
+          <x14:cfRule type="dataBar" id="{A99E49C9-82BB-4DBA-ABC4-AF1E3DC61D39}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{52D55F30-454D-4441-842B-ADBD56BE2C01}">
+          <x14:cfRule type="dataBar" id="{7DC85811-50C7-4C13-B403-945A9212E6F8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D30F656D-98F1-4CC8-BE26-718ABE82AABD}">
+          <x14:cfRule type="dataBar" id="{2EA09098-0B52-4513-983C-4F32544C9DCA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{487C563C-1CB1-4CA4-96F2-1C7F272AAC51}">
+          <x14:cfRule type="dataBar" id="{02D56062-0C7E-4B56-9E76-A142B9C3965F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07AE2089-9754-4886-BC47-D30335DA97EC}</x14:id>
+          <x14:id>{8020CA06-28F3-45CE-A154-769AEA64710E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D39A41A8-67F0-4E66-976A-6E595358760B}</x14:id>
+          <x14:id>{2ADBA456-B365-47AD-B2AD-BFE8510DEFF7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A4879A86-4D08-40D8-8A93-FC8539AD2B0F}</x14:id>
+          <x14:id>{95C069C2-2A1C-4C30-8C1A-B01B80D131A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC8106AE-C825-4BE1-8753-9F733727C893}</x14:id>
+          <x14:id>{5453DA97-2468-4578-B036-808C4B027967}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07AE2089-9754-4886-BC47-D30335DA97EC}">
+          <x14:cfRule type="dataBar" id="{8020CA06-28F3-45CE-A154-769AEA64710E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D39A41A8-67F0-4E66-976A-6E595358760B}">
+          <x14:cfRule type="dataBar" id="{2ADBA456-B365-47AD-B2AD-BFE8510DEFF7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A4879A86-4D08-40D8-8A93-FC8539AD2B0F}">
+          <x14:cfRule type="dataBar" id="{95C069C2-2A1C-4C30-8C1A-B01B80D131A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC8106AE-C825-4BE1-8753-9F733727C893}">
+          <x14:cfRule type="dataBar" id="{5453DA97-2468-4578-B036-808C4B027967}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A99E49C9-82BB-4DBA-ABC4-AF1E3DC61D39}</x14:id>
+          <x14:id>{D08E561D-9C61-4A60-9990-555B2F47B008}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7DC85811-50C7-4C13-B403-945A9212E6F8}</x14:id>
+          <x14:id>{3062EB0B-BEC3-486B-869C-6185BCC9207B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2EA09098-0B52-4513-983C-4F32544C9DCA}</x14:id>
+          <x14:id>{F8A7D818-97AF-4D23-95C5-D5482D353FA7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{02D56062-0C7E-4B56-9E76-A142B9C3965F}</x14:id>
+          <x14:id>{548D801F-053D-48CC-88D4-B917240692BB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A99E49C9-82BB-4DBA-ABC4-AF1E3DC61D39}">
+          <x14:cfRule type="dataBar" id="{D08E561D-9C61-4A60-9990-555B2F47B008}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7DC85811-50C7-4C13-B403-945A9212E6F8}">
+          <x14:cfRule type="dataBar" id="{3062EB0B-BEC3-486B-869C-6185BCC9207B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2EA09098-0B52-4513-983C-4F32544C9DCA}">
+          <x14:cfRule type="dataBar" id="{F8A7D818-97AF-4D23-95C5-D5482D353FA7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{02D56062-0C7E-4B56-9E76-A142B9C3965F}">
+          <x14:cfRule type="dataBar" id="{548D801F-053D-48CC-88D4-B917240692BB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8020CA06-28F3-45CE-A154-769AEA64710E}</x14:id>
+          <x14:id>{AFD2DE3C-650E-47B8-90A0-D1371F81C64C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2ADBA456-B365-47AD-B2AD-BFE8510DEFF7}</x14:id>
+          <x14:id>{EC01439C-CEF4-4053-A999-3B3A459B1D76}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95C069C2-2A1C-4C30-8C1A-B01B80D131A2}</x14:id>
+          <x14:id>{66F8929B-9D60-4B2B-9E86-E850F7135615}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5453DA97-2468-4578-B036-808C4B027967}</x14:id>
+          <x14:id>{F64A9680-8644-476A-8034-603B572445E7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8020CA06-28F3-45CE-A154-769AEA64710E}">
+          <x14:cfRule type="dataBar" id="{AFD2DE3C-650E-47B8-90A0-D1371F81C64C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2ADBA456-B365-47AD-B2AD-BFE8510DEFF7}">
+          <x14:cfRule type="dataBar" id="{EC01439C-CEF4-4053-A999-3B3A459B1D76}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95C069C2-2A1C-4C30-8C1A-B01B80D131A2}">
+          <x14:cfRule type="dataBar" id="{66F8929B-9D60-4B2B-9E86-E850F7135615}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5453DA97-2468-4578-B036-808C4B027967}">
+          <x14:cfRule type="dataBar" id="{F64A9680-8644-476A-8034-603B572445E7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D08E561D-9C61-4A60-9990-555B2F47B008}</x14:id>
+          <x14:id>{132879BE-552B-49B7-8F79-6B6229D902B6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3062EB0B-BEC3-486B-869C-6185BCC9207B}</x14:id>
+          <x14:id>{D1587FD9-A9A1-4D04-B6DC-EDE8DE75DE69}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F8A7D818-97AF-4D23-95C5-D5482D353FA7}</x14:id>
+          <x14:id>{A0F95D52-C90A-485F-A1CC-41ED4CAFC8EB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{548D801F-053D-48CC-88D4-B917240692BB}</x14:id>
+          <x14:id>{7E64734A-9638-44DD-BFED-5DFC4F17077C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D08E561D-9C61-4A60-9990-555B2F47B008}">
+          <x14:cfRule type="dataBar" id="{132879BE-552B-49B7-8F79-6B6229D902B6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3062EB0B-BEC3-486B-869C-6185BCC9207B}">
+          <x14:cfRule type="dataBar" id="{D1587FD9-A9A1-4D04-B6DC-EDE8DE75DE69}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F8A7D818-97AF-4D23-95C5-D5482D353FA7}">
+          <x14:cfRule type="dataBar" id="{A0F95D52-C90A-485F-A1CC-41ED4CAFC8EB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{548D801F-053D-48CC-88D4-B917240692BB}">
+          <x14:cfRule type="dataBar" id="{7E64734A-9638-44DD-BFED-5DFC4F17077C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AFD2DE3C-650E-47B8-90A0-D1371F81C64C}</x14:id>
+          <x14:id>{4132B745-9E8C-400E-8C61-FA65EFEADCFF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC01439C-CEF4-4053-A999-3B3A459B1D76}</x14:id>
+          <x14:id>{41C75A7C-208C-4862-BF4C-A2ABAB42A8C1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66F8929B-9D60-4B2B-9E86-E850F7135615}</x14:id>
+          <x14:id>{EF9653EF-7858-41B6-9FD5-3853510BC12E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F64A9680-8644-476A-8034-603B572445E7}</x14:id>
+          <x14:id>{C142180E-7465-47DD-8B40-C14816153A13}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AFD2DE3C-650E-47B8-90A0-D1371F81C64C}">
+          <x14:cfRule type="dataBar" id="{4132B745-9E8C-400E-8C61-FA65EFEADCFF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC01439C-CEF4-4053-A999-3B3A459B1D76}">
+          <x14:cfRule type="dataBar" id="{41C75A7C-208C-4862-BF4C-A2ABAB42A8C1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66F8929B-9D60-4B2B-9E86-E850F7135615}">
+          <x14:cfRule type="dataBar" id="{EF9653EF-7858-41B6-9FD5-3853510BC12E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F64A9680-8644-476A-8034-603B572445E7}">
+          <x14:cfRule type="dataBar" id="{C142180E-7465-47DD-8B40-C14816153A13}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{132879BE-552B-49B7-8F79-6B6229D902B6}</x14:id>
+          <x14:id>{0CEAB687-FE7E-43EC-BBCC-EAC81AE65E52}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D1587FD9-A9A1-4D04-B6DC-EDE8DE75DE69}</x14:id>
+          <x14:id>{0923E224-7F8D-4236-BAB6-7FC981315466}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0F95D52-C90A-485F-A1CC-41ED4CAFC8EB}</x14:id>
+          <x14:id>{DE5FABEF-EFDE-4AF8-8A3D-99F7A4342CA8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E64734A-9638-44DD-BFED-5DFC4F17077C}</x14:id>
+          <x14:id>{582EA657-9D17-42F3-8C05-FCB64E8312D9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{132879BE-552B-49B7-8F79-6B6229D902B6}">
+          <x14:cfRule type="dataBar" id="{0CEAB687-FE7E-43EC-BBCC-EAC81AE65E52}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D1587FD9-A9A1-4D04-B6DC-EDE8DE75DE69}">
+          <x14:cfRule type="dataBar" id="{0923E224-7F8D-4236-BAB6-7FC981315466}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0F95D52-C90A-485F-A1CC-41ED4CAFC8EB}">
+          <x14:cfRule type="dataBar" id="{DE5FABEF-EFDE-4AF8-8A3D-99F7A4342CA8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E64734A-9638-44DD-BFED-5DFC4F17077C}">
+          <x14:cfRule type="dataBar" id="{582EA657-9D17-42F3-8C05-FCB64E8312D9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4132B745-9E8C-400E-8C61-FA65EFEADCFF}</x14:id>
+          <x14:id>{D4535937-FBBB-4CC0-BF3A-22F739E01424}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{41C75A7C-208C-4862-BF4C-A2ABAB42A8C1}</x14:id>
+          <x14:id>{117042FF-1499-4C07-9204-A1C3FF91C23D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EF9653EF-7858-41B6-9FD5-3853510BC12E}</x14:id>
+          <x14:id>{58AF6E51-8800-474A-9C0B-A6FFD754ED42}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C142180E-7465-47DD-8B40-C14816153A13}</x14:id>
+          <x14:id>{3BFE33E5-4C57-4993-8A77-6921073BA87C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4132B745-9E8C-400E-8C61-FA65EFEADCFF}">
+          <x14:cfRule type="dataBar" id="{D4535937-FBBB-4CC0-BF3A-22F739E01424}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{41C75A7C-208C-4862-BF4C-A2ABAB42A8C1}">
+          <x14:cfRule type="dataBar" id="{117042FF-1499-4C07-9204-A1C3FF91C23D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EF9653EF-7858-41B6-9FD5-3853510BC12E}">
+          <x14:cfRule type="dataBar" id="{58AF6E51-8800-474A-9C0B-A6FFD754ED42}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C142180E-7465-47DD-8B40-C14816153A13}">
+          <x14:cfRule type="dataBar" id="{3BFE33E5-4C57-4993-8A77-6921073BA87C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0CEAB687-FE7E-43EC-BBCC-EAC81AE65E52}</x14:id>
+          <x14:id>{2E6B99CC-7A1A-4D26-B2D1-8D918FEA2682}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0923E224-7F8D-4236-BAB6-7FC981315466}</x14:id>
+          <x14:id>{0373401D-56DC-4E7C-8D8A-C216BE28888D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DE5FABEF-EFDE-4AF8-8A3D-99F7A4342CA8}</x14:id>
+          <x14:id>{E4FCB12D-9E16-4A23-9261-E8F774E68A30}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{582EA657-9D17-42F3-8C05-FCB64E8312D9}</x14:id>
+          <x14:id>{9BB25B3A-6CB6-4A73-AAAD-9C11557AC6E5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0CEAB687-FE7E-43EC-BBCC-EAC81AE65E52}">
+          <x14:cfRule type="dataBar" id="{2E6B99CC-7A1A-4D26-B2D1-8D918FEA2682}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0923E224-7F8D-4236-BAB6-7FC981315466}">
+          <x14:cfRule type="dataBar" id="{0373401D-56DC-4E7C-8D8A-C216BE28888D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DE5FABEF-EFDE-4AF8-8A3D-99F7A4342CA8}">
+          <x14:cfRule type="dataBar" id="{E4FCB12D-9E16-4A23-9261-E8F774E68A30}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{582EA657-9D17-42F3-8C05-FCB64E8312D9}">
+          <x14:cfRule type="dataBar" id="{9BB25B3A-6CB6-4A73-AAAD-9C11557AC6E5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D4535937-FBBB-4CC0-BF3A-22F739E01424}</x14:id>
+          <x14:id>{EEB55794-6174-45E2-8FBC-1D8571C87E07}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{117042FF-1499-4C07-9204-A1C3FF91C23D}</x14:id>
+          <x14:id>{35CFF20D-5F39-4D2C-8B9D-4169CD40A366}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58AF6E51-8800-474A-9C0B-A6FFD754ED42}</x14:id>
+          <x14:id>{CD42E54D-6F06-44AC-9D4B-4C02700C37F5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3BFE33E5-4C57-4993-8A77-6921073BA87C}</x14:id>
+          <x14:id>{F08D00A1-F436-44A2-B925-4D27F51C2A0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D4535937-FBBB-4CC0-BF3A-22F739E01424}">
+          <x14:cfRule type="dataBar" id="{EEB55794-6174-45E2-8FBC-1D8571C87E07}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{117042FF-1499-4C07-9204-A1C3FF91C23D}">
+          <x14:cfRule type="dataBar" id="{35CFF20D-5F39-4D2C-8B9D-4169CD40A366}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58AF6E51-8800-474A-9C0B-A6FFD754ED42}">
+          <x14:cfRule type="dataBar" id="{CD42E54D-6F06-44AC-9D4B-4C02700C37F5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3BFE33E5-4C57-4993-8A77-6921073BA87C}">
+          <x14:cfRule type="dataBar" id="{F08D00A1-F436-44A2-B925-4D27F51C2A0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E6B99CC-7A1A-4D26-B2D1-8D918FEA2682}</x14:id>
+          <x14:id>{3C7CBC62-A517-4948-931C-C833D694B571}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0373401D-56DC-4E7C-8D8A-C216BE28888D}</x14:id>
+          <x14:id>{BD8CCE90-2E04-4304-9256-7549EF43D9DF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4FCB12D-9E16-4A23-9261-E8F774E68A30}</x14:id>
+          <x14:id>{B4A5DF3C-0A87-4D55-A0BE-F2AE0346C373}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9BB25B3A-6CB6-4A73-AAAD-9C11557AC6E5}</x14:id>
+          <x14:id>{A185A4D8-1A22-4D0C-810A-99341E2AE940}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E6B99CC-7A1A-4D26-B2D1-8D918FEA2682}">
+          <x14:cfRule type="dataBar" id="{3C7CBC62-A517-4948-931C-C833D694B571}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0373401D-56DC-4E7C-8D8A-C216BE28888D}">
+          <x14:cfRule type="dataBar" id="{BD8CCE90-2E04-4304-9256-7549EF43D9DF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4FCB12D-9E16-4A23-9261-E8F774E68A30}">
+          <x14:cfRule type="dataBar" id="{B4A5DF3C-0A87-4D55-A0BE-F2AE0346C373}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9BB25B3A-6CB6-4A73-AAAD-9C11557AC6E5}">
+          <x14:cfRule type="dataBar" id="{A185A4D8-1A22-4D0C-810A-99341E2AE940}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEB55794-6174-45E2-8FBC-1D8571C87E07}</x14:id>
+          <x14:id>{5F689630-8868-4AB7-8F86-1FCC59BEB3AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{35CFF20D-5F39-4D2C-8B9D-4169CD40A366}</x14:id>
+          <x14:id>{510167E7-7F6D-4D50-9B3F-F4C92DC4F92E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD42E54D-6F06-44AC-9D4B-4C02700C37F5}</x14:id>
+          <x14:id>{33FF2834-EEDD-4437-B16D-040079F825E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F08D00A1-F436-44A2-B925-4D27F51C2A0B}</x14:id>
+          <x14:id>{6BE374C2-C10E-4A7C-AB09-4CF5FFDEC3BC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEB55794-6174-45E2-8FBC-1D8571C87E07}">
+          <x14:cfRule type="dataBar" id="{5F689630-8868-4AB7-8F86-1FCC59BEB3AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{35CFF20D-5F39-4D2C-8B9D-4169CD40A366}">
+          <x14:cfRule type="dataBar" id="{510167E7-7F6D-4D50-9B3F-F4C92DC4F92E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD42E54D-6F06-44AC-9D4B-4C02700C37F5}">
+          <x14:cfRule type="dataBar" id="{33FF2834-EEDD-4437-B16D-040079F825E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F08D00A1-F436-44A2-B925-4D27F51C2A0B}">
+          <x14:cfRule type="dataBar" id="{6BE374C2-C10E-4A7C-AB09-4CF5FFDEC3BC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3C7CBC62-A517-4948-931C-C833D694B571}</x14:id>
+          <x14:id>{3165569F-703B-41FC-B235-98528853FFAA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BD8CCE90-2E04-4304-9256-7549EF43D9DF}</x14:id>
+          <x14:id>{4FB4E81F-9654-40A8-8BC5-6A26B17C0C2D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B4A5DF3C-0A87-4D55-A0BE-F2AE0346C373}</x14:id>
+          <x14:id>{C0C1B8EF-AAC8-464A-B5B9-0B54EEE113B6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A185A4D8-1A22-4D0C-810A-99341E2AE940}</x14:id>
+          <x14:id>{CEA8736D-E58D-4103-A39F-B51DBB02E23D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3C7CBC62-A517-4948-931C-C833D694B571}">
+          <x14:cfRule type="dataBar" id="{3165569F-703B-41FC-B235-98528853FFAA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BD8CCE90-2E04-4304-9256-7549EF43D9DF}">
+          <x14:cfRule type="dataBar" id="{4FB4E81F-9654-40A8-8BC5-6A26B17C0C2D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B4A5DF3C-0A87-4D55-A0BE-F2AE0346C373}">
+          <x14:cfRule type="dataBar" id="{C0C1B8EF-AAC8-464A-B5B9-0B54EEE113B6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A185A4D8-1A22-4D0C-810A-99341E2AE940}">
+          <x14:cfRule type="dataBar" id="{CEA8736D-E58D-4103-A39F-B51DBB02E23D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5F689630-8868-4AB7-8F86-1FCC59BEB3AF}</x14:id>
+          <x14:id>{F7459B57-F595-48A4-A054-1662CC822282}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{510167E7-7F6D-4D50-9B3F-F4C92DC4F92E}</x14:id>
+          <x14:id>{4B40C42C-A2E6-4C3F-9706-B6D8021CC9DC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{33FF2834-EEDD-4437-B16D-040079F825E6}</x14:id>
+          <x14:id>{6B85DB42-5D8A-4409-BB6F-E5C89FF0AB42}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6BE374C2-C10E-4A7C-AB09-4CF5FFDEC3BC}</x14:id>
+          <x14:id>{A2B404B4-1D0A-45EA-BDF6-08E7F9D2B5D3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5F689630-8868-4AB7-8F86-1FCC59BEB3AF}">
+          <x14:cfRule type="dataBar" id="{F7459B57-F595-48A4-A054-1662CC822282}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{510167E7-7F6D-4D50-9B3F-F4C92DC4F92E}">
+          <x14:cfRule type="dataBar" id="{4B40C42C-A2E6-4C3F-9706-B6D8021CC9DC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{33FF2834-EEDD-4437-B16D-040079F825E6}">
+          <x14:cfRule type="dataBar" id="{6B85DB42-5D8A-4409-BB6F-E5C89FF0AB42}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6BE374C2-C10E-4A7C-AB09-4CF5FFDEC3BC}">
+          <x14:cfRule type="dataBar" id="{A2B404B4-1D0A-45EA-BDF6-08E7F9D2B5D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3165569F-703B-41FC-B235-98528853FFAA}</x14:id>
+          <x14:id>{A29E1BD2-EEB1-4932-BA12-CBD512EBF4DC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4FB4E81F-9654-40A8-8BC5-6A26B17C0C2D}</x14:id>
+          <x14:id>{8F2769A9-F17D-4B3D-8190-8D7E8067C450}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C0C1B8EF-AAC8-464A-B5B9-0B54EEE113B6}</x14:id>
+          <x14:id>{3E82D2DE-5934-4025-96C6-5CA4FF77FC20}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CEA8736D-E58D-4103-A39F-B51DBB02E23D}</x14:id>
+          <x14:id>{567F87D9-9CCF-46E9-AEF0-C358D941D7D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3165569F-703B-41FC-B235-98528853FFAA}">
+          <x14:cfRule type="dataBar" id="{A29E1BD2-EEB1-4932-BA12-CBD512EBF4DC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4FB4E81F-9654-40A8-8BC5-6A26B17C0C2D}">
+          <x14:cfRule type="dataBar" id="{8F2769A9-F17D-4B3D-8190-8D7E8067C450}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C0C1B8EF-AAC8-464A-B5B9-0B54EEE113B6}">
+          <x14:cfRule type="dataBar" id="{3E82D2DE-5934-4025-96C6-5CA4FF77FC20}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CEA8736D-E58D-4103-A39F-B51DBB02E23D}">
+          <x14:cfRule type="dataBar" id="{567F87D9-9CCF-46E9-AEF0-C358D941D7D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F7459B57-F595-48A4-A054-1662CC822282}</x14:id>
+          <x14:id>{08A21B32-58BD-4BB5-B819-ED273CE2DA88}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4B40C42C-A2E6-4C3F-9706-B6D8021CC9DC}</x14:id>
+          <x14:id>{33BFEC8F-3ABF-4DD2-AE1B-FED4A186DA14}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B85DB42-5D8A-4409-BB6F-E5C89FF0AB42}</x14:id>
+          <x14:id>{853B59FF-F3E7-444F-8BEE-2CC73F632E28}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A2B404B4-1D0A-45EA-BDF6-08E7F9D2B5D3}</x14:id>
+          <x14:id>{3EFF047E-72F3-41F8-B636-90458A6BEBF7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F7459B57-F595-48A4-A054-1662CC822282}">
+          <x14:cfRule type="dataBar" id="{08A21B32-58BD-4BB5-B819-ED273CE2DA88}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4B40C42C-A2E6-4C3F-9706-B6D8021CC9DC}">
+          <x14:cfRule type="dataBar" id="{33BFEC8F-3ABF-4DD2-AE1B-FED4A186DA14}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B85DB42-5D8A-4409-BB6F-E5C89FF0AB42}">
+          <x14:cfRule type="dataBar" id="{853B59FF-F3E7-444F-8BEE-2CC73F632E28}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A2B404B4-1D0A-45EA-BDF6-08E7F9D2B5D3}">
+          <x14:cfRule type="dataBar" id="{3EFF047E-72F3-41F8-B636-90458A6BEBF7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A29E1BD2-EEB1-4932-BA12-CBD512EBF4DC}</x14:id>
+          <x14:id>{8D34CA7B-57EE-406C-9DFA-79FA3922B0E5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F2769A9-F17D-4B3D-8190-8D7E8067C450}</x14:id>
+          <x14:id>{026BA282-A3EA-4AE2-92B7-08B80DD71491}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3E82D2DE-5934-4025-96C6-5CA4FF77FC20}</x14:id>
+          <x14:id>{5195D95E-2B49-4FE5-9DE5-BA4CE4DBAD7B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{567F87D9-9CCF-46E9-AEF0-C358D941D7D0}</x14:id>
+          <x14:id>{411A81E9-87D2-48BE-A37B-DAB55C5326FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A29E1BD2-EEB1-4932-BA12-CBD512EBF4DC}">
+          <x14:cfRule type="dataBar" id="{8D34CA7B-57EE-406C-9DFA-79FA3922B0E5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F2769A9-F17D-4B3D-8190-8D7E8067C450}">
+          <x14:cfRule type="dataBar" id="{026BA282-A3EA-4AE2-92B7-08B80DD71491}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3E82D2DE-5934-4025-96C6-5CA4FF77FC20}">
+          <x14:cfRule type="dataBar" id="{5195D95E-2B49-4FE5-9DE5-BA4CE4DBAD7B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{567F87D9-9CCF-46E9-AEF0-C358D941D7D0}">
+          <x14:cfRule type="dataBar" id="{411A81E9-87D2-48BE-A37B-DAB55C5326FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{08A21B32-58BD-4BB5-B819-ED273CE2DA88}</x14:id>
+          <x14:id>{49887AD6-34B4-4A57-8B93-AAA7702BF4B8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{33BFEC8F-3ABF-4DD2-AE1B-FED4A186DA14}</x14:id>
+          <x14:id>{E9636D68-EEFD-438E-8893-4A2535C15695}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{853B59FF-F3E7-444F-8BEE-2CC73F632E28}</x14:id>
+          <x14:id>{3F91D15D-5EBA-431B-8C23-CFB6D59BF588}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3EFF047E-72F3-41F8-B636-90458A6BEBF7}</x14:id>
+          <x14:id>{16352CD1-DDC1-4A30-AB48-B84A3D150080}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{08A21B32-58BD-4BB5-B819-ED273CE2DA88}">
+          <x14:cfRule type="dataBar" id="{49887AD6-34B4-4A57-8B93-AAA7702BF4B8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{33BFEC8F-3ABF-4DD2-AE1B-FED4A186DA14}">
+          <x14:cfRule type="dataBar" id="{E9636D68-EEFD-438E-8893-4A2535C15695}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{853B59FF-F3E7-444F-8BEE-2CC73F632E28}">
+          <x14:cfRule type="dataBar" id="{3F91D15D-5EBA-431B-8C23-CFB6D59BF588}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3EFF047E-72F3-41F8-B636-90458A6BEBF7}">
+          <x14:cfRule type="dataBar" id="{16352CD1-DDC1-4A30-AB48-B84A3D150080}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8D34CA7B-57EE-406C-9DFA-79FA3922B0E5}</x14:id>
+          <x14:id>{83F27422-A5AD-47F0-B6F0-ADEAE9409CF4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{026BA282-A3EA-4AE2-92B7-08B80DD71491}</x14:id>
+          <x14:id>{5EBF3103-38AD-4B8C-BBC1-D1D9C9CC2486}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5195D95E-2B49-4FE5-9DE5-BA4CE4DBAD7B}</x14:id>
+          <x14:id>{F073DE64-0E56-44F0-BAB3-50D7D3BF8C86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{411A81E9-87D2-48BE-A37B-DAB55C5326FD}</x14:id>
+          <x14:id>{F27C47D1-D564-4C6E-97F4-696A457D1F8A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8D34CA7B-57EE-406C-9DFA-79FA3922B0E5}">
+          <x14:cfRule type="dataBar" id="{83F27422-A5AD-47F0-B6F0-ADEAE9409CF4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{026BA282-A3EA-4AE2-92B7-08B80DD71491}">
+          <x14:cfRule type="dataBar" id="{5EBF3103-38AD-4B8C-BBC1-D1D9C9CC2486}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5195D95E-2B49-4FE5-9DE5-BA4CE4DBAD7B}">
+          <x14:cfRule type="dataBar" id="{F073DE64-0E56-44F0-BAB3-50D7D3BF8C86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{411A81E9-87D2-48BE-A37B-DAB55C5326FD}">
+          <x14:cfRule type="dataBar" id="{F27C47D1-D564-4C6E-97F4-696A457D1F8A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49887AD6-34B4-4A57-8B93-AAA7702BF4B8}</x14:id>
+          <x14:id>{A10DC1B8-A849-4525-87F8-DC7676CE67B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E9636D68-EEFD-438E-8893-4A2535C15695}</x14:id>
+          <x14:id>{CE1147CE-91A6-4475-9443-58D5902EDDE7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3F91D15D-5EBA-431B-8C23-CFB6D59BF588}</x14:id>
+          <x14:id>{99B2CC16-C381-43DA-AF3E-BF1DE8AE2154}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{16352CD1-DDC1-4A30-AB48-B84A3D150080}</x14:id>
+          <x14:id>{9062987E-F598-4B94-B852-DA11937941C3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49887AD6-34B4-4A57-8B93-AAA7702BF4B8}">
+          <x14:cfRule type="dataBar" id="{A10DC1B8-A849-4525-87F8-DC7676CE67B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E9636D68-EEFD-438E-8893-4A2535C15695}">
+          <x14:cfRule type="dataBar" id="{CE1147CE-91A6-4475-9443-58D5902EDDE7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3F91D15D-5EBA-431B-8C23-CFB6D59BF588}">
+          <x14:cfRule type="dataBar" id="{99B2CC16-C381-43DA-AF3E-BF1DE8AE2154}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{16352CD1-DDC1-4A30-AB48-B84A3D150080}">
+          <x14:cfRule type="dataBar" id="{9062987E-F598-4B94-B852-DA11937941C3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{83F27422-A5AD-47F0-B6F0-ADEAE9409CF4}</x14:id>
+          <x14:id>{4D28500C-F2A9-4F31-9239-89BB6FED021F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5EBF3103-38AD-4B8C-BBC1-D1D9C9CC2486}</x14:id>
+          <x14:id>{19D3A8D0-02E1-4490-87B8-7968F68C7295}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F073DE64-0E56-44F0-BAB3-50D7D3BF8C86}</x14:id>
+          <x14:id>{792E054F-3D1C-48F7-942E-C75501754BCD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F27C47D1-D564-4C6E-97F4-696A457D1F8A}</x14:id>
+          <x14:id>{6D46BE9B-8CB7-4B51-B0F9-FF6D34F15F90}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{83F27422-A5AD-47F0-B6F0-ADEAE9409CF4}">
+          <x14:cfRule type="dataBar" id="{4D28500C-F2A9-4F31-9239-89BB6FED021F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5EBF3103-38AD-4B8C-BBC1-D1D9C9CC2486}">
+          <x14:cfRule type="dataBar" id="{19D3A8D0-02E1-4490-87B8-7968F68C7295}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F073DE64-0E56-44F0-BAB3-50D7D3BF8C86}">
+          <x14:cfRule type="dataBar" id="{792E054F-3D1C-48F7-942E-C75501754BCD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F27C47D1-D564-4C6E-97F4-696A457D1F8A}">
+          <x14:cfRule type="dataBar" id="{6D46BE9B-8CB7-4B51-B0F9-FF6D34F15F90}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A10DC1B8-A849-4525-87F8-DC7676CE67B0}</x14:id>
+          <x14:id>{14C6F1D7-0CD3-4652-884A-A602AD31E9ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CE1147CE-91A6-4475-9443-58D5902EDDE7}</x14:id>
+          <x14:id>{CF91B040-930B-45D6-8123-CBC820DD1892}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99B2CC16-C381-43DA-AF3E-BF1DE8AE2154}</x14:id>
+          <x14:id>{0CF31A5A-264C-4258-A080-A6EF7BD48645}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9062987E-F598-4B94-B852-DA11937941C3}</x14:id>
+          <x14:id>{AF06107D-018A-40FF-918D-81BEA97902D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A10DC1B8-A849-4525-87F8-DC7676CE67B0}">
+          <x14:cfRule type="dataBar" id="{14C6F1D7-0CD3-4652-884A-A602AD31E9ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CE1147CE-91A6-4475-9443-58D5902EDDE7}">
+          <x14:cfRule type="dataBar" id="{CF91B040-930B-45D6-8123-CBC820DD1892}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99B2CC16-C381-43DA-AF3E-BF1DE8AE2154}">
+          <x14:cfRule type="dataBar" id="{0CF31A5A-264C-4258-A080-A6EF7BD48645}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9062987E-F598-4B94-B852-DA11937941C3}">
+          <x14:cfRule type="dataBar" id="{AF06107D-018A-40FF-918D-81BEA97902D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4D28500C-F2A9-4F31-9239-89BB6FED021F}</x14:id>
+          <x14:id>{2F284888-F710-4624-895A-E16F11C19C65}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19D3A8D0-02E1-4490-87B8-7968F68C7295}</x14:id>
+          <x14:id>{86C465F7-A7DE-4867-8753-34B5D68C7A85}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{792E054F-3D1C-48F7-942E-C75501754BCD}</x14:id>
+          <x14:id>{F65EE673-22BF-4D96-84D9-6C3071D7EC9F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D46BE9B-8CB7-4B51-B0F9-FF6D34F15F90}</x14:id>
+          <x14:id>{F6C37D5D-7F34-430E-90BE-B7E7BD858E90}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4D28500C-F2A9-4F31-9239-89BB6FED021F}">
+          <x14:cfRule type="dataBar" id="{2F284888-F710-4624-895A-E16F11C19C65}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19D3A8D0-02E1-4490-87B8-7968F68C7295}">
+          <x14:cfRule type="dataBar" id="{86C465F7-A7DE-4867-8753-34B5D68C7A85}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{792E054F-3D1C-48F7-942E-C75501754BCD}">
+          <x14:cfRule type="dataBar" id="{F65EE673-22BF-4D96-84D9-6C3071D7EC9F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D46BE9B-8CB7-4B51-B0F9-FF6D34F15F90}">
+          <x14:cfRule type="dataBar" id="{F6C37D5D-7F34-430E-90BE-B7E7BD858E90}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{14C6F1D7-0CD3-4652-884A-A602AD31E9ED}</x14:id>
+          <x14:id>{F59CFC9D-A9D2-417C-A667-36E01998D2AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CF91B040-930B-45D6-8123-CBC820DD1892}</x14:id>
+          <x14:id>{AFF5BCFC-7B5C-43DF-B3AB-565DB43D35BF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0CF31A5A-264C-4258-A080-A6EF7BD48645}</x14:id>
+          <x14:id>{C6314353-CF5F-4381-A3C3-D12E5909EB33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF06107D-018A-40FF-918D-81BEA97902D0}</x14:id>
+          <x14:id>{122F383C-9B2D-4F0F-ABF6-8BFE325491BF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{14C6F1D7-0CD3-4652-884A-A602AD31E9ED}">
+          <x14:cfRule type="dataBar" id="{F59CFC9D-A9D2-417C-A667-36E01998D2AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CF91B040-930B-45D6-8123-CBC820DD1892}">
+          <x14:cfRule type="dataBar" id="{AFF5BCFC-7B5C-43DF-B3AB-565DB43D35BF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0CF31A5A-264C-4258-A080-A6EF7BD48645}">
+          <x14:cfRule type="dataBar" id="{C6314353-CF5F-4381-A3C3-D12E5909EB33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF06107D-018A-40FF-918D-81BEA97902D0}">
+          <x14:cfRule type="dataBar" id="{122F383C-9B2D-4F0F-ABF6-8BFE325491BF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2F284888-F710-4624-895A-E16F11C19C65}</x14:id>
+          <x14:id>{1B932935-6280-4CB2-A2EC-4AB047725D9D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{86C465F7-A7DE-4867-8753-34B5D68C7A85}</x14:id>
+          <x14:id>{7FE5DA38-FEB0-4658-95E8-7BD47743B613}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F65EE673-22BF-4D96-84D9-6C3071D7EC9F}</x14:id>
+          <x14:id>{8220CE15-98AE-4797-BC2E-AA5A47349F53}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F6C37D5D-7F34-430E-90BE-B7E7BD858E90}</x14:id>
+          <x14:id>{7116F4BE-55C4-4DB3-A8F8-DF7ADF19F5A7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2F284888-F710-4624-895A-E16F11C19C65}">
+          <x14:cfRule type="dataBar" id="{1B932935-6280-4CB2-A2EC-4AB047725D9D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{86C465F7-A7DE-4867-8753-34B5D68C7A85}">
+          <x14:cfRule type="dataBar" id="{7FE5DA38-FEB0-4658-95E8-7BD47743B613}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F65EE673-22BF-4D96-84D9-6C3071D7EC9F}">
+          <x14:cfRule type="dataBar" id="{8220CE15-98AE-4797-BC2E-AA5A47349F53}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F6C37D5D-7F34-430E-90BE-B7E7BD858E90}">
+          <x14:cfRule type="dataBar" id="{7116F4BE-55C4-4DB3-A8F8-DF7ADF19F5A7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-27 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -10643,7 +10643,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F59CFC9D-A9D2-417C-A667-36E01998D2AC}</x14:id>
+          <x14:id>{9440D91B-DBBB-4BB7-B385-3462FBB203A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10657,7 +10657,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AFF5BCFC-7B5C-43DF-B3AB-565DB43D35BF}</x14:id>
+          <x14:id>{F2476145-C04B-40E5-B7A5-9C396BA37E06}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10671,7 +10671,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6314353-CF5F-4381-A3C3-D12E5909EB33}</x14:id>
+          <x14:id>{C6816D40-92C9-4F30-BB29-56A978725A7A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10685,7 +10685,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{122F383C-9B2D-4F0F-ABF6-8BFE325491BF}</x14:id>
+          <x14:id>{BDA7638F-5C6D-414D-BFF0-69F369466DC4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10695,7 +10695,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F59CFC9D-A9D2-417C-A667-36E01998D2AC}">
+          <x14:cfRule type="dataBar" id="{9440D91B-DBBB-4BB7-B385-3462FBB203A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10708,7 +10708,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AFF5BCFC-7B5C-43DF-B3AB-565DB43D35BF}">
+          <x14:cfRule type="dataBar" id="{F2476145-C04B-40E5-B7A5-9C396BA37E06}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10721,7 +10721,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6314353-CF5F-4381-A3C3-D12E5909EB33}">
+          <x14:cfRule type="dataBar" id="{C6816D40-92C9-4F30-BB29-56A978725A7A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10734,7 +10734,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{122F383C-9B2D-4F0F-ABF6-8BFE325491BF}">
+          <x14:cfRule type="dataBar" id="{BDA7638F-5C6D-414D-BFF0-69F369466DC4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26178,7 +26178,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1B932935-6280-4CB2-A2EC-4AB047725D9D}</x14:id>
+          <x14:id>{F89EA3BB-1D19-44BC-B3C3-B518111CD700}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26192,7 +26192,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7FE5DA38-FEB0-4658-95E8-7BD47743B613}</x14:id>
+          <x14:id>{D63212F1-1B0D-45BF-B394-4D76111D618B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26206,7 +26206,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8220CE15-98AE-4797-BC2E-AA5A47349F53}</x14:id>
+          <x14:id>{9F602EF3-7E3A-4CCD-A4DA-7D54DD08C671}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26220,7 +26220,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7116F4BE-55C4-4DB3-A8F8-DF7ADF19F5A7}</x14:id>
+          <x14:id>{F708126F-FFAF-4CB0-B58A-96BFCEFEA790}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26230,7 +26230,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1B932935-6280-4CB2-A2EC-4AB047725D9D}">
+          <x14:cfRule type="dataBar" id="{F89EA3BB-1D19-44BC-B3C3-B518111CD700}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26243,7 +26243,7 @@
           <xm:sqref>N6:N175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7FE5DA38-FEB0-4658-95E8-7BD47743B613}">
+          <x14:cfRule type="dataBar" id="{D63212F1-1B0D-45BF-B394-4D76111D618B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26256,7 +26256,7 @@
           <xm:sqref>P6:P175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8220CE15-98AE-4797-BC2E-AA5A47349F53}">
+          <x14:cfRule type="dataBar" id="{9F602EF3-7E3A-4CCD-A4DA-7D54DD08C671}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26269,7 +26269,7 @@
           <xm:sqref>Y6:Y175</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7116F4BE-55C4-4DB3-A8F8-DF7ADF19F5A7}">
+          <x14:cfRule type="dataBar" id="{F708126F-FFAF-4CB0-B58A-96BFCEFEA790}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-28 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -11549,7 +11549,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EB8E8D25-1788-4999-83D9-94F182BD1058}</x14:id>
+          <x14:id>{69D09703-A792-4FEC-A5B6-08FB545DAB60}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11563,7 +11563,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{46066A37-D924-4E63-AB37-E5B232D10FC3}</x14:id>
+          <x14:id>{75235CC8-33CE-4C51-9DC7-6FCFC9543C33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11577,7 +11577,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7FA6CB6A-EDFD-4B43-BA61-5218320105BC}</x14:id>
+          <x14:id>{4924861B-5DF4-4FE3-84BD-DF213C11FD22}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11591,7 +11591,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84AFB452-677F-49F4-B2F7-2C0FA9A8F5A9}</x14:id>
+          <x14:id>{1B439DCF-6B33-4F0D-B5B9-214D1299F001}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11601,7 +11601,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EB8E8D25-1788-4999-83D9-94F182BD1058}">
+          <x14:cfRule type="dataBar" id="{69D09703-A792-4FEC-A5B6-08FB545DAB60}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11614,7 +11614,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{46066A37-D924-4E63-AB37-E5B232D10FC3}">
+          <x14:cfRule type="dataBar" id="{75235CC8-33CE-4C51-9DC7-6FCFC9543C33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11627,7 +11627,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7FA6CB6A-EDFD-4B43-BA61-5218320105BC}">
+          <x14:cfRule type="dataBar" id="{4924861B-5DF4-4FE3-84BD-DF213C11FD22}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11640,7 +11640,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84AFB452-677F-49F4-B2F7-2C0FA9A8F5A9}">
+          <x14:cfRule type="dataBar" id="{1B439DCF-6B33-4F0D-B5B9-214D1299F001}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27025,7 +27025,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3E15F2C6-BE35-44F0-A0BA-A9A5E6463252}</x14:id>
+          <x14:id>{3F44ED14-49E1-4818-93BA-0365ECB8A815}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27039,7 +27039,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7CB3A95D-EB71-47B1-93EB-B5AEC4FEE6FA}</x14:id>
+          <x14:id>{C2B17F28-E24B-4C39-BFA6-93E182C4D0E8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27053,7 +27053,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3B1275C6-C44A-4A70-B467-0D3162C4A97C}</x14:id>
+          <x14:id>{07AAE745-56C1-4CC9-A7BA-0DCA774A0D7A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27067,7 +27067,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11BE290D-2EBB-4449-934A-2FCB099793B7}</x14:id>
+          <x14:id>{110C5405-8172-4F89-9D80-26D8CFA4E4DF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27077,7 +27077,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3E15F2C6-BE35-44F0-A0BA-A9A5E6463252}">
+          <x14:cfRule type="dataBar" id="{3F44ED14-49E1-4818-93BA-0365ECB8A815}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27090,7 +27090,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7CB3A95D-EB71-47B1-93EB-B5AEC4FEE6FA}">
+          <x14:cfRule type="dataBar" id="{C2B17F28-E24B-4C39-BFA6-93E182C4D0E8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27103,7 +27103,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3B1275C6-C44A-4A70-B467-0D3162C4A97C}">
+          <x14:cfRule type="dataBar" id="{07AAE745-56C1-4CC9-A7BA-0DCA774A0D7A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27116,7 +27116,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11BE290D-2EBB-4449-934A-2FCB099793B7}">
+          <x14:cfRule type="dataBar" id="{110C5405-8172-4F89-9D80-26D8CFA4E4DF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1266B2F7-4265-4B98-9A8D-FA86761B92FD}</x14:id>
+          <x14:id>{105EED5F-FE9A-412F-AFF1-4ED27E34FC47}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3ED1C793-EEE5-4CB1-9775-64004142924E}</x14:id>
+          <x14:id>{0C054CD4-E2CF-4477-B402-F8B25FE004F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FB640C01-64A5-4E7E-B253-F92CEF50537D}</x14:id>
+          <x14:id>{C532B192-3C36-461E-BE07-9730D97CE494}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5479BDB6-0BF4-4264-8506-F9B6DBBFCD4A}</x14:id>
+          <x14:id>{B11E7DAE-36C3-4EEA-9BA4-92BDC244D882}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1266B2F7-4265-4B98-9A8D-FA86761B92FD}">
+          <x14:cfRule type="dataBar" id="{105EED5F-FE9A-412F-AFF1-4ED27E34FC47}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3ED1C793-EEE5-4CB1-9775-64004142924E}">
+          <x14:cfRule type="dataBar" id="{0C054CD4-E2CF-4477-B402-F8B25FE004F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FB640C01-64A5-4E7E-B253-F92CEF50537D}">
+          <x14:cfRule type="dataBar" id="{C532B192-3C36-461E-BE07-9730D97CE494}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5479BDB6-0BF4-4264-8506-F9B6DBBFCD4A}">
+          <x14:cfRule type="dataBar" id="{B11E7DAE-36C3-4EEA-9BA4-92BDC244D882}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{21A7879F-2514-4EAA-8FFD-6ED218A0D6C0}</x14:id>
+          <x14:id>{93426B34-7830-4C8E-9731-8B43C273D926}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C5010202-3821-4FF2-88DB-4BF0758A2565}</x14:id>
+          <x14:id>{8C0A1F01-7B6B-44BA-86C1-C0F3C41F99A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A901AF00-62AF-4F40-B9C1-FB001E35F45F}</x14:id>
+          <x14:id>{961B1072-FD6B-462B-88F8-8C8012FE303D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4B35C728-03DB-40CB-A755-15AFEF99AA6C}</x14:id>
+          <x14:id>{7C79B556-5707-423E-8062-13616BD63709}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{21A7879F-2514-4EAA-8FFD-6ED218A0D6C0}">
+          <x14:cfRule type="dataBar" id="{93426B34-7830-4C8E-9731-8B43C273D926}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C5010202-3821-4FF2-88DB-4BF0758A2565}">
+          <x14:cfRule type="dataBar" id="{8C0A1F01-7B6B-44BA-86C1-C0F3C41F99A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A901AF00-62AF-4F40-B9C1-FB001E35F45F}">
+          <x14:cfRule type="dataBar" id="{961B1072-FD6B-462B-88F8-8C8012FE303D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4B35C728-03DB-40CB-A755-15AFEF99AA6C}">
+          <x14:cfRule type="dataBar" id="{7C79B556-5707-423E-8062-13616BD63709}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{105EED5F-FE9A-412F-AFF1-4ED27E34FC47}</x14:id>
+          <x14:id>{90A41CA0-0F7D-46AD-BC24-540761A9D4CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0C054CD4-E2CF-4477-B402-F8B25FE004F1}</x14:id>
+          <x14:id>{F1DCBAFA-1695-4BCF-B032-9BEE42C4A58B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C532B192-3C36-461E-BE07-9730D97CE494}</x14:id>
+          <x14:id>{FFD9700B-CF5C-4B8F-9DE1-307EE78AFCA0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B11E7DAE-36C3-4EEA-9BA4-92BDC244D882}</x14:id>
+          <x14:id>{6459D2F2-F4E3-4151-A45F-5D64BF0F6C19}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{105EED5F-FE9A-412F-AFF1-4ED27E34FC47}">
+          <x14:cfRule type="dataBar" id="{90A41CA0-0F7D-46AD-BC24-540761A9D4CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0C054CD4-E2CF-4477-B402-F8B25FE004F1}">
+          <x14:cfRule type="dataBar" id="{F1DCBAFA-1695-4BCF-B032-9BEE42C4A58B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C532B192-3C36-461E-BE07-9730D97CE494}">
+          <x14:cfRule type="dataBar" id="{FFD9700B-CF5C-4B8F-9DE1-307EE78AFCA0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B11E7DAE-36C3-4EEA-9BA4-92BDC244D882}">
+          <x14:cfRule type="dataBar" id="{6459D2F2-F4E3-4151-A45F-5D64BF0F6C19}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{93426B34-7830-4C8E-9731-8B43C273D926}</x14:id>
+          <x14:id>{4D9D6E1A-166D-476E-9DDF-0FDC7F1317D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C0A1F01-7B6B-44BA-86C1-C0F3C41F99A0}</x14:id>
+          <x14:id>{1BB12D41-0BC5-4DBA-99A1-FE6B3590C0DA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{961B1072-FD6B-462B-88F8-8C8012FE303D}</x14:id>
+          <x14:id>{966C8518-4B35-4581-9BC4-C6B41C6A1B96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7C79B556-5707-423E-8062-13616BD63709}</x14:id>
+          <x14:id>{B706BF9E-BC31-491F-9124-13DB93BE0031}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{93426B34-7830-4C8E-9731-8B43C273D926}">
+          <x14:cfRule type="dataBar" id="{4D9D6E1A-166D-476E-9DDF-0FDC7F1317D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C0A1F01-7B6B-44BA-86C1-C0F3C41F99A0}">
+          <x14:cfRule type="dataBar" id="{1BB12D41-0BC5-4DBA-99A1-FE6B3590C0DA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{961B1072-FD6B-462B-88F8-8C8012FE303D}">
+          <x14:cfRule type="dataBar" id="{966C8518-4B35-4581-9BC4-C6B41C6A1B96}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7C79B556-5707-423E-8062-13616BD63709}">
+          <x14:cfRule type="dataBar" id="{B706BF9E-BC31-491F-9124-13DB93BE0031}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90A41CA0-0F7D-46AD-BC24-540761A9D4CF}</x14:id>
+          <x14:id>{132AC9C2-D17D-464F-BC01-C3CA92E33A64}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F1DCBAFA-1695-4BCF-B032-9BEE42C4A58B}</x14:id>
+          <x14:id>{9FB19609-0FA8-439D-B5D0-CE0BFCF1600A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FFD9700B-CF5C-4B8F-9DE1-307EE78AFCA0}</x14:id>
+          <x14:id>{8BC65635-2628-4B76-8E46-438FFFF240E4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6459D2F2-F4E3-4151-A45F-5D64BF0F6C19}</x14:id>
+          <x14:id>{92360E1D-6593-4CE2-8B46-6AF26581A09A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90A41CA0-0F7D-46AD-BC24-540761A9D4CF}">
+          <x14:cfRule type="dataBar" id="{132AC9C2-D17D-464F-BC01-C3CA92E33A64}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F1DCBAFA-1695-4BCF-B032-9BEE42C4A58B}">
+          <x14:cfRule type="dataBar" id="{9FB19609-0FA8-439D-B5D0-CE0BFCF1600A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FFD9700B-CF5C-4B8F-9DE1-307EE78AFCA0}">
+          <x14:cfRule type="dataBar" id="{8BC65635-2628-4B76-8E46-438FFFF240E4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6459D2F2-F4E3-4151-A45F-5D64BF0F6C19}">
+          <x14:cfRule type="dataBar" id="{92360E1D-6593-4CE2-8B46-6AF26581A09A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4D9D6E1A-166D-476E-9DDF-0FDC7F1317D5}</x14:id>
+          <x14:id>{8BB9D621-85BF-4439-ABAF-37E5B5714440}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1BB12D41-0BC5-4DBA-99A1-FE6B3590C0DA}</x14:id>
+          <x14:id>{B9C5E506-C539-4659-930B-0AA1A957C6AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{966C8518-4B35-4581-9BC4-C6B41C6A1B96}</x14:id>
+          <x14:id>{6D6BCDA9-E71A-4669-91C6-2CCA704F3350}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B706BF9E-BC31-491F-9124-13DB93BE0031}</x14:id>
+          <x14:id>{D7291800-91A0-4B50-89BA-39E63253F744}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4D9D6E1A-166D-476E-9DDF-0FDC7F1317D5}">
+          <x14:cfRule type="dataBar" id="{8BB9D621-85BF-4439-ABAF-37E5B5714440}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1BB12D41-0BC5-4DBA-99A1-FE6B3590C0DA}">
+          <x14:cfRule type="dataBar" id="{B9C5E506-C539-4659-930B-0AA1A957C6AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{966C8518-4B35-4581-9BC4-C6B41C6A1B96}">
+          <x14:cfRule type="dataBar" id="{6D6BCDA9-E71A-4669-91C6-2CCA704F3350}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B706BF9E-BC31-491F-9124-13DB93BE0031}">
+          <x14:cfRule type="dataBar" id="{D7291800-91A0-4B50-89BA-39E63253F744}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{132AC9C2-D17D-464F-BC01-C3CA92E33A64}</x14:id>
+          <x14:id>{1C63C983-10E8-46CE-98F5-7CB3488E4923}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FB19609-0FA8-439D-B5D0-CE0BFCF1600A}</x14:id>
+          <x14:id>{2697F0C5-BEDD-4002-94A6-2B38E1BBB209}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8BC65635-2628-4B76-8E46-438FFFF240E4}</x14:id>
+          <x14:id>{5F60EF8E-3EAC-4F5E-88C4-B07D72317083}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{92360E1D-6593-4CE2-8B46-6AF26581A09A}</x14:id>
+          <x14:id>{4C556552-5717-4E55-8D1A-F395663B19AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{132AC9C2-D17D-464F-BC01-C3CA92E33A64}">
+          <x14:cfRule type="dataBar" id="{1C63C983-10E8-46CE-98F5-7CB3488E4923}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FB19609-0FA8-439D-B5D0-CE0BFCF1600A}">
+          <x14:cfRule type="dataBar" id="{2697F0C5-BEDD-4002-94A6-2B38E1BBB209}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8BC65635-2628-4B76-8E46-438FFFF240E4}">
+          <x14:cfRule type="dataBar" id="{5F60EF8E-3EAC-4F5E-88C4-B07D72317083}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{92360E1D-6593-4CE2-8B46-6AF26581A09A}">
+          <x14:cfRule type="dataBar" id="{4C556552-5717-4E55-8D1A-F395663B19AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8BB9D621-85BF-4439-ABAF-37E5B5714440}</x14:id>
+          <x14:id>{24AACDF4-2C1C-4BB6-94FF-6699C1546B68}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B9C5E506-C539-4659-930B-0AA1A957C6AF}</x14:id>
+          <x14:id>{0B4B6594-E8B9-4F48-B4D5-18699912759B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D6BCDA9-E71A-4669-91C6-2CCA704F3350}</x14:id>
+          <x14:id>{A6B8E138-9B0C-4FA1-85B0-BBA920F25945}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D7291800-91A0-4B50-89BA-39E63253F744}</x14:id>
+          <x14:id>{D54F815E-4E2F-4784-86CC-D4402CE39E08}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8BB9D621-85BF-4439-ABAF-37E5B5714440}">
+          <x14:cfRule type="dataBar" id="{24AACDF4-2C1C-4BB6-94FF-6699C1546B68}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B9C5E506-C539-4659-930B-0AA1A957C6AF}">
+          <x14:cfRule type="dataBar" id="{0B4B6594-E8B9-4F48-B4D5-18699912759B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D6BCDA9-E71A-4669-91C6-2CCA704F3350}">
+          <x14:cfRule type="dataBar" id="{A6B8E138-9B0C-4FA1-85B0-BBA920F25945}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D7291800-91A0-4B50-89BA-39E63253F744}">
+          <x14:cfRule type="dataBar" id="{D54F815E-4E2F-4784-86CC-D4402CE39E08}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1C63C983-10E8-46CE-98F5-7CB3488E4923}</x14:id>
+          <x14:id>{B17F7E8D-AE77-4D1E-8A46-505566A66D33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2697F0C5-BEDD-4002-94A6-2B38E1BBB209}</x14:id>
+          <x14:id>{537F03EA-640C-448B-B28A-DBA56F75A11A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5F60EF8E-3EAC-4F5E-88C4-B07D72317083}</x14:id>
+          <x14:id>{D11EB82B-9BEA-4BD1-AC73-B667A955A21C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C556552-5717-4E55-8D1A-F395663B19AF}</x14:id>
+          <x14:id>{BE5644E0-F5B7-41DE-899B-0B7698A6B7FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1C63C983-10E8-46CE-98F5-7CB3488E4923}">
+          <x14:cfRule type="dataBar" id="{B17F7E8D-AE77-4D1E-8A46-505566A66D33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2697F0C5-BEDD-4002-94A6-2B38E1BBB209}">
+          <x14:cfRule type="dataBar" id="{537F03EA-640C-448B-B28A-DBA56F75A11A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5F60EF8E-3EAC-4F5E-88C4-B07D72317083}">
+          <x14:cfRule type="dataBar" id="{D11EB82B-9BEA-4BD1-AC73-B667A955A21C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C556552-5717-4E55-8D1A-F395663B19AF}">
+          <x14:cfRule type="dataBar" id="{BE5644E0-F5B7-41DE-899B-0B7698A6B7FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24AACDF4-2C1C-4BB6-94FF-6699C1546B68}</x14:id>
+          <x14:id>{26309998-4C3B-45C8-A357-7200CB74C148}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B4B6594-E8B9-4F48-B4D5-18699912759B}</x14:id>
+          <x14:id>{97EDD3CF-8F8E-4807-B9CF-661488D409AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A6B8E138-9B0C-4FA1-85B0-BBA920F25945}</x14:id>
+          <x14:id>{290C3425-D26B-44E6-89CE-1FD6B1AAE2BE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D54F815E-4E2F-4784-86CC-D4402CE39E08}</x14:id>
+          <x14:id>{FDE29A02-DAA7-4D86-B820-7FF01E1F96C4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24AACDF4-2C1C-4BB6-94FF-6699C1546B68}">
+          <x14:cfRule type="dataBar" id="{26309998-4C3B-45C8-A357-7200CB74C148}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B4B6594-E8B9-4F48-B4D5-18699912759B}">
+          <x14:cfRule type="dataBar" id="{97EDD3CF-8F8E-4807-B9CF-661488D409AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A6B8E138-9B0C-4FA1-85B0-BBA920F25945}">
+          <x14:cfRule type="dataBar" id="{290C3425-D26B-44E6-89CE-1FD6B1AAE2BE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D54F815E-4E2F-4784-86CC-D4402CE39E08}">
+          <x14:cfRule type="dataBar" id="{FDE29A02-DAA7-4D86-B820-7FF01E1F96C4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B17F7E8D-AE77-4D1E-8A46-505566A66D33}</x14:id>
+          <x14:id>{49A5061B-7563-4CB6-990E-4F52C167E2BD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{537F03EA-640C-448B-B28A-DBA56F75A11A}</x14:id>
+          <x14:id>{7F3A90EE-8DC1-425E-ABED-41C65E86F4F7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D11EB82B-9BEA-4BD1-AC73-B667A955A21C}</x14:id>
+          <x14:id>{EEDB19C7-9F73-436F-BBD1-4057E2D01C97}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BE5644E0-F5B7-41DE-899B-0B7698A6B7FD}</x14:id>
+          <x14:id>{B106CD61-37D1-4881-972B-6F8D23E17905}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B17F7E8D-AE77-4D1E-8A46-505566A66D33}">
+          <x14:cfRule type="dataBar" id="{49A5061B-7563-4CB6-990E-4F52C167E2BD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{537F03EA-640C-448B-B28A-DBA56F75A11A}">
+          <x14:cfRule type="dataBar" id="{7F3A90EE-8DC1-425E-ABED-41C65E86F4F7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D11EB82B-9BEA-4BD1-AC73-B667A955A21C}">
+          <x14:cfRule type="dataBar" id="{EEDB19C7-9F73-436F-BBD1-4057E2D01C97}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BE5644E0-F5B7-41DE-899B-0B7698A6B7FD}">
+          <x14:cfRule type="dataBar" id="{B106CD61-37D1-4881-972B-6F8D23E17905}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26309998-4C3B-45C8-A357-7200CB74C148}</x14:id>
+          <x14:id>{0EE3C7DD-78AF-44B4-9FAB-28C88C60A504}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{97EDD3CF-8F8E-4807-B9CF-661488D409AB}</x14:id>
+          <x14:id>{0812355D-738F-4EDA-9468-04FA2A232DEF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{290C3425-D26B-44E6-89CE-1FD6B1AAE2BE}</x14:id>
+          <x14:id>{6F0AE0E9-5362-4D27-875D-19CE22CA569C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FDE29A02-DAA7-4D86-B820-7FF01E1F96C4}</x14:id>
+          <x14:id>{6C8C3E47-9BC9-400B-B6C6-DE21FB4CB51A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26309998-4C3B-45C8-A357-7200CB74C148}">
+          <x14:cfRule type="dataBar" id="{0EE3C7DD-78AF-44B4-9FAB-28C88C60A504}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{97EDD3CF-8F8E-4807-B9CF-661488D409AB}">
+          <x14:cfRule type="dataBar" id="{0812355D-738F-4EDA-9468-04FA2A232DEF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{290C3425-D26B-44E6-89CE-1FD6B1AAE2BE}">
+          <x14:cfRule type="dataBar" id="{6F0AE0E9-5362-4D27-875D-19CE22CA569C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FDE29A02-DAA7-4D86-B820-7FF01E1F96C4}">
+          <x14:cfRule type="dataBar" id="{6C8C3E47-9BC9-400B-B6C6-DE21FB4CB51A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49A5061B-7563-4CB6-990E-4F52C167E2BD}</x14:id>
+          <x14:id>{11ACF266-3333-4B42-ADCF-63E70894ABB9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F3A90EE-8DC1-425E-ABED-41C65E86F4F7}</x14:id>
+          <x14:id>{54E0667F-F775-4622-A568-2A3BFF3D000E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEDB19C7-9F73-436F-BBD1-4057E2D01C97}</x14:id>
+          <x14:id>{E1B783F5-09E1-4061-BB1F-B59A6B205C3B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B106CD61-37D1-4881-972B-6F8D23E17905}</x14:id>
+          <x14:id>{70C094E9-41E8-4506-86F2-E9C3DBDF5748}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49A5061B-7563-4CB6-990E-4F52C167E2BD}">
+          <x14:cfRule type="dataBar" id="{11ACF266-3333-4B42-ADCF-63E70894ABB9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F3A90EE-8DC1-425E-ABED-41C65E86F4F7}">
+          <x14:cfRule type="dataBar" id="{54E0667F-F775-4622-A568-2A3BFF3D000E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEDB19C7-9F73-436F-BBD1-4057E2D01C97}">
+          <x14:cfRule type="dataBar" id="{E1B783F5-09E1-4061-BB1F-B59A6B205C3B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B106CD61-37D1-4881-972B-6F8D23E17905}">
+          <x14:cfRule type="dataBar" id="{70C094E9-41E8-4506-86F2-E9C3DBDF5748}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0EE3C7DD-78AF-44B4-9FAB-28C88C60A504}</x14:id>
+          <x14:id>{2915D5C8-996C-4C73-98EB-51739A0EE6EF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0812355D-738F-4EDA-9468-04FA2A232DEF}</x14:id>
+          <x14:id>{FF3EC900-5170-48A1-B656-6341334278D7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F0AE0E9-5362-4D27-875D-19CE22CA569C}</x14:id>
+          <x14:id>{E9607B4A-20B5-4960-BDAE-46F0F3CF0656}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6C8C3E47-9BC9-400B-B6C6-DE21FB4CB51A}</x14:id>
+          <x14:id>{6D00B664-3F21-4AEC-B890-8D34541CF50D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0EE3C7DD-78AF-44B4-9FAB-28C88C60A504}">
+          <x14:cfRule type="dataBar" id="{2915D5C8-996C-4C73-98EB-51739A0EE6EF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0812355D-738F-4EDA-9468-04FA2A232DEF}">
+          <x14:cfRule type="dataBar" id="{FF3EC900-5170-48A1-B656-6341334278D7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F0AE0E9-5362-4D27-875D-19CE22CA569C}">
+          <x14:cfRule type="dataBar" id="{E9607B4A-20B5-4960-BDAE-46F0F3CF0656}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6C8C3E47-9BC9-400B-B6C6-DE21FB4CB51A}">
+          <x14:cfRule type="dataBar" id="{6D00B664-3F21-4AEC-B890-8D34541CF50D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11ACF266-3333-4B42-ADCF-63E70894ABB9}</x14:id>
+          <x14:id>{D90430D0-0002-4C1B-AD98-122EC9715D70}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{54E0667F-F775-4622-A568-2A3BFF3D000E}</x14:id>
+          <x14:id>{C1151B36-D617-4791-9308-377B4798D41F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E1B783F5-09E1-4061-BB1F-B59A6B205C3B}</x14:id>
+          <x14:id>{2BF557D3-125B-44EC-A23D-C8468A966AF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{70C094E9-41E8-4506-86F2-E9C3DBDF5748}</x14:id>
+          <x14:id>{65C904A8-61E8-494D-ADE0-B4381B027EBE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11ACF266-3333-4B42-ADCF-63E70894ABB9}">
+          <x14:cfRule type="dataBar" id="{D90430D0-0002-4C1B-AD98-122EC9715D70}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{54E0667F-F775-4622-A568-2A3BFF3D000E}">
+          <x14:cfRule type="dataBar" id="{C1151B36-D617-4791-9308-377B4798D41F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E1B783F5-09E1-4061-BB1F-B59A6B205C3B}">
+          <x14:cfRule type="dataBar" id="{2BF557D3-125B-44EC-A23D-C8468A966AF6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{70C094E9-41E8-4506-86F2-E9C3DBDF5748}">
+          <x14:cfRule type="dataBar" id="{65C904A8-61E8-494D-ADE0-B4381B027EBE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2915D5C8-996C-4C73-98EB-51739A0EE6EF}</x14:id>
+          <x14:id>{E83F3FCC-6CC9-4DF5-B354-C7B39FE6CF9E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF3EC900-5170-48A1-B656-6341334278D7}</x14:id>
+          <x14:id>{AA37F83E-1FB7-4D31-AAA6-247EE92EC382}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E9607B4A-20B5-4960-BDAE-46F0F3CF0656}</x14:id>
+          <x14:id>{37F92445-96A8-4AA9-B14B-2BCD38D91DC6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D00B664-3F21-4AEC-B890-8D34541CF50D}</x14:id>
+          <x14:id>{3F33F60A-C693-4F4B-982D-993BB21EFA22}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2915D5C8-996C-4C73-98EB-51739A0EE6EF}">
+          <x14:cfRule type="dataBar" id="{E83F3FCC-6CC9-4DF5-B354-C7B39FE6CF9E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF3EC900-5170-48A1-B656-6341334278D7}">
+          <x14:cfRule type="dataBar" id="{AA37F83E-1FB7-4D31-AAA6-247EE92EC382}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E9607B4A-20B5-4960-BDAE-46F0F3CF0656}">
+          <x14:cfRule type="dataBar" id="{37F92445-96A8-4AA9-B14B-2BCD38D91DC6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D00B664-3F21-4AEC-B890-8D34541CF50D}">
+          <x14:cfRule type="dataBar" id="{3F33F60A-C693-4F4B-982D-993BB21EFA22}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D90430D0-0002-4C1B-AD98-122EC9715D70}</x14:id>
+          <x14:id>{03119A41-BE61-4415-BD11-6618FD171E45}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C1151B36-D617-4791-9308-377B4798D41F}</x14:id>
+          <x14:id>{0E0EE0ED-BB64-4340-BE46-4B19E1644ABE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2BF557D3-125B-44EC-A23D-C8468A966AF6}</x14:id>
+          <x14:id>{D4152B1F-1C28-414E-8354-82CACC445B47}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{65C904A8-61E8-494D-ADE0-B4381B027EBE}</x14:id>
+          <x14:id>{24459895-0192-44AC-85A1-F346262A4CA9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D90430D0-0002-4C1B-AD98-122EC9715D70}">
+          <x14:cfRule type="dataBar" id="{03119A41-BE61-4415-BD11-6618FD171E45}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C1151B36-D617-4791-9308-377B4798D41F}">
+          <x14:cfRule type="dataBar" id="{0E0EE0ED-BB64-4340-BE46-4B19E1644ABE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2BF557D3-125B-44EC-A23D-C8468A966AF6}">
+          <x14:cfRule type="dataBar" id="{D4152B1F-1C28-414E-8354-82CACC445B47}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{65C904A8-61E8-494D-ADE0-B4381B027EBE}">
+          <x14:cfRule type="dataBar" id="{24459895-0192-44AC-85A1-F346262A4CA9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E83F3FCC-6CC9-4DF5-B354-C7B39FE6CF9E}</x14:id>
+          <x14:id>{655EDE83-0EF2-46F2-8EE4-912A4CCD13B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA37F83E-1FB7-4D31-AAA6-247EE92EC382}</x14:id>
+          <x14:id>{10C1F5AB-7101-4331-86CF-92EDF912D799}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{37F92445-96A8-4AA9-B14B-2BCD38D91DC6}</x14:id>
+          <x14:id>{B1EA713F-9CD9-4BCB-9057-3BA4AEA08ADA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3F33F60A-C693-4F4B-982D-993BB21EFA22}</x14:id>
+          <x14:id>{C65A3CEF-84D0-454A-AE33-9AC9824D3BB8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E83F3FCC-6CC9-4DF5-B354-C7B39FE6CF9E}">
+          <x14:cfRule type="dataBar" id="{655EDE83-0EF2-46F2-8EE4-912A4CCD13B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA37F83E-1FB7-4D31-AAA6-247EE92EC382}">
+          <x14:cfRule type="dataBar" id="{10C1F5AB-7101-4331-86CF-92EDF912D799}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{37F92445-96A8-4AA9-B14B-2BCD38D91DC6}">
+          <x14:cfRule type="dataBar" id="{B1EA713F-9CD9-4BCB-9057-3BA4AEA08ADA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3F33F60A-C693-4F4B-982D-993BB21EFA22}">
+          <x14:cfRule type="dataBar" id="{C65A3CEF-84D0-454A-AE33-9AC9824D3BB8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{03119A41-BE61-4415-BD11-6618FD171E45}</x14:id>
+          <x14:id>{CC097C5B-231B-4A91-8BC4-890091EB436A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0E0EE0ED-BB64-4340-BE46-4B19E1644ABE}</x14:id>
+          <x14:id>{EC7DD340-7E7E-4670-83A2-CA2582B60B50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D4152B1F-1C28-414E-8354-82CACC445B47}</x14:id>
+          <x14:id>{F838C1D8-62A5-45F5-B29F-645740FE4C01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24459895-0192-44AC-85A1-F346262A4CA9}</x14:id>
+          <x14:id>{E51510E0-75CF-43BF-9696-BDE9B7FB88F9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{03119A41-BE61-4415-BD11-6618FD171E45}">
+          <x14:cfRule type="dataBar" id="{CC097C5B-231B-4A91-8BC4-890091EB436A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0E0EE0ED-BB64-4340-BE46-4B19E1644ABE}">
+          <x14:cfRule type="dataBar" id="{EC7DD340-7E7E-4670-83A2-CA2582B60B50}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D4152B1F-1C28-414E-8354-82CACC445B47}">
+          <x14:cfRule type="dataBar" id="{F838C1D8-62A5-45F5-B29F-645740FE4C01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24459895-0192-44AC-85A1-F346262A4CA9}">
+          <x14:cfRule type="dataBar" id="{E51510E0-75CF-43BF-9696-BDE9B7FB88F9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{655EDE83-0EF2-46F2-8EE4-912A4CCD13B4}</x14:id>
+          <x14:id>{FF00E227-65C5-4C49-BD5E-A6D8DE2BFF91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{10C1F5AB-7101-4331-86CF-92EDF912D799}</x14:id>
+          <x14:id>{72869A00-FA2B-4B4D-9E76-B15C2F95E1CD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B1EA713F-9CD9-4BCB-9057-3BA4AEA08ADA}</x14:id>
+          <x14:id>{089DA838-6A24-46B3-99D7-CE8BFDAC86BD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C65A3CEF-84D0-454A-AE33-9AC9824D3BB8}</x14:id>
+          <x14:id>{A3D4FBB7-382D-4DB8-8E1F-FA88A30E869D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{655EDE83-0EF2-46F2-8EE4-912A4CCD13B4}">
+          <x14:cfRule type="dataBar" id="{FF00E227-65C5-4C49-BD5E-A6D8DE2BFF91}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{10C1F5AB-7101-4331-86CF-92EDF912D799}">
+          <x14:cfRule type="dataBar" id="{72869A00-FA2B-4B4D-9E76-B15C2F95E1CD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B1EA713F-9CD9-4BCB-9057-3BA4AEA08ADA}">
+          <x14:cfRule type="dataBar" id="{089DA838-6A24-46B3-99D7-CE8BFDAC86BD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C65A3CEF-84D0-454A-AE33-9AC9824D3BB8}">
+          <x14:cfRule type="dataBar" id="{A3D4FBB7-382D-4DB8-8E1F-FA88A30E869D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CC097C5B-231B-4A91-8BC4-890091EB436A}</x14:id>
+          <x14:id>{95060B5C-3719-4892-A337-F04DF355C963}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC7DD340-7E7E-4670-83A2-CA2582B60B50}</x14:id>
+          <x14:id>{4A9DDA9D-95ED-4AF1-A818-86A9DD76E4BD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F838C1D8-62A5-45F5-B29F-645740FE4C01}</x14:id>
+          <x14:id>{E56812EC-0F5A-488D-A752-AC3915851238}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E51510E0-75CF-43BF-9696-BDE9B7FB88F9}</x14:id>
+          <x14:id>{7FC2EECC-438C-4926-9591-CFC435584CF4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CC097C5B-231B-4A91-8BC4-890091EB436A}">
+          <x14:cfRule type="dataBar" id="{95060B5C-3719-4892-A337-F04DF355C963}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC7DD340-7E7E-4670-83A2-CA2582B60B50}">
+          <x14:cfRule type="dataBar" id="{4A9DDA9D-95ED-4AF1-A818-86A9DD76E4BD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F838C1D8-62A5-45F5-B29F-645740FE4C01}">
+          <x14:cfRule type="dataBar" id="{E56812EC-0F5A-488D-A752-AC3915851238}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E51510E0-75CF-43BF-9696-BDE9B7FB88F9}">
+          <x14:cfRule type="dataBar" id="{7FC2EECC-438C-4926-9591-CFC435584CF4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF00E227-65C5-4C49-BD5E-A6D8DE2BFF91}</x14:id>
+          <x14:id>{CCBC9624-46FF-460A-88BA-CD75032653AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{72869A00-FA2B-4B4D-9E76-B15C2F95E1CD}</x14:id>
+          <x14:id>{3D4B0444-7E9C-4C8F-9A9F-9B5A6BEBBA77}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{089DA838-6A24-46B3-99D7-CE8BFDAC86BD}</x14:id>
+          <x14:id>{3CCFF1C2-CB32-46DD-B618-0A46554A61C5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A3D4FBB7-382D-4DB8-8E1F-FA88A30E869D}</x14:id>
+          <x14:id>{6EF8E894-F7A8-427F-B51F-09DDB9542BB3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF00E227-65C5-4C49-BD5E-A6D8DE2BFF91}">
+          <x14:cfRule type="dataBar" id="{CCBC9624-46FF-460A-88BA-CD75032653AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{72869A00-FA2B-4B4D-9E76-B15C2F95E1CD}">
+          <x14:cfRule type="dataBar" id="{3D4B0444-7E9C-4C8F-9A9F-9B5A6BEBBA77}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{089DA838-6A24-46B3-99D7-CE8BFDAC86BD}">
+          <x14:cfRule type="dataBar" id="{3CCFF1C2-CB32-46DD-B618-0A46554A61C5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A3D4FBB7-382D-4DB8-8E1F-FA88A30E869D}">
+          <x14:cfRule type="dataBar" id="{6EF8E894-F7A8-427F-B51F-09DDB9542BB3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95060B5C-3719-4892-A337-F04DF355C963}</x14:id>
+          <x14:id>{41FA7C9A-3DF4-44D8-B619-B5D4E9DB1540}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4A9DDA9D-95ED-4AF1-A818-86A9DD76E4BD}</x14:id>
+          <x14:id>{53698431-C6A8-407B-8C8A-415C9C1926DE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E56812EC-0F5A-488D-A752-AC3915851238}</x14:id>
+          <x14:id>{CD06CE85-E3E4-4E14-8C03-66757E1AACD5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7FC2EECC-438C-4926-9591-CFC435584CF4}</x14:id>
+          <x14:id>{C2D4ABEC-BED4-4A85-9B4A-B15F1776736D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95060B5C-3719-4892-A337-F04DF355C963}">
+          <x14:cfRule type="dataBar" id="{41FA7C9A-3DF4-44D8-B619-B5D4E9DB1540}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4A9DDA9D-95ED-4AF1-A818-86A9DD76E4BD}">
+          <x14:cfRule type="dataBar" id="{53698431-C6A8-407B-8C8A-415C9C1926DE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E56812EC-0F5A-488D-A752-AC3915851238}">
+          <x14:cfRule type="dataBar" id="{CD06CE85-E3E4-4E14-8C03-66757E1AACD5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7FC2EECC-438C-4926-9591-CFC435584CF4}">
+          <x14:cfRule type="dataBar" id="{C2D4ABEC-BED4-4A85-9B4A-B15F1776736D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CCBC9624-46FF-460A-88BA-CD75032653AB}</x14:id>
+          <x14:id>{47599B86-47C8-4EA6-B087-5AA66010958D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D4B0444-7E9C-4C8F-9A9F-9B5A6BEBBA77}</x14:id>
+          <x14:id>{708D6523-1862-4983-893C-62F33480BCBF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CCFF1C2-CB32-46DD-B618-0A46554A61C5}</x14:id>
+          <x14:id>{C4634E90-7F11-4EDA-8BE8-521C24C559A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6EF8E894-F7A8-427F-B51F-09DDB9542BB3}</x14:id>
+          <x14:id>{AF3C4B5D-091D-4585-8A0C-CF853F95E6C7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CCBC9624-46FF-460A-88BA-CD75032653AB}">
+          <x14:cfRule type="dataBar" id="{47599B86-47C8-4EA6-B087-5AA66010958D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D4B0444-7E9C-4C8F-9A9F-9B5A6BEBBA77}">
+          <x14:cfRule type="dataBar" id="{708D6523-1862-4983-893C-62F33480BCBF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CCFF1C2-CB32-46DD-B618-0A46554A61C5}">
+          <x14:cfRule type="dataBar" id="{C4634E90-7F11-4EDA-8BE8-521C24C559A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6EF8E894-F7A8-427F-B51F-09DDB9542BB3}">
+          <x14:cfRule type="dataBar" id="{AF3C4B5D-091D-4585-8A0C-CF853F95E6C7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{41FA7C9A-3DF4-44D8-B619-B5D4E9DB1540}</x14:id>
+          <x14:id>{0ABF8377-B77F-42FC-A42A-E17B0D52BE65}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53698431-C6A8-407B-8C8A-415C9C1926DE}</x14:id>
+          <x14:id>{49B6A445-FE64-4D25-A3D5-41391F2BABCE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD06CE85-E3E4-4E14-8C03-66757E1AACD5}</x14:id>
+          <x14:id>{9A881416-B9AC-4E17-ABB0-654579CEF1D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C2D4ABEC-BED4-4A85-9B4A-B15F1776736D}</x14:id>
+          <x14:id>{44C98A21-0CA5-4BE7-B46D-2377B3E07EB1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{41FA7C9A-3DF4-44D8-B619-B5D4E9DB1540}">
+          <x14:cfRule type="dataBar" id="{0ABF8377-B77F-42FC-A42A-E17B0D52BE65}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53698431-C6A8-407B-8C8A-415C9C1926DE}">
+          <x14:cfRule type="dataBar" id="{49B6A445-FE64-4D25-A3D5-41391F2BABCE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD06CE85-E3E4-4E14-8C03-66757E1AACD5}">
+          <x14:cfRule type="dataBar" id="{9A881416-B9AC-4E17-ABB0-654579CEF1D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C2D4ABEC-BED4-4A85-9B4A-B15F1776736D}">
+          <x14:cfRule type="dataBar" id="{44C98A21-0CA5-4BE7-B46D-2377B3E07EB1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{47599B86-47C8-4EA6-B087-5AA66010958D}</x14:id>
+          <x14:id>{64AB7C17-EFBA-481B-A48D-C9689E42ED8E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{708D6523-1862-4983-893C-62F33480BCBF}</x14:id>
+          <x14:id>{4C357E7E-B9A0-4EC4-B5FB-AEB78563F6C9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C4634E90-7F11-4EDA-8BE8-521C24C559A2}</x14:id>
+          <x14:id>{D3B9BCC0-FA3D-4E2E-8875-297C772AD638}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF3C4B5D-091D-4585-8A0C-CF853F95E6C7}</x14:id>
+          <x14:id>{52F2D6CB-B618-4093-8BDC-DF498A974C99}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{47599B86-47C8-4EA6-B087-5AA66010958D}">
+          <x14:cfRule type="dataBar" id="{64AB7C17-EFBA-481B-A48D-C9689E42ED8E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{708D6523-1862-4983-893C-62F33480BCBF}">
+          <x14:cfRule type="dataBar" id="{4C357E7E-B9A0-4EC4-B5FB-AEB78563F6C9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C4634E90-7F11-4EDA-8BE8-521C24C559A2}">
+          <x14:cfRule type="dataBar" id="{D3B9BCC0-FA3D-4E2E-8875-297C772AD638}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF3C4B5D-091D-4585-8A0C-CF853F95E6C7}">
+          <x14:cfRule type="dataBar" id="{52F2D6CB-B618-4093-8BDC-DF498A974C99}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0ABF8377-B77F-42FC-A42A-E17B0D52BE65}</x14:id>
+          <x14:id>{B3929DFE-757C-4FD1-82F1-F993448B4FDC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49B6A445-FE64-4D25-A3D5-41391F2BABCE}</x14:id>
+          <x14:id>{02CE07C1-8C32-4E9C-8D8A-493D35C9F36E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9A881416-B9AC-4E17-ABB0-654579CEF1D5}</x14:id>
+          <x14:id>{133D09B5-F6E9-42FB-964F-D91946AF9454}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{44C98A21-0CA5-4BE7-B46D-2377B3E07EB1}</x14:id>
+          <x14:id>{F7F8F2FA-1B5D-4E8E-A4DF-DA9F7DE24144}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0ABF8377-B77F-42FC-A42A-E17B0D52BE65}">
+          <x14:cfRule type="dataBar" id="{B3929DFE-757C-4FD1-82F1-F993448B4FDC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49B6A445-FE64-4D25-A3D5-41391F2BABCE}">
+          <x14:cfRule type="dataBar" id="{02CE07C1-8C32-4E9C-8D8A-493D35C9F36E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9A881416-B9AC-4E17-ABB0-654579CEF1D5}">
+          <x14:cfRule type="dataBar" id="{133D09B5-F6E9-42FB-964F-D91946AF9454}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{44C98A21-0CA5-4BE7-B46D-2377B3E07EB1}">
+          <x14:cfRule type="dataBar" id="{F7F8F2FA-1B5D-4E8E-A4DF-DA9F7DE24144}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{64AB7C17-EFBA-481B-A48D-C9689E42ED8E}</x14:id>
+          <x14:id>{1107000B-C968-455A-A0D8-619325DC3B44}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C357E7E-B9A0-4EC4-B5FB-AEB78563F6C9}</x14:id>
+          <x14:id>{F8E856B8-CE5C-40F4-BA86-674AE8AB78E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D3B9BCC0-FA3D-4E2E-8875-297C772AD638}</x14:id>
+          <x14:id>{3919CBE4-F55D-42EA-8645-28F7141364CE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{52F2D6CB-B618-4093-8BDC-DF498A974C99}</x14:id>
+          <x14:id>{D9204F61-3A42-41BA-B2AC-E942DB01579E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{64AB7C17-EFBA-481B-A48D-C9689E42ED8E}">
+          <x14:cfRule type="dataBar" id="{1107000B-C968-455A-A0D8-619325DC3B44}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C357E7E-B9A0-4EC4-B5FB-AEB78563F6C9}">
+          <x14:cfRule type="dataBar" id="{F8E856B8-CE5C-40F4-BA86-674AE8AB78E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D3B9BCC0-FA3D-4E2E-8875-297C772AD638}">
+          <x14:cfRule type="dataBar" id="{3919CBE4-F55D-42EA-8645-28F7141364CE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{52F2D6CB-B618-4093-8BDC-DF498A974C99}">
+          <x14:cfRule type="dataBar" id="{D9204F61-3A42-41BA-B2AC-E942DB01579E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B3929DFE-757C-4FD1-82F1-F993448B4FDC}</x14:id>
+          <x14:id>{AB594940-C91E-47C2-819B-014B7EAC71C8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{02CE07C1-8C32-4E9C-8D8A-493D35C9F36E}</x14:id>
+          <x14:id>{F0293117-8024-415A-B177-9480C7ACBE8E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{133D09B5-F6E9-42FB-964F-D91946AF9454}</x14:id>
+          <x14:id>{D2F042E1-A308-49EB-9E46-FA3042CCE22D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F7F8F2FA-1B5D-4E8E-A4DF-DA9F7DE24144}</x14:id>
+          <x14:id>{60A5B706-F318-4EB9-8979-380C1B91637C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B3929DFE-757C-4FD1-82F1-F993448B4FDC}">
+          <x14:cfRule type="dataBar" id="{AB594940-C91E-47C2-819B-014B7EAC71C8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{02CE07C1-8C32-4E9C-8D8A-493D35C9F36E}">
+          <x14:cfRule type="dataBar" id="{F0293117-8024-415A-B177-9480C7ACBE8E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{133D09B5-F6E9-42FB-964F-D91946AF9454}">
+          <x14:cfRule type="dataBar" id="{D2F042E1-A308-49EB-9E46-FA3042CCE22D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F7F8F2FA-1B5D-4E8E-A4DF-DA9F7DE24144}">
+          <x14:cfRule type="dataBar" id="{60A5B706-F318-4EB9-8979-380C1B91637C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1107000B-C968-455A-A0D8-619325DC3B44}</x14:id>
+          <x14:id>{B3CF6207-7299-438C-88D5-E4550FD70A33}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F8E856B8-CE5C-40F4-BA86-674AE8AB78E9}</x14:id>
+          <x14:id>{6CA05A8A-2278-413B-A689-E17EAD7FD9E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3919CBE4-F55D-42EA-8645-28F7141364CE}</x14:id>
+          <x14:id>{5E2B710F-4CFC-41E6-ACA9-62AEED674656}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D9204F61-3A42-41BA-B2AC-E942DB01579E}</x14:id>
+          <x14:id>{E2D03D87-7A08-4A8F-8405-8C95DED38366}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1107000B-C968-455A-A0D8-619325DC3B44}">
+          <x14:cfRule type="dataBar" id="{B3CF6207-7299-438C-88D5-E4550FD70A33}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F8E856B8-CE5C-40F4-BA86-674AE8AB78E9}">
+          <x14:cfRule type="dataBar" id="{6CA05A8A-2278-413B-A689-E17EAD7FD9E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3919CBE4-F55D-42EA-8645-28F7141364CE}">
+          <x14:cfRule type="dataBar" id="{5E2B710F-4CFC-41E6-ACA9-62AEED674656}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D9204F61-3A42-41BA-B2AC-E942DB01579E}">
+          <x14:cfRule type="dataBar" id="{E2D03D87-7A08-4A8F-8405-8C95DED38366}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AB594940-C91E-47C2-819B-014B7EAC71C8}</x14:id>
+          <x14:id>{7A75DE5B-2A4C-486D-86FC-FB5A2F3B17FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F0293117-8024-415A-B177-9480C7ACBE8E}</x14:id>
+          <x14:id>{7B648F31-312A-4F1B-A0BD-B398E2EA38D3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D2F042E1-A308-49EB-9E46-FA3042CCE22D}</x14:id>
+          <x14:id>{19621220-AA6D-472C-B5E4-E1AE2D27AA20}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{60A5B706-F318-4EB9-8979-380C1B91637C}</x14:id>
+          <x14:id>{6B2082C4-0BD9-4286-B40E-963BE8D36B64}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AB594940-C91E-47C2-819B-014B7EAC71C8}">
+          <x14:cfRule type="dataBar" id="{7A75DE5B-2A4C-486D-86FC-FB5A2F3B17FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F0293117-8024-415A-B177-9480C7ACBE8E}">
+          <x14:cfRule type="dataBar" id="{7B648F31-312A-4F1B-A0BD-B398E2EA38D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D2F042E1-A308-49EB-9E46-FA3042CCE22D}">
+          <x14:cfRule type="dataBar" id="{19621220-AA6D-472C-B5E4-E1AE2D27AA20}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{60A5B706-F318-4EB9-8979-380C1B91637C}">
+          <x14:cfRule type="dataBar" id="{6B2082C4-0BD9-4286-B40E-963BE8D36B64}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B3CF6207-7299-438C-88D5-E4550FD70A33}</x14:id>
+          <x14:id>{C84616AB-15D5-473B-808F-390AEA70C9C5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6CA05A8A-2278-413B-A689-E17EAD7FD9E9}</x14:id>
+          <x14:id>{0D2F903F-31AA-44A7-987D-23EDD657373E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5E2B710F-4CFC-41E6-ACA9-62AEED674656}</x14:id>
+          <x14:id>{42134F4E-93C6-4793-A143-861A48631BA8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E2D03D87-7A08-4A8F-8405-8C95DED38366}</x14:id>
+          <x14:id>{E8A5DA38-E213-4CD0-99FC-10EA84E7D703}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B3CF6207-7299-438C-88D5-E4550FD70A33}">
+          <x14:cfRule type="dataBar" id="{C84616AB-15D5-473B-808F-390AEA70C9C5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6CA05A8A-2278-413B-A689-E17EAD7FD9E9}">
+          <x14:cfRule type="dataBar" id="{0D2F903F-31AA-44A7-987D-23EDD657373E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5E2B710F-4CFC-41E6-ACA9-62AEED674656}">
+          <x14:cfRule type="dataBar" id="{42134F4E-93C6-4793-A143-861A48631BA8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E2D03D87-7A08-4A8F-8405-8C95DED38366}">
+          <x14:cfRule type="dataBar" id="{E8A5DA38-E213-4CD0-99FC-10EA84E7D703}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7A75DE5B-2A4C-486D-86FC-FB5A2F3B17FA}</x14:id>
+          <x14:id>{8F834759-4960-418E-B528-A39CCD461F24}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7B648F31-312A-4F1B-A0BD-B398E2EA38D3}</x14:id>
+          <x14:id>{A7091EAC-F927-4E6B-9BCE-6FA9E85D344D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19621220-AA6D-472C-B5E4-E1AE2D27AA20}</x14:id>
+          <x14:id>{E4802929-3C3F-4BAE-9946-8EF68A14ACC7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B2082C4-0BD9-4286-B40E-963BE8D36B64}</x14:id>
+          <x14:id>{75DF331A-0C47-484B-9278-BDDCE5DAFC4E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7A75DE5B-2A4C-486D-86FC-FB5A2F3B17FA}">
+          <x14:cfRule type="dataBar" id="{8F834759-4960-418E-B528-A39CCD461F24}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7B648F31-312A-4F1B-A0BD-B398E2EA38D3}">
+          <x14:cfRule type="dataBar" id="{A7091EAC-F927-4E6B-9BCE-6FA9E85D344D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19621220-AA6D-472C-B5E4-E1AE2D27AA20}">
+          <x14:cfRule type="dataBar" id="{E4802929-3C3F-4BAE-9946-8EF68A14ACC7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B2082C4-0BD9-4286-B40E-963BE8D36B64}">
+          <x14:cfRule type="dataBar" id="{75DF331A-0C47-484B-9278-BDDCE5DAFC4E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C84616AB-15D5-473B-808F-390AEA70C9C5}</x14:id>
+          <x14:id>{E27CDDC2-6AA6-4CC6-B022-F7AF0E78366E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D2F903F-31AA-44A7-987D-23EDD657373E}</x14:id>
+          <x14:id>{29306635-A52D-4C9E-B988-DBF27BD4CEEB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42134F4E-93C6-4793-A143-861A48631BA8}</x14:id>
+          <x14:id>{F86B9855-215B-4443-B3CC-30A9538EA9FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E8A5DA38-E213-4CD0-99FC-10EA84E7D703}</x14:id>
+          <x14:id>{7F9966CC-EDC0-4EFF-89F5-273C022757CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C84616AB-15D5-473B-808F-390AEA70C9C5}">
+          <x14:cfRule type="dataBar" id="{E27CDDC2-6AA6-4CC6-B022-F7AF0E78366E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D2F903F-31AA-44A7-987D-23EDD657373E}">
+          <x14:cfRule type="dataBar" id="{29306635-A52D-4C9E-B988-DBF27BD4CEEB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42134F4E-93C6-4793-A143-861A48631BA8}">
+          <x14:cfRule type="dataBar" id="{F86B9855-215B-4443-B3CC-30A9538EA9FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E8A5DA38-E213-4CD0-99FC-10EA84E7D703}">
+          <x14:cfRule type="dataBar" id="{7F9966CC-EDC0-4EFF-89F5-273C022757CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F834759-4960-418E-B528-A39CCD461F24}</x14:id>
+          <x14:id>{D0739A8A-0C7F-4EEE-9D10-78EB806E435B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A7091EAC-F927-4E6B-9BCE-6FA9E85D344D}</x14:id>
+          <x14:id>{07D86FAA-CA69-47F5-8C22-AD6682457ECA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4802929-3C3F-4BAE-9946-8EF68A14ACC7}</x14:id>
+          <x14:id>{85E5EA9A-24C4-4EF9-9CC7-1608590E21CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{75DF331A-0C47-484B-9278-BDDCE5DAFC4E}</x14:id>
+          <x14:id>{492F08A8-3677-4C2C-8E3E-37219B61ACB1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F834759-4960-418E-B528-A39CCD461F24}">
+          <x14:cfRule type="dataBar" id="{D0739A8A-0C7F-4EEE-9D10-78EB806E435B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A7091EAC-F927-4E6B-9BCE-6FA9E85D344D}">
+          <x14:cfRule type="dataBar" id="{07D86FAA-CA69-47F5-8C22-AD6682457ECA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4802929-3C3F-4BAE-9946-8EF68A14ACC7}">
+          <x14:cfRule type="dataBar" id="{85E5EA9A-24C4-4EF9-9CC7-1608590E21CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{75DF331A-0C47-484B-9278-BDDCE5DAFC4E}">
+          <x14:cfRule type="dataBar" id="{492F08A8-3677-4C2C-8E3E-37219B61ACB1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E27CDDC2-6AA6-4CC6-B022-F7AF0E78366E}</x14:id>
+          <x14:id>{7516D542-D6C4-4D81-B099-4E4C94595EB1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{29306635-A52D-4C9E-B988-DBF27BD4CEEB}</x14:id>
+          <x14:id>{6266D9EF-266F-4D25-B1DB-668026FC54E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F86B9855-215B-4443-B3CC-30A9538EA9FA}</x14:id>
+          <x14:id>{8B2FE127-BCE0-4117-A481-9B70A49DBFC1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F9966CC-EDC0-4EFF-89F5-273C022757CB}</x14:id>
+          <x14:id>{A0776D1F-D76D-4EA0-8BBC-70B5275BDD6A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E27CDDC2-6AA6-4CC6-B022-F7AF0E78366E}">
+          <x14:cfRule type="dataBar" id="{7516D542-D6C4-4D81-B099-4E4C94595EB1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{29306635-A52D-4C9E-B988-DBF27BD4CEEB}">
+          <x14:cfRule type="dataBar" id="{6266D9EF-266F-4D25-B1DB-668026FC54E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F86B9855-215B-4443-B3CC-30A9538EA9FA}">
+          <x14:cfRule type="dataBar" id="{8B2FE127-BCE0-4117-A481-9B70A49DBFC1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F9966CC-EDC0-4EFF-89F5-273C022757CB}">
+          <x14:cfRule type="dataBar" id="{A0776D1F-D76D-4EA0-8BBC-70B5275BDD6A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0739A8A-0C7F-4EEE-9D10-78EB806E435B}</x14:id>
+          <x14:id>{DA010253-5FD9-494A-B3D4-7313E818418A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07D86FAA-CA69-47F5-8C22-AD6682457ECA}</x14:id>
+          <x14:id>{307711D9-3805-4CAF-B89A-9CA5F2594E71}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{85E5EA9A-24C4-4EF9-9CC7-1608590E21CB}</x14:id>
+          <x14:id>{B61A5F38-701C-4031-8127-F0E9D0270103}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{492F08A8-3677-4C2C-8E3E-37219B61ACB1}</x14:id>
+          <x14:id>{74FBFF40-B0DA-4436-B5E7-A663DAD0FA32}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0739A8A-0C7F-4EEE-9D10-78EB806E435B}">
+          <x14:cfRule type="dataBar" id="{DA010253-5FD9-494A-B3D4-7313E818418A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07D86FAA-CA69-47F5-8C22-AD6682457ECA}">
+          <x14:cfRule type="dataBar" id="{307711D9-3805-4CAF-B89A-9CA5F2594E71}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{85E5EA9A-24C4-4EF9-9CC7-1608590E21CB}">
+          <x14:cfRule type="dataBar" id="{B61A5F38-701C-4031-8127-F0E9D0270103}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{492F08A8-3677-4C2C-8E3E-37219B61ACB1}">
+          <x14:cfRule type="dataBar" id="{74FBFF40-B0DA-4436-B5E7-A663DAD0FA32}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7516D542-D6C4-4D81-B099-4E4C94595EB1}</x14:id>
+          <x14:id>{E0B89C96-F0AF-481A-83A5-43B2E75DF1F7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6266D9EF-266F-4D25-B1DB-668026FC54E6}</x14:id>
+          <x14:id>{7F255F93-F065-4528-9164-4403CBF1D132}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8B2FE127-BCE0-4117-A481-9B70A49DBFC1}</x14:id>
+          <x14:id>{EB37EB78-A809-497B-B989-98C7B8AD53A4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0776D1F-D76D-4EA0-8BBC-70B5275BDD6A}</x14:id>
+          <x14:id>{1B876B2A-5B52-4D1B-A4AD-C33E3FB5517B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7516D542-D6C4-4D81-B099-4E4C94595EB1}">
+          <x14:cfRule type="dataBar" id="{E0B89C96-F0AF-481A-83A5-43B2E75DF1F7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6266D9EF-266F-4D25-B1DB-668026FC54E6}">
+          <x14:cfRule type="dataBar" id="{7F255F93-F065-4528-9164-4403CBF1D132}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8B2FE127-BCE0-4117-A481-9B70A49DBFC1}">
+          <x14:cfRule type="dataBar" id="{EB37EB78-A809-497B-B989-98C7B8AD53A4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0776D1F-D76D-4EA0-8BBC-70B5275BDD6A}">
+          <x14:cfRule type="dataBar" id="{1B876B2A-5B52-4D1B-A4AD-C33E3FB5517B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DA010253-5FD9-494A-B3D4-7313E818418A}</x14:id>
+          <x14:id>{857E12D1-C27B-43CF-81E0-9E37518509D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{307711D9-3805-4CAF-B89A-9CA5F2594E71}</x14:id>
+          <x14:id>{6F6B6A36-41A4-4E43-9B6A-776A962C5276}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B61A5F38-701C-4031-8127-F0E9D0270103}</x14:id>
+          <x14:id>{AF18B6C5-4470-46D4-BA01-B1D377EA36A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74FBFF40-B0DA-4436-B5E7-A663DAD0FA32}</x14:id>
+          <x14:id>{CA724AC5-DF11-4853-BFC8-4C0E2DA67A83}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DA010253-5FD9-494A-B3D4-7313E818418A}">
+          <x14:cfRule type="dataBar" id="{857E12D1-C27B-43CF-81E0-9E37518509D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{307711D9-3805-4CAF-B89A-9CA5F2594E71}">
+          <x14:cfRule type="dataBar" id="{6F6B6A36-41A4-4E43-9B6A-776A962C5276}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B61A5F38-701C-4031-8127-F0E9D0270103}">
+          <x14:cfRule type="dataBar" id="{AF18B6C5-4470-46D4-BA01-B1D377EA36A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74FBFF40-B0DA-4436-B5E7-A663DAD0FA32}">
+          <x14:cfRule type="dataBar" id="{CA724AC5-DF11-4853-BFC8-4C0E2DA67A83}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E0B89C96-F0AF-481A-83A5-43B2E75DF1F7}</x14:id>
+          <x14:id>{F58B5753-AE19-4475-AAE2-8E996308A7B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F255F93-F065-4528-9164-4403CBF1D132}</x14:id>
+          <x14:id>{42509B89-47F0-4EBE-B4A6-D87E077A967B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EB37EB78-A809-497B-B989-98C7B8AD53A4}</x14:id>
+          <x14:id>{50594F52-6B27-445E-9C5C-4E84E63444FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1B876B2A-5B52-4D1B-A4AD-C33E3FB5517B}</x14:id>
+          <x14:id>{1C79B98E-1B48-42BD-BBDE-8F086C10A8F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E0B89C96-F0AF-481A-83A5-43B2E75DF1F7}">
+          <x14:cfRule type="dataBar" id="{F58B5753-AE19-4475-AAE2-8E996308A7B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F255F93-F065-4528-9164-4403CBF1D132}">
+          <x14:cfRule type="dataBar" id="{42509B89-47F0-4EBE-B4A6-D87E077A967B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EB37EB78-A809-497B-B989-98C7B8AD53A4}">
+          <x14:cfRule type="dataBar" id="{50594F52-6B27-445E-9C5C-4E84E63444FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1B876B2A-5B52-4D1B-A4AD-C33E3FB5517B}">
+          <x14:cfRule type="dataBar" id="{1C79B98E-1B48-42BD-BBDE-8F086C10A8F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{857E12D1-C27B-43CF-81E0-9E37518509D0}</x14:id>
+          <x14:id>{0A7C1E13-EF2F-4CD7-BCD7-0E77B12A685E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F6B6A36-41A4-4E43-9B6A-776A962C5276}</x14:id>
+          <x14:id>{9AFA80C4-7521-4517-8E5E-DAD6FD914336}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF18B6C5-4470-46D4-BA01-B1D377EA36A9}</x14:id>
+          <x14:id>{2A16A99D-A21A-4764-9675-C4AA7B0500D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CA724AC5-DF11-4853-BFC8-4C0E2DA67A83}</x14:id>
+          <x14:id>{F9E6533C-494B-419C-BD69-A526F5EF9A5E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{857E12D1-C27B-43CF-81E0-9E37518509D0}">
+          <x14:cfRule type="dataBar" id="{0A7C1E13-EF2F-4CD7-BCD7-0E77B12A685E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F6B6A36-41A4-4E43-9B6A-776A962C5276}">
+          <x14:cfRule type="dataBar" id="{9AFA80C4-7521-4517-8E5E-DAD6FD914336}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF18B6C5-4470-46D4-BA01-B1D377EA36A9}">
+          <x14:cfRule type="dataBar" id="{2A16A99D-A21A-4764-9675-C4AA7B0500D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CA724AC5-DF11-4853-BFC8-4C0E2DA67A83}">
+          <x14:cfRule type="dataBar" id="{F9E6533C-494B-419C-BD69-A526F5EF9A5E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F58B5753-AE19-4475-AAE2-8E996308A7B7}</x14:id>
+          <x14:id>{C9370611-D634-41C2-B6AD-5882C49D69D8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42509B89-47F0-4EBE-B4A6-D87E077A967B}</x14:id>
+          <x14:id>{1AD0BEA4-81C0-4344-8C04-E1C8AC54D2C2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{50594F52-6B27-445E-9C5C-4E84E63444FC}</x14:id>
+          <x14:id>{158B6D3B-6636-4499-8A25-42C5546CD2A4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1C79B98E-1B48-42BD-BBDE-8F086C10A8F2}</x14:id>
+          <x14:id>{9CD2787B-850D-4060-9335-D994E31D8AEE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F58B5753-AE19-4475-AAE2-8E996308A7B7}">
+          <x14:cfRule type="dataBar" id="{C9370611-D634-41C2-B6AD-5882C49D69D8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42509B89-47F0-4EBE-B4A6-D87E077A967B}">
+          <x14:cfRule type="dataBar" id="{1AD0BEA4-81C0-4344-8C04-E1C8AC54D2C2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{50594F52-6B27-445E-9C5C-4E84E63444FC}">
+          <x14:cfRule type="dataBar" id="{158B6D3B-6636-4499-8A25-42C5546CD2A4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1C79B98E-1B48-42BD-BBDE-8F086C10A8F2}">
+          <x14:cfRule type="dataBar" id="{9CD2787B-850D-4060-9335-D994E31D8AEE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0A7C1E13-EF2F-4CD7-BCD7-0E77B12A685E}</x14:id>
+          <x14:id>{AC3DD1DC-18FF-4D42-B3BD-22DCE96913DE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9AFA80C4-7521-4517-8E5E-DAD6FD914336}</x14:id>
+          <x14:id>{A48E4F96-6794-47E6-ABD1-6E450781416D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A16A99D-A21A-4764-9675-C4AA7B0500D2}</x14:id>
+          <x14:id>{9FE8AB75-E628-4EBF-B0FB-EE0A0FCFADD9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F9E6533C-494B-419C-BD69-A526F5EF9A5E}</x14:id>
+          <x14:id>{BEA14B19-7ACB-4AFB-A704-FE6128E72D28}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0A7C1E13-EF2F-4CD7-BCD7-0E77B12A685E}">
+          <x14:cfRule type="dataBar" id="{AC3DD1DC-18FF-4D42-B3BD-22DCE96913DE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9AFA80C4-7521-4517-8E5E-DAD6FD914336}">
+          <x14:cfRule type="dataBar" id="{A48E4F96-6794-47E6-ABD1-6E450781416D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A16A99D-A21A-4764-9675-C4AA7B0500D2}">
+          <x14:cfRule type="dataBar" id="{9FE8AB75-E628-4EBF-B0FB-EE0A0FCFADD9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F9E6533C-494B-419C-BD69-A526F5EF9A5E}">
+          <x14:cfRule type="dataBar" id="{BEA14B19-7ACB-4AFB-A704-FE6128E72D28}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C9370611-D634-41C2-B6AD-5882C49D69D8}</x14:id>
+          <x14:id>{00F1E328-9BD0-4A14-A3D7-7CE9B35F57AE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1AD0BEA4-81C0-4344-8C04-E1C8AC54D2C2}</x14:id>
+          <x14:id>{9914AD46-733B-4FD6-BBCF-3D0ACE73D549}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{158B6D3B-6636-4499-8A25-42C5546CD2A4}</x14:id>
+          <x14:id>{40614265-CB14-4DD2-B28D-33FA46A7C52B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9CD2787B-850D-4060-9335-D994E31D8AEE}</x14:id>
+          <x14:id>{D6B68F18-9479-4D71-ACC3-909D6BBDECCB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C9370611-D634-41C2-B6AD-5882C49D69D8}">
+          <x14:cfRule type="dataBar" id="{00F1E328-9BD0-4A14-A3D7-7CE9B35F57AE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1AD0BEA4-81C0-4344-8C04-E1C8AC54D2C2}">
+          <x14:cfRule type="dataBar" id="{9914AD46-733B-4FD6-BBCF-3D0ACE73D549}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{158B6D3B-6636-4499-8A25-42C5546CD2A4}">
+          <x14:cfRule type="dataBar" id="{40614265-CB14-4DD2-B28D-33FA46A7C52B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9CD2787B-850D-4060-9335-D994E31D8AEE}">
+          <x14:cfRule type="dataBar" id="{D6B68F18-9479-4D71-ACC3-909D6BBDECCB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AC3DD1DC-18FF-4D42-B3BD-22DCE96913DE}</x14:id>
+          <x14:id>{1AAE112C-46B7-4DCD-8F57-38AAA84A8C1F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A48E4F96-6794-47E6-ABD1-6E450781416D}</x14:id>
+          <x14:id>{69323B7D-5A0D-4AF5-AAC7-9199F359DF19}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9FE8AB75-E628-4EBF-B0FB-EE0A0FCFADD9}</x14:id>
+          <x14:id>{0B0D172B-22CD-4BD2-BF60-80747B8AD476}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BEA14B19-7ACB-4AFB-A704-FE6128E72D28}</x14:id>
+          <x14:id>{42954A0C-6E37-4297-8829-389BF269EDC7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AC3DD1DC-18FF-4D42-B3BD-22DCE96913DE}">
+          <x14:cfRule type="dataBar" id="{1AAE112C-46B7-4DCD-8F57-38AAA84A8C1F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A48E4F96-6794-47E6-ABD1-6E450781416D}">
+          <x14:cfRule type="dataBar" id="{69323B7D-5A0D-4AF5-AAC7-9199F359DF19}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9FE8AB75-E628-4EBF-B0FB-EE0A0FCFADD9}">
+          <x14:cfRule type="dataBar" id="{0B0D172B-22CD-4BD2-BF60-80747B8AD476}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BEA14B19-7ACB-4AFB-A704-FE6128E72D28}">
+          <x14:cfRule type="dataBar" id="{42954A0C-6E37-4297-8829-389BF269EDC7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00F1E328-9BD0-4A14-A3D7-7CE9B35F57AE}</x14:id>
+          <x14:id>{1C39CD09-3E2B-40FE-B8F9-3D62BF57D824}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9914AD46-733B-4FD6-BBCF-3D0ACE73D549}</x14:id>
+          <x14:id>{2EE747EA-B906-46F9-AB67-6CE09CA738D3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{40614265-CB14-4DD2-B28D-33FA46A7C52B}</x14:id>
+          <x14:id>{48CC2E28-89DC-445B-9F5B-C10E46AC21C9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D6B68F18-9479-4D71-ACC3-909D6BBDECCB}</x14:id>
+          <x14:id>{9D83E961-51FE-4BA2-A5F3-DCE94D1485C4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00F1E328-9BD0-4A14-A3D7-7CE9B35F57AE}">
+          <x14:cfRule type="dataBar" id="{1C39CD09-3E2B-40FE-B8F9-3D62BF57D824}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9914AD46-733B-4FD6-BBCF-3D0ACE73D549}">
+          <x14:cfRule type="dataBar" id="{2EE747EA-B906-46F9-AB67-6CE09CA738D3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{40614265-CB14-4DD2-B28D-33FA46A7C52B}">
+          <x14:cfRule type="dataBar" id="{48CC2E28-89DC-445B-9F5B-C10E46AC21C9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D6B68F18-9479-4D71-ACC3-909D6BBDECCB}">
+          <x14:cfRule type="dataBar" id="{9D83E961-51FE-4BA2-A5F3-DCE94D1485C4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1AAE112C-46B7-4DCD-8F57-38AAA84A8C1F}</x14:id>
+          <x14:id>{E7DE30EC-4E46-4458-AB84-F2D04205BAA0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{69323B7D-5A0D-4AF5-AAC7-9199F359DF19}</x14:id>
+          <x14:id>{CFEFEEA3-1EB4-41EF-A8BC-5D58FB70A9A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B0D172B-22CD-4BD2-BF60-80747B8AD476}</x14:id>
+          <x14:id>{B15A5FED-1CDB-414D-BD6D-4D0C1A1A58B6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42954A0C-6E37-4297-8829-389BF269EDC7}</x14:id>
+          <x14:id>{6C291CBE-A63C-41C8-9D1E-0F0EE9FAFE94}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1AAE112C-46B7-4DCD-8F57-38AAA84A8C1F}">
+          <x14:cfRule type="dataBar" id="{E7DE30EC-4E46-4458-AB84-F2D04205BAA0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{69323B7D-5A0D-4AF5-AAC7-9199F359DF19}">
+          <x14:cfRule type="dataBar" id="{CFEFEEA3-1EB4-41EF-A8BC-5D58FB70A9A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B0D172B-22CD-4BD2-BF60-80747B8AD476}">
+          <x14:cfRule type="dataBar" id="{B15A5FED-1CDB-414D-BD6D-4D0C1A1A58B6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42954A0C-6E37-4297-8829-389BF269EDC7}">
+          <x14:cfRule type="dataBar" id="{6C291CBE-A63C-41C8-9D1E-0F0EE9FAFE94}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1C39CD09-3E2B-40FE-B8F9-3D62BF57D824}</x14:id>
+          <x14:id>{B9477F18-066A-4358-87DC-25B26C0A9230}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2EE747EA-B906-46F9-AB67-6CE09CA738D3}</x14:id>
+          <x14:id>{B40F2BB9-8534-4B37-A98D-23075CE2B001}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{48CC2E28-89DC-445B-9F5B-C10E46AC21C9}</x14:id>
+          <x14:id>{8E96BD5B-21C7-4251-918C-1283D3D24FD2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9D83E961-51FE-4BA2-A5F3-DCE94D1485C4}</x14:id>
+          <x14:id>{86D5406E-B359-4948-A446-1100D844CA01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1C39CD09-3E2B-40FE-B8F9-3D62BF57D824}">
+          <x14:cfRule type="dataBar" id="{B9477F18-066A-4358-87DC-25B26C0A9230}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2EE747EA-B906-46F9-AB67-6CE09CA738D3}">
+          <x14:cfRule type="dataBar" id="{B40F2BB9-8534-4B37-A98D-23075CE2B001}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{48CC2E28-89DC-445B-9F5B-C10E46AC21C9}">
+          <x14:cfRule type="dataBar" id="{8E96BD5B-21C7-4251-918C-1283D3D24FD2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9D83E961-51FE-4BA2-A5F3-DCE94D1485C4}">
+          <x14:cfRule type="dataBar" id="{86D5406E-B359-4948-A446-1100D844CA01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-29 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12344,7 +12344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E7DE30EC-4E46-4458-AB84-F2D04205BAA0}</x14:id>
+          <x14:id>{228AD978-8219-4367-ACFD-90A4CB80AC52}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12358,7 +12358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CFEFEEA3-1EB4-41EF-A8BC-5D58FB70A9A9}</x14:id>
+          <x14:id>{D0DA25FD-5062-4457-9EA8-74358DEB00E5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12372,7 +12372,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B15A5FED-1CDB-414D-BD6D-4D0C1A1A58B6}</x14:id>
+          <x14:id>{42F0D0C7-B490-4D89-923E-5341A222FDC6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12386,7 +12386,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6C291CBE-A63C-41C8-9D1E-0F0EE9FAFE94}</x14:id>
+          <x14:id>{60FD9E4B-3690-4BFA-A4E3-363414793947}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12396,7 +12396,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E7DE30EC-4E46-4458-AB84-F2D04205BAA0}">
+          <x14:cfRule type="dataBar" id="{228AD978-8219-4367-ACFD-90A4CB80AC52}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12409,7 +12409,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CFEFEEA3-1EB4-41EF-A8BC-5D58FB70A9A9}">
+          <x14:cfRule type="dataBar" id="{D0DA25FD-5062-4457-9EA8-74358DEB00E5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12422,7 +12422,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B15A5FED-1CDB-414D-BD6D-4D0C1A1A58B6}">
+          <x14:cfRule type="dataBar" id="{42F0D0C7-B490-4D89-923E-5341A222FDC6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12435,7 +12435,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6C291CBE-A63C-41C8-9D1E-0F0EE9FAFE94}">
+          <x14:cfRule type="dataBar" id="{60FD9E4B-3690-4BFA-A4E3-363414793947}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27884,7 +27884,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B9477F18-066A-4358-87DC-25B26C0A9230}</x14:id>
+          <x14:id>{50440E90-D7DF-433B-9CB9-45BC5F2FEFB7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27898,7 +27898,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B40F2BB9-8534-4B37-A98D-23075CE2B001}</x14:id>
+          <x14:id>{37E4340E-8754-4A18-BDEF-9539AE059D3D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27912,7 +27912,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8E96BD5B-21C7-4251-918C-1283D3D24FD2}</x14:id>
+          <x14:id>{1572CE57-4832-436F-8CB3-790E660FCFA0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27926,7 +27926,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{86D5406E-B359-4948-A446-1100D844CA01}</x14:id>
+          <x14:id>{592B1812-A3E5-4FF0-98C6-FC9DB1645AA5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27936,7 +27936,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B9477F18-066A-4358-87DC-25B26C0A9230}">
+          <x14:cfRule type="dataBar" id="{50440E90-D7DF-433B-9CB9-45BC5F2FEFB7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27949,7 +27949,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B40F2BB9-8534-4B37-A98D-23075CE2B001}">
+          <x14:cfRule type="dataBar" id="{37E4340E-8754-4A18-BDEF-9539AE059D3D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27962,7 +27962,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8E96BD5B-21C7-4251-918C-1283D3D24FD2}">
+          <x14:cfRule type="dataBar" id="{1572CE57-4832-436F-8CB3-790E660FCFA0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27975,7 +27975,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{86D5406E-B359-4948-A446-1100D844CA01}">
+          <x14:cfRule type="dataBar" id="{592B1812-A3E5-4FF0-98C6-FC9DB1645AA5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6BE42E9-68C1-46FF-8DCB-C635121D4722}</x14:id>
+          <x14:id>{62046B8C-5987-495B-87BF-08F95CF030E1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9AAD47FA-E8FA-44BF-952D-97E113FA8616}</x14:id>
+          <x14:id>{1915DBFA-849A-47F5-B4CA-73737D348DD5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{54FC6FFD-A407-47A2-9B48-36023D742918}</x14:id>
+          <x14:id>{F1A3772D-0CDE-4A1C-AB7C-445A41C7F2C1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C9225C2A-3173-4D94-B880-85A127BAA202}</x14:id>
+          <x14:id>{D40FAA4D-7AF9-4C4C-B30E-3BB89F657B7B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6BE42E9-68C1-46FF-8DCB-C635121D4722}">
+          <x14:cfRule type="dataBar" id="{62046B8C-5987-495B-87BF-08F95CF030E1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9AAD47FA-E8FA-44BF-952D-97E113FA8616}">
+          <x14:cfRule type="dataBar" id="{1915DBFA-849A-47F5-B4CA-73737D348DD5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{54FC6FFD-A407-47A2-9B48-36023D742918}">
+          <x14:cfRule type="dataBar" id="{F1A3772D-0CDE-4A1C-AB7C-445A41C7F2C1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C9225C2A-3173-4D94-B880-85A127BAA202}">
+          <x14:cfRule type="dataBar" id="{D40FAA4D-7AF9-4C4C-B30E-3BB89F657B7B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49B913B7-5AC1-4440-93C3-F915EDFED523}</x14:id>
+          <x14:id>{18EACE66-D9A6-423C-8356-5DBBF26599F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FB8733CC-86D1-4C61-B3B6-AC51473A3073}</x14:id>
+          <x14:id>{8882ABF5-D69E-4656-BF91-68AF5D9C2D40}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BEC232FC-E68A-4BD6-A8D3-D1208BCF75F5}</x14:id>
+          <x14:id>{0EB70FE4-15C6-4B64-9D7B-938199E36041}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{47C02CA0-4F35-4457-BF88-1EA8355DB978}</x14:id>
+          <x14:id>{54033968-1D3B-4C3F-8F7C-EF0E8E4F758D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49B913B7-5AC1-4440-93C3-F915EDFED523}">
+          <x14:cfRule type="dataBar" id="{18EACE66-D9A6-423C-8356-5DBBF26599F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FB8733CC-86D1-4C61-B3B6-AC51473A3073}">
+          <x14:cfRule type="dataBar" id="{8882ABF5-D69E-4656-BF91-68AF5D9C2D40}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BEC232FC-E68A-4BD6-A8D3-D1208BCF75F5}">
+          <x14:cfRule type="dataBar" id="{0EB70FE4-15C6-4B64-9D7B-938199E36041}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{47C02CA0-4F35-4457-BF88-1EA8355DB978}">
+          <x14:cfRule type="dataBar" id="{54033968-1D3B-4C3F-8F7C-EF0E8E4F758D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62046B8C-5987-495B-87BF-08F95CF030E1}</x14:id>
+          <x14:id>{613042ED-1017-4A70-98E4-8FD262CE30CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1915DBFA-849A-47F5-B4CA-73737D348DD5}</x14:id>
+          <x14:id>{3CFA769E-76AC-4F46-88FA-20DF499A2DEE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F1A3772D-0CDE-4A1C-AB7C-445A41C7F2C1}</x14:id>
+          <x14:id>{E06A2CE2-1593-4A06-831E-40EC7BA283B6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D40FAA4D-7AF9-4C4C-B30E-3BB89F657B7B}</x14:id>
+          <x14:id>{4DFF573E-2D85-4014-898E-02876FBB6A31}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62046B8C-5987-495B-87BF-08F95CF030E1}">
+          <x14:cfRule type="dataBar" id="{613042ED-1017-4A70-98E4-8FD262CE30CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1915DBFA-849A-47F5-B4CA-73737D348DD5}">
+          <x14:cfRule type="dataBar" id="{3CFA769E-76AC-4F46-88FA-20DF499A2DEE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F1A3772D-0CDE-4A1C-AB7C-445A41C7F2C1}">
+          <x14:cfRule type="dataBar" id="{E06A2CE2-1593-4A06-831E-40EC7BA283B6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D40FAA4D-7AF9-4C4C-B30E-3BB89F657B7B}">
+          <x14:cfRule type="dataBar" id="{4DFF573E-2D85-4014-898E-02876FBB6A31}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{18EACE66-D9A6-423C-8356-5DBBF26599F1}</x14:id>
+          <x14:id>{75D499DA-682C-42A2-9C51-2A8B2C109E42}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8882ABF5-D69E-4656-BF91-68AF5D9C2D40}</x14:id>
+          <x14:id>{8C745096-5015-43AE-8B56-350B456F13F6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0EB70FE4-15C6-4B64-9D7B-938199E36041}</x14:id>
+          <x14:id>{13B8DAF8-52D4-4B14-9E5E-CC3EB7F227DA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{54033968-1D3B-4C3F-8F7C-EF0E8E4F758D}</x14:id>
+          <x14:id>{A1D7FED1-4CA1-4B51-A97F-7E38DC4396A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{18EACE66-D9A6-423C-8356-5DBBF26599F1}">
+          <x14:cfRule type="dataBar" id="{75D499DA-682C-42A2-9C51-2A8B2C109E42}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8882ABF5-D69E-4656-BF91-68AF5D9C2D40}">
+          <x14:cfRule type="dataBar" id="{8C745096-5015-43AE-8B56-350B456F13F6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0EB70FE4-15C6-4B64-9D7B-938199E36041}">
+          <x14:cfRule type="dataBar" id="{13B8DAF8-52D4-4B14-9E5E-CC3EB7F227DA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{54033968-1D3B-4C3F-8F7C-EF0E8E4F758D}">
+          <x14:cfRule type="dataBar" id="{A1D7FED1-4CA1-4B51-A97F-7E38DC4396A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{613042ED-1017-4A70-98E4-8FD262CE30CB}</x14:id>
+          <x14:id>{9519AB48-8120-4771-95B0-617A3250CEFD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CFA769E-76AC-4F46-88FA-20DF499A2DEE}</x14:id>
+          <x14:id>{BED71F5F-1589-4529-956C-F26BAD68C577}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E06A2CE2-1593-4A06-831E-40EC7BA283B6}</x14:id>
+          <x14:id>{E94B900C-AC4B-40AA-94FC-E1E07502EF12}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4DFF573E-2D85-4014-898E-02876FBB6A31}</x14:id>
+          <x14:id>{A22EC5CB-29CC-4FAB-8526-F0BDA38CC52F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{613042ED-1017-4A70-98E4-8FD262CE30CB}">
+          <x14:cfRule type="dataBar" id="{9519AB48-8120-4771-95B0-617A3250CEFD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CFA769E-76AC-4F46-88FA-20DF499A2DEE}">
+          <x14:cfRule type="dataBar" id="{BED71F5F-1589-4529-956C-F26BAD68C577}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E06A2CE2-1593-4A06-831E-40EC7BA283B6}">
+          <x14:cfRule type="dataBar" id="{E94B900C-AC4B-40AA-94FC-E1E07502EF12}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4DFF573E-2D85-4014-898E-02876FBB6A31}">
+          <x14:cfRule type="dataBar" id="{A22EC5CB-29CC-4FAB-8526-F0BDA38CC52F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{75D499DA-682C-42A2-9C51-2A8B2C109E42}</x14:id>
+          <x14:id>{9CCF5D1A-9BCC-4586-B943-F9181F0D0ECB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C745096-5015-43AE-8B56-350B456F13F6}</x14:id>
+          <x14:id>{6509D986-7219-4046-B942-ABE23A6D4E8E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13B8DAF8-52D4-4B14-9E5E-CC3EB7F227DA}</x14:id>
+          <x14:id>{AC8B00AC-C9FC-4C41-B472-9E58E9820312}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A1D7FED1-4CA1-4B51-A97F-7E38DC4396A2}</x14:id>
+          <x14:id>{05943673-8A60-4A73-B98D-F96BFA8C2812}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{75D499DA-682C-42A2-9C51-2A8B2C109E42}">
+          <x14:cfRule type="dataBar" id="{9CCF5D1A-9BCC-4586-B943-F9181F0D0ECB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C745096-5015-43AE-8B56-350B456F13F6}">
+          <x14:cfRule type="dataBar" id="{6509D986-7219-4046-B942-ABE23A6D4E8E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13B8DAF8-52D4-4B14-9E5E-CC3EB7F227DA}">
+          <x14:cfRule type="dataBar" id="{AC8B00AC-C9FC-4C41-B472-9E58E9820312}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A1D7FED1-4CA1-4B51-A97F-7E38DC4396A2}">
+          <x14:cfRule type="dataBar" id="{05943673-8A60-4A73-B98D-F96BFA8C2812}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9519AB48-8120-4771-95B0-617A3250CEFD}</x14:id>
+          <x14:id>{274F242A-CEEB-46FD-97AF-41D2A9203E59}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BED71F5F-1589-4529-956C-F26BAD68C577}</x14:id>
+          <x14:id>{F80EFA54-4CF7-4078-B8E8-103541A7ED05}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E94B900C-AC4B-40AA-94FC-E1E07502EF12}</x14:id>
+          <x14:id>{E64EC18B-E606-4053-B710-E2C5D0174431}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A22EC5CB-29CC-4FAB-8526-F0BDA38CC52F}</x14:id>
+          <x14:id>{903851FC-2EDF-43FC-A5E9-6266F9E04942}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9519AB48-8120-4771-95B0-617A3250CEFD}">
+          <x14:cfRule type="dataBar" id="{274F242A-CEEB-46FD-97AF-41D2A9203E59}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BED71F5F-1589-4529-956C-F26BAD68C577}">
+          <x14:cfRule type="dataBar" id="{F80EFA54-4CF7-4078-B8E8-103541A7ED05}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E94B900C-AC4B-40AA-94FC-E1E07502EF12}">
+          <x14:cfRule type="dataBar" id="{E64EC18B-E606-4053-B710-E2C5D0174431}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A22EC5CB-29CC-4FAB-8526-F0BDA38CC52F}">
+          <x14:cfRule type="dataBar" id="{903851FC-2EDF-43FC-A5E9-6266F9E04942}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9CCF5D1A-9BCC-4586-B943-F9181F0D0ECB}</x14:id>
+          <x14:id>{8C11E8F5-E3DA-411E-84D7-9A991E361AFE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6509D986-7219-4046-B942-ABE23A6D4E8E}</x14:id>
+          <x14:id>{C901F2A0-65E9-4412-9917-6DD7A6A00B50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AC8B00AC-C9FC-4C41-B472-9E58E9820312}</x14:id>
+          <x14:id>{6E884661-3188-47C9-885A-AE0F46B89AA2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05943673-8A60-4A73-B98D-F96BFA8C2812}</x14:id>
+          <x14:id>{95E35D96-45BE-44AE-B053-1BB5172441ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9CCF5D1A-9BCC-4586-B943-F9181F0D0ECB}">
+          <x14:cfRule type="dataBar" id="{8C11E8F5-E3DA-411E-84D7-9A991E361AFE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6509D986-7219-4046-B942-ABE23A6D4E8E}">
+          <x14:cfRule type="dataBar" id="{C901F2A0-65E9-4412-9917-6DD7A6A00B50}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AC8B00AC-C9FC-4C41-B472-9E58E9820312}">
+          <x14:cfRule type="dataBar" id="{6E884661-3188-47C9-885A-AE0F46B89AA2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05943673-8A60-4A73-B98D-F96BFA8C2812}">
+          <x14:cfRule type="dataBar" id="{95E35D96-45BE-44AE-B053-1BB5172441ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{274F242A-CEEB-46FD-97AF-41D2A9203E59}</x14:id>
+          <x14:id>{67B1BB34-51F8-44C9-88A1-C53FCEC902C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F80EFA54-4CF7-4078-B8E8-103541A7ED05}</x14:id>
+          <x14:id>{277A9F52-AFD1-47B5-AAFF-A7DFC965B5CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E64EC18B-E606-4053-B710-E2C5D0174431}</x14:id>
+          <x14:id>{EA5DE4DB-C6E7-4EAB-8BAB-52DD040B1EC8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{903851FC-2EDF-43FC-A5E9-6266F9E04942}</x14:id>
+          <x14:id>{84FFDF18-DA27-446F-AFD1-8A2ABAC75FA3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{274F242A-CEEB-46FD-97AF-41D2A9203E59}">
+          <x14:cfRule type="dataBar" id="{67B1BB34-51F8-44C9-88A1-C53FCEC902C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F80EFA54-4CF7-4078-B8E8-103541A7ED05}">
+          <x14:cfRule type="dataBar" id="{277A9F52-AFD1-47B5-AAFF-A7DFC965B5CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E64EC18B-E606-4053-B710-E2C5D0174431}">
+          <x14:cfRule type="dataBar" id="{EA5DE4DB-C6E7-4EAB-8BAB-52DD040B1EC8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{903851FC-2EDF-43FC-A5E9-6266F9E04942}">
+          <x14:cfRule type="dataBar" id="{84FFDF18-DA27-446F-AFD1-8A2ABAC75FA3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C11E8F5-E3DA-411E-84D7-9A991E361AFE}</x14:id>
+          <x14:id>{25408225-7523-402F-B001-5E54F1115103}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C901F2A0-65E9-4412-9917-6DD7A6A00B50}</x14:id>
+          <x14:id>{84505720-16CC-4598-A21C-8F7ED3E0EABE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6E884661-3188-47C9-885A-AE0F46B89AA2}</x14:id>
+          <x14:id>{578BC212-A73E-4C1E-8666-1F2FC9CA85EB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95E35D96-45BE-44AE-B053-1BB5172441ED}</x14:id>
+          <x14:id>{BDEBD416-B3F2-46E6-8F5C-2AB1F7A3B31E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C11E8F5-E3DA-411E-84D7-9A991E361AFE}">
+          <x14:cfRule type="dataBar" id="{25408225-7523-402F-B001-5E54F1115103}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C901F2A0-65E9-4412-9917-6DD7A6A00B50}">
+          <x14:cfRule type="dataBar" id="{84505720-16CC-4598-A21C-8F7ED3E0EABE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6E884661-3188-47C9-885A-AE0F46B89AA2}">
+          <x14:cfRule type="dataBar" id="{578BC212-A73E-4C1E-8666-1F2FC9CA85EB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95E35D96-45BE-44AE-B053-1BB5172441ED}">
+          <x14:cfRule type="dataBar" id="{BDEBD416-B3F2-46E6-8F5C-2AB1F7A3B31E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{67B1BB34-51F8-44C9-88A1-C53FCEC902C0}</x14:id>
+          <x14:id>{9B86DB4C-0D1C-4387-97CB-EFE4BF7DFD61}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{277A9F52-AFD1-47B5-AAFF-A7DFC965B5CF}</x14:id>
+          <x14:id>{E02AF512-823E-465C-B5D1-B20D592048B5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EA5DE4DB-C6E7-4EAB-8BAB-52DD040B1EC8}</x14:id>
+          <x14:id>{25DF2390-C6AE-4445-A9C7-632F99510B10}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84FFDF18-DA27-446F-AFD1-8A2ABAC75FA3}</x14:id>
+          <x14:id>{8B25D3A1-4D68-4E8F-95DC-D26C3FD460AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{67B1BB34-51F8-44C9-88A1-C53FCEC902C0}">
+          <x14:cfRule type="dataBar" id="{9B86DB4C-0D1C-4387-97CB-EFE4BF7DFD61}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{277A9F52-AFD1-47B5-AAFF-A7DFC965B5CF}">
+          <x14:cfRule type="dataBar" id="{E02AF512-823E-465C-B5D1-B20D592048B5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EA5DE4DB-C6E7-4EAB-8BAB-52DD040B1EC8}">
+          <x14:cfRule type="dataBar" id="{25DF2390-C6AE-4445-A9C7-632F99510B10}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84FFDF18-DA27-446F-AFD1-8A2ABAC75FA3}">
+          <x14:cfRule type="dataBar" id="{8B25D3A1-4D68-4E8F-95DC-D26C3FD460AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25408225-7523-402F-B001-5E54F1115103}</x14:id>
+          <x14:id>{7F004B3D-354E-4234-8470-0F6D16FB25A2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84505720-16CC-4598-A21C-8F7ED3E0EABE}</x14:id>
+          <x14:id>{11B16246-0C87-4D6E-BC57-B1822ADAB3CC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{578BC212-A73E-4C1E-8666-1F2FC9CA85EB}</x14:id>
+          <x14:id>{FEEF7A40-354C-4089-ACD0-C6DC574AAE52}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BDEBD416-B3F2-46E6-8F5C-2AB1F7A3B31E}</x14:id>
+          <x14:id>{49F599A2-E4A3-4562-B31A-6710D762A483}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25408225-7523-402F-B001-5E54F1115103}">
+          <x14:cfRule type="dataBar" id="{7F004B3D-354E-4234-8470-0F6D16FB25A2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84505720-16CC-4598-A21C-8F7ED3E0EABE}">
+          <x14:cfRule type="dataBar" id="{11B16246-0C87-4D6E-BC57-B1822ADAB3CC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{578BC212-A73E-4C1E-8666-1F2FC9CA85EB}">
+          <x14:cfRule type="dataBar" id="{FEEF7A40-354C-4089-ACD0-C6DC574AAE52}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BDEBD416-B3F2-46E6-8F5C-2AB1F7A3B31E}">
+          <x14:cfRule type="dataBar" id="{49F599A2-E4A3-4562-B31A-6710D762A483}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9B86DB4C-0D1C-4387-97CB-EFE4BF7DFD61}</x14:id>
+          <x14:id>{D06A4C1D-39AC-436F-ABA0-D616178E4DF3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E02AF512-823E-465C-B5D1-B20D592048B5}</x14:id>
+          <x14:id>{64A7F66E-82D2-4794-982C-683F29635678}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{25DF2390-C6AE-4445-A9C7-632F99510B10}</x14:id>
+          <x14:id>{CACFC225-4D19-48DF-8F91-B88DBB88E3ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8B25D3A1-4D68-4E8F-95DC-D26C3FD460AB}</x14:id>
+          <x14:id>{7F3AAEA1-6E3C-4B03-8333-1CEFA8D8D2BB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9B86DB4C-0D1C-4387-97CB-EFE4BF7DFD61}">
+          <x14:cfRule type="dataBar" id="{D06A4C1D-39AC-436F-ABA0-D616178E4DF3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E02AF512-823E-465C-B5D1-B20D592048B5}">
+          <x14:cfRule type="dataBar" id="{64A7F66E-82D2-4794-982C-683F29635678}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{25DF2390-C6AE-4445-A9C7-632F99510B10}">
+          <x14:cfRule type="dataBar" id="{CACFC225-4D19-48DF-8F91-B88DBB88E3ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8B25D3A1-4D68-4E8F-95DC-D26C3FD460AB}">
+          <x14:cfRule type="dataBar" id="{7F3AAEA1-6E3C-4B03-8333-1CEFA8D8D2BB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F004B3D-354E-4234-8470-0F6D16FB25A2}</x14:id>
+          <x14:id>{CB371F75-E764-4E58-8817-5DDFE6862AE7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11B16246-0C87-4D6E-BC57-B1822ADAB3CC}</x14:id>
+          <x14:id>{1E24B5C2-C47F-4449-9B3F-E9AA929297FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FEEF7A40-354C-4089-ACD0-C6DC574AAE52}</x14:id>
+          <x14:id>{965CB77A-D760-4943-9846-F9CBBBEA975A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49F599A2-E4A3-4562-B31A-6710D762A483}</x14:id>
+          <x14:id>{3BEAF4D9-FDDC-4534-9BE3-18C91CE332B3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F004B3D-354E-4234-8470-0F6D16FB25A2}">
+          <x14:cfRule type="dataBar" id="{CB371F75-E764-4E58-8817-5DDFE6862AE7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11B16246-0C87-4D6E-BC57-B1822ADAB3CC}">
+          <x14:cfRule type="dataBar" id="{1E24B5C2-C47F-4449-9B3F-E9AA929297FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FEEF7A40-354C-4089-ACD0-C6DC574AAE52}">
+          <x14:cfRule type="dataBar" id="{965CB77A-D760-4943-9846-F9CBBBEA975A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49F599A2-E4A3-4562-B31A-6710D762A483}">
+          <x14:cfRule type="dataBar" id="{3BEAF4D9-FDDC-4534-9BE3-18C91CE332B3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D06A4C1D-39AC-436F-ABA0-D616178E4DF3}</x14:id>
+          <x14:id>{B4E76975-F00C-4234-9242-E99F26EABD0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{64A7F66E-82D2-4794-982C-683F29635678}</x14:id>
+          <x14:id>{F918BA3B-901E-46A5-9BAB-85159D92891D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CACFC225-4D19-48DF-8F91-B88DBB88E3ED}</x14:id>
+          <x14:id>{229BE71F-8137-4193-A8BD-3F5E69512703}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F3AAEA1-6E3C-4B03-8333-1CEFA8D8D2BB}</x14:id>
+          <x14:id>{9E30FFEC-38F9-470D-BB77-E41E7BBB5C1F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D06A4C1D-39AC-436F-ABA0-D616178E4DF3}">
+          <x14:cfRule type="dataBar" id="{B4E76975-F00C-4234-9242-E99F26EABD0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{64A7F66E-82D2-4794-982C-683F29635678}">
+          <x14:cfRule type="dataBar" id="{F918BA3B-901E-46A5-9BAB-85159D92891D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CACFC225-4D19-48DF-8F91-B88DBB88E3ED}">
+          <x14:cfRule type="dataBar" id="{229BE71F-8137-4193-A8BD-3F5E69512703}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F3AAEA1-6E3C-4B03-8333-1CEFA8D8D2BB}">
+          <x14:cfRule type="dataBar" id="{9E30FFEC-38F9-470D-BB77-E41E7BBB5C1F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CB371F75-E764-4E58-8817-5DDFE6862AE7}</x14:id>
+          <x14:id>{B1A3C777-F171-49D8-BA34-2B9737CE87D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1E24B5C2-C47F-4449-9B3F-E9AA929297FA}</x14:id>
+          <x14:id>{21A80A15-9B4B-4E2C-AADF-CB20A1FE5DA1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{965CB77A-D760-4943-9846-F9CBBBEA975A}</x14:id>
+          <x14:id>{2B0A5E7D-0EDB-400D-8F6A-99EEFD1E58DC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3BEAF4D9-FDDC-4534-9BE3-18C91CE332B3}</x14:id>
+          <x14:id>{10C7DB64-F3CF-4F1C-A03B-85E2E1DDF378}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CB371F75-E764-4E58-8817-5DDFE6862AE7}">
+          <x14:cfRule type="dataBar" id="{B1A3C777-F171-49D8-BA34-2B9737CE87D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1E24B5C2-C47F-4449-9B3F-E9AA929297FA}">
+          <x14:cfRule type="dataBar" id="{21A80A15-9B4B-4E2C-AADF-CB20A1FE5DA1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{965CB77A-D760-4943-9846-F9CBBBEA975A}">
+          <x14:cfRule type="dataBar" id="{2B0A5E7D-0EDB-400D-8F6A-99EEFD1E58DC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3BEAF4D9-FDDC-4534-9BE3-18C91CE332B3}">
+          <x14:cfRule type="dataBar" id="{10C7DB64-F3CF-4F1C-A03B-85E2E1DDF378}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B4E76975-F00C-4234-9242-E99F26EABD0B}</x14:id>
+          <x14:id>{EA352346-5DD4-4D89-B8E5-F32AF3B74001}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F918BA3B-901E-46A5-9BAB-85159D92891D}</x14:id>
+          <x14:id>{655F91F4-133F-4375-92D6-5FE5CA1751FE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{229BE71F-8137-4193-A8BD-3F5E69512703}</x14:id>
+          <x14:id>{031E9460-EFB2-4D60-9BA1-CEB333440CB7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9E30FFEC-38F9-470D-BB77-E41E7BBB5C1F}</x14:id>
+          <x14:id>{9CA64B33-4C24-49E7-8D7D-2B1A37D1A035}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B4E76975-F00C-4234-9242-E99F26EABD0B}">
+          <x14:cfRule type="dataBar" id="{EA352346-5DD4-4D89-B8E5-F32AF3B74001}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F918BA3B-901E-46A5-9BAB-85159D92891D}">
+          <x14:cfRule type="dataBar" id="{655F91F4-133F-4375-92D6-5FE5CA1751FE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{229BE71F-8137-4193-A8BD-3F5E69512703}">
+          <x14:cfRule type="dataBar" id="{031E9460-EFB2-4D60-9BA1-CEB333440CB7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9E30FFEC-38F9-470D-BB77-E41E7BBB5C1F}">
+          <x14:cfRule type="dataBar" id="{9CA64B33-4C24-49E7-8D7D-2B1A37D1A035}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B1A3C777-F171-49D8-BA34-2B9737CE87D2}</x14:id>
+          <x14:id>{1BE520ED-089A-473F-A810-560B6DBCC6F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{21A80A15-9B4B-4E2C-AADF-CB20A1FE5DA1}</x14:id>
+          <x14:id>{0836A528-1DA5-4670-B1A7-205934B3CAEC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2B0A5E7D-0EDB-400D-8F6A-99EEFD1E58DC}</x14:id>
+          <x14:id>{887E71B7-BB09-48EC-A32C-91BE11076976}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{10C7DB64-F3CF-4F1C-A03B-85E2E1DDF378}</x14:id>
+          <x14:id>{7D99927B-AFE7-4EF3-8116-1ADC382B1629}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B1A3C777-F171-49D8-BA34-2B9737CE87D2}">
+          <x14:cfRule type="dataBar" id="{1BE520ED-089A-473F-A810-560B6DBCC6F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{21A80A15-9B4B-4E2C-AADF-CB20A1FE5DA1}">
+          <x14:cfRule type="dataBar" id="{0836A528-1DA5-4670-B1A7-205934B3CAEC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2B0A5E7D-0EDB-400D-8F6A-99EEFD1E58DC}">
+          <x14:cfRule type="dataBar" id="{887E71B7-BB09-48EC-A32C-91BE11076976}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{10C7DB64-F3CF-4F1C-A03B-85E2E1DDF378}">
+          <x14:cfRule type="dataBar" id="{7D99927B-AFE7-4EF3-8116-1ADC382B1629}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EA352346-5DD4-4D89-B8E5-F32AF3B74001}</x14:id>
+          <x14:id>{2055CE40-0B3A-437B-8A2F-4779886D3367}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{655F91F4-133F-4375-92D6-5FE5CA1751FE}</x14:id>
+          <x14:id>{F844DFA2-A65B-48F3-92F9-757BC4B93851}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{031E9460-EFB2-4D60-9BA1-CEB333440CB7}</x14:id>
+          <x14:id>{1DD67F2F-EA9A-40C8-99A2-33F0D39ED62B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9CA64B33-4C24-49E7-8D7D-2B1A37D1A035}</x14:id>
+          <x14:id>{D2FFA51A-4F14-46D8-98F4-101C1BEE7541}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EA352346-5DD4-4D89-B8E5-F32AF3B74001}">
+          <x14:cfRule type="dataBar" id="{2055CE40-0B3A-437B-8A2F-4779886D3367}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{655F91F4-133F-4375-92D6-5FE5CA1751FE}">
+          <x14:cfRule type="dataBar" id="{F844DFA2-A65B-48F3-92F9-757BC4B93851}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{031E9460-EFB2-4D60-9BA1-CEB333440CB7}">
+          <x14:cfRule type="dataBar" id="{1DD67F2F-EA9A-40C8-99A2-33F0D39ED62B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9CA64B33-4C24-49E7-8D7D-2B1A37D1A035}">
+          <x14:cfRule type="dataBar" id="{D2FFA51A-4F14-46D8-98F4-101C1BEE7541}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1BE520ED-089A-473F-A810-560B6DBCC6F1}</x14:id>
+          <x14:id>{8A29CF3C-099A-41C5-B5D3-9E94E6364AFC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0836A528-1DA5-4670-B1A7-205934B3CAEC}</x14:id>
+          <x14:id>{B5ECA05F-1433-4F5A-A1EA-C77A6395EEBC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{887E71B7-BB09-48EC-A32C-91BE11076976}</x14:id>
+          <x14:id>{A67F384A-1C38-4F90-8D4B-23BCFDDC6624}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7D99927B-AFE7-4EF3-8116-1ADC382B1629}</x14:id>
+          <x14:id>{55F5ACD0-02C1-482F-B65C-37EB08ADFAD2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1BE520ED-089A-473F-A810-560B6DBCC6F1}">
+          <x14:cfRule type="dataBar" id="{8A29CF3C-099A-41C5-B5D3-9E94E6364AFC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0836A528-1DA5-4670-B1A7-205934B3CAEC}">
+          <x14:cfRule type="dataBar" id="{B5ECA05F-1433-4F5A-A1EA-C77A6395EEBC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{887E71B7-BB09-48EC-A32C-91BE11076976}">
+          <x14:cfRule type="dataBar" id="{A67F384A-1C38-4F90-8D4B-23BCFDDC6624}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7D99927B-AFE7-4EF3-8116-1ADC382B1629}">
+          <x14:cfRule type="dataBar" id="{55F5ACD0-02C1-482F-B65C-37EB08ADFAD2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2055CE40-0B3A-437B-8A2F-4779886D3367}</x14:id>
+          <x14:id>{252B592A-B082-488D-8CB8-E13F41783533}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F844DFA2-A65B-48F3-92F9-757BC4B93851}</x14:id>
+          <x14:id>{2BB9114A-F143-4B5E-BA69-6612EB1877E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1DD67F2F-EA9A-40C8-99A2-33F0D39ED62B}</x14:id>
+          <x14:id>{BEE22F85-F6E2-45DD-92D3-540CB6437000}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D2FFA51A-4F14-46D8-98F4-101C1BEE7541}</x14:id>
+          <x14:id>{DC7579BB-16C0-40E4-8F59-8B07B46FAB75}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2055CE40-0B3A-437B-8A2F-4779886D3367}">
+          <x14:cfRule type="dataBar" id="{252B592A-B082-488D-8CB8-E13F41783533}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F844DFA2-A65B-48F3-92F9-757BC4B93851}">
+          <x14:cfRule type="dataBar" id="{2BB9114A-F143-4B5E-BA69-6612EB1877E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1DD67F2F-EA9A-40C8-99A2-33F0D39ED62B}">
+          <x14:cfRule type="dataBar" id="{BEE22F85-F6E2-45DD-92D3-540CB6437000}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D2FFA51A-4F14-46D8-98F4-101C1BEE7541}">
+          <x14:cfRule type="dataBar" id="{DC7579BB-16C0-40E4-8F59-8B07B46FAB75}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8A29CF3C-099A-41C5-B5D3-9E94E6364AFC}</x14:id>
+          <x14:id>{5D1E0B3D-D4E6-4522-A8E4-393E9A8BD742}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B5ECA05F-1433-4F5A-A1EA-C77A6395EEBC}</x14:id>
+          <x14:id>{C26A350D-C3BC-4A32-AD9A-012E4FA6CF3E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A67F384A-1C38-4F90-8D4B-23BCFDDC6624}</x14:id>
+          <x14:id>{BE1FB0B3-DFE7-418D-81F6-B44E8A591D80}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{55F5ACD0-02C1-482F-B65C-37EB08ADFAD2}</x14:id>
+          <x14:id>{3AB1CB8D-211E-4335-9DD5-D38EADB3F67A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8A29CF3C-099A-41C5-B5D3-9E94E6364AFC}">
+          <x14:cfRule type="dataBar" id="{5D1E0B3D-D4E6-4522-A8E4-393E9A8BD742}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B5ECA05F-1433-4F5A-A1EA-C77A6395EEBC}">
+          <x14:cfRule type="dataBar" id="{C26A350D-C3BC-4A32-AD9A-012E4FA6CF3E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A67F384A-1C38-4F90-8D4B-23BCFDDC6624}">
+          <x14:cfRule type="dataBar" id="{BE1FB0B3-DFE7-418D-81F6-B44E8A591D80}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{55F5ACD0-02C1-482F-B65C-37EB08ADFAD2}">
+          <x14:cfRule type="dataBar" id="{3AB1CB8D-211E-4335-9DD5-D38EADB3F67A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{252B592A-B082-488D-8CB8-E13F41783533}</x14:id>
+          <x14:id>{27CF9A45-7554-48BD-932D-A87C5A420AC9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2BB9114A-F143-4B5E-BA69-6612EB1877E9}</x14:id>
+          <x14:id>{FED67B75-40D8-4EF3-80DC-F6AF502EC761}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BEE22F85-F6E2-45DD-92D3-540CB6437000}</x14:id>
+          <x14:id>{F619B6F7-634B-4944-803C-20112C04C79E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DC7579BB-16C0-40E4-8F59-8B07B46FAB75}</x14:id>
+          <x14:id>{79469FD8-E7AE-4502-8AF1-5BEA662E449E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{252B592A-B082-488D-8CB8-E13F41783533}">
+          <x14:cfRule type="dataBar" id="{27CF9A45-7554-48BD-932D-A87C5A420AC9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2BB9114A-F143-4B5E-BA69-6612EB1877E9}">
+          <x14:cfRule type="dataBar" id="{FED67B75-40D8-4EF3-80DC-F6AF502EC761}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BEE22F85-F6E2-45DD-92D3-540CB6437000}">
+          <x14:cfRule type="dataBar" id="{F619B6F7-634B-4944-803C-20112C04C79E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DC7579BB-16C0-40E4-8F59-8B07B46FAB75}">
+          <x14:cfRule type="dataBar" id="{79469FD8-E7AE-4502-8AF1-5BEA662E449E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5D1E0B3D-D4E6-4522-A8E4-393E9A8BD742}</x14:id>
+          <x14:id>{7EA83347-C158-4919-846D-F7E5EE616BDC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C26A350D-C3BC-4A32-AD9A-012E4FA6CF3E}</x14:id>
+          <x14:id>{F257620D-AA2D-4EC2-BD30-DF50279D467B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BE1FB0B3-DFE7-418D-81F6-B44E8A591D80}</x14:id>
+          <x14:id>{C6D76804-0846-4E13-9333-71116D79B1A5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3AB1CB8D-211E-4335-9DD5-D38EADB3F67A}</x14:id>
+          <x14:id>{A23FB3EF-5A66-4A85-9777-5C30FA102708}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5D1E0B3D-D4E6-4522-A8E4-393E9A8BD742}">
+          <x14:cfRule type="dataBar" id="{7EA83347-C158-4919-846D-F7E5EE616BDC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C26A350D-C3BC-4A32-AD9A-012E4FA6CF3E}">
+          <x14:cfRule type="dataBar" id="{F257620D-AA2D-4EC2-BD30-DF50279D467B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BE1FB0B3-DFE7-418D-81F6-B44E8A591D80}">
+          <x14:cfRule type="dataBar" id="{C6D76804-0846-4E13-9333-71116D79B1A5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3AB1CB8D-211E-4335-9DD5-D38EADB3F67A}">
+          <x14:cfRule type="dataBar" id="{A23FB3EF-5A66-4A85-9777-5C30FA102708}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 08:56Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27CF9A45-7554-48BD-932D-A87C5A420AC9}</x14:id>
+          <x14:id>{9E1F7E03-D82E-424D-B04C-B15B9C8A0B17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FED67B75-40D8-4EF3-80DC-F6AF502EC761}</x14:id>
+          <x14:id>{CE136404-8DF7-4B83-9528-09DA906C3D9F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F619B6F7-634B-4944-803C-20112C04C79E}</x14:id>
+          <x14:id>{052E9841-3B34-4692-BCDD-830FE5D8EA3B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79469FD8-E7AE-4502-8AF1-5BEA662E449E}</x14:id>
+          <x14:id>{E5942922-A063-46F4-B6AD-20C585C424FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27CF9A45-7554-48BD-932D-A87C5A420AC9}">
+          <x14:cfRule type="dataBar" id="{9E1F7E03-D82E-424D-B04C-B15B9C8A0B17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FED67B75-40D8-4EF3-80DC-F6AF502EC761}">
+          <x14:cfRule type="dataBar" id="{CE136404-8DF7-4B83-9528-09DA906C3D9F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F619B6F7-634B-4944-803C-20112C04C79E}">
+          <x14:cfRule type="dataBar" id="{052E9841-3B34-4692-BCDD-830FE5D8EA3B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79469FD8-E7AE-4502-8AF1-5BEA662E449E}">
+          <x14:cfRule type="dataBar" id="{E5942922-A063-46F4-B6AD-20C585C424FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7EA83347-C158-4919-846D-F7E5EE616BDC}</x14:id>
+          <x14:id>{B486EA0B-8798-464C-96FA-EFD00971D69D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F257620D-AA2D-4EC2-BD30-DF50279D467B}</x14:id>
+          <x14:id>{889F9588-3DA1-4084-9B02-A0CD8CD3B8B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6D76804-0846-4E13-9333-71116D79B1A5}</x14:id>
+          <x14:id>{05BAB5EE-3157-413C-8587-66D461D1BC9C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A23FB3EF-5A66-4A85-9777-5C30FA102708}</x14:id>
+          <x14:id>{66D71849-614A-4345-98A7-10EA61EBBFAA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7EA83347-C158-4919-846D-F7E5EE616BDC}">
+          <x14:cfRule type="dataBar" id="{B486EA0B-8798-464C-96FA-EFD00971D69D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F257620D-AA2D-4EC2-BD30-DF50279D467B}">
+          <x14:cfRule type="dataBar" id="{889F9588-3DA1-4084-9B02-A0CD8CD3B8B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6D76804-0846-4E13-9333-71116D79B1A5}">
+          <x14:cfRule type="dataBar" id="{05BAB5EE-3157-413C-8587-66D461D1BC9C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A23FB3EF-5A66-4A85-9777-5C30FA102708}">
+          <x14:cfRule type="dataBar" id="{66D71849-614A-4345-98A7-10EA61EBBFAA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9E1F7E03-D82E-424D-B04C-B15B9C8A0B17}</x14:id>
+          <x14:id>{AA1316DD-1311-4528-B827-E4A6C1CDA62A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CE136404-8DF7-4B83-9528-09DA906C3D9F}</x14:id>
+          <x14:id>{7EFC6A89-F994-4148-A546-5713E369358F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{052E9841-3B34-4692-BCDD-830FE5D8EA3B}</x14:id>
+          <x14:id>{5111B66F-B15A-45E3-976D-6CB7889FEDB6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E5942922-A063-46F4-B6AD-20C585C424FC}</x14:id>
+          <x14:id>{D2DE1928-5720-42DC-A69C-BEE228E94B01}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9E1F7E03-D82E-424D-B04C-B15B9C8A0B17}">
+          <x14:cfRule type="dataBar" id="{AA1316DD-1311-4528-B827-E4A6C1CDA62A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CE136404-8DF7-4B83-9528-09DA906C3D9F}">
+          <x14:cfRule type="dataBar" id="{7EFC6A89-F994-4148-A546-5713E369358F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{052E9841-3B34-4692-BCDD-830FE5D8EA3B}">
+          <x14:cfRule type="dataBar" id="{5111B66F-B15A-45E3-976D-6CB7889FEDB6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E5942922-A063-46F4-B6AD-20C585C424FC}">
+          <x14:cfRule type="dataBar" id="{D2DE1928-5720-42DC-A69C-BEE228E94B01}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B486EA0B-8798-464C-96FA-EFD00971D69D}</x14:id>
+          <x14:id>{FE0B1FA8-717F-403A-A146-D307A5D33918}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{889F9588-3DA1-4084-9B02-A0CD8CD3B8B0}</x14:id>
+          <x14:id>{3D76B48E-0E26-4335-BF3A-03489CC2EDFE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05BAB5EE-3157-413C-8587-66D461D1BC9C}</x14:id>
+          <x14:id>{6E8203FB-7904-4041-B54D-9DDA2E94AB0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66D71849-614A-4345-98A7-10EA61EBBFAA}</x14:id>
+          <x14:id>{3B96F22B-DB3D-4053-B132-8D1122FF78BF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B486EA0B-8798-464C-96FA-EFD00971D69D}">
+          <x14:cfRule type="dataBar" id="{FE0B1FA8-717F-403A-A146-D307A5D33918}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{889F9588-3DA1-4084-9B02-A0CD8CD3B8B0}">
+          <x14:cfRule type="dataBar" id="{3D76B48E-0E26-4335-BF3A-03489CC2EDFE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05BAB5EE-3157-413C-8587-66D461D1BC9C}">
+          <x14:cfRule type="dataBar" id="{6E8203FB-7904-4041-B54D-9DDA2E94AB0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66D71849-614A-4345-98A7-10EA61EBBFAA}">
+          <x14:cfRule type="dataBar" id="{3B96F22B-DB3D-4053-B132-8D1122FF78BF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA1316DD-1311-4528-B827-E4A6C1CDA62A}</x14:id>
+          <x14:id>{2D711A45-BDDD-45C0-A33C-731AF4F4B456}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7EFC6A89-F994-4148-A546-5713E369358F}</x14:id>
+          <x14:id>{26760BFE-180D-46B9-A009-ECD58C13B04C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5111B66F-B15A-45E3-976D-6CB7889FEDB6}</x14:id>
+          <x14:id>{2C36CD71-654E-4A9E-B16A-0EA6DBC2BED6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D2DE1928-5720-42DC-A69C-BEE228E94B01}</x14:id>
+          <x14:id>{D10E4FA4-AB80-41DA-A541-4D06E39A5D95}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA1316DD-1311-4528-B827-E4A6C1CDA62A}">
+          <x14:cfRule type="dataBar" id="{2D711A45-BDDD-45C0-A33C-731AF4F4B456}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7EFC6A89-F994-4148-A546-5713E369358F}">
+          <x14:cfRule type="dataBar" id="{26760BFE-180D-46B9-A009-ECD58C13B04C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5111B66F-B15A-45E3-976D-6CB7889FEDB6}">
+          <x14:cfRule type="dataBar" id="{2C36CD71-654E-4A9E-B16A-0EA6DBC2BED6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D2DE1928-5720-42DC-A69C-BEE228E94B01}">
+          <x14:cfRule type="dataBar" id="{D10E4FA4-AB80-41DA-A541-4D06E39A5D95}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE0B1FA8-717F-403A-A146-D307A5D33918}</x14:id>
+          <x14:id>{6D0E7306-4F31-42CF-B91C-A08504E520B9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D76B48E-0E26-4335-BF3A-03489CC2EDFE}</x14:id>
+          <x14:id>{C1E2736A-0FEA-4504-B0AC-B476EA33BE8F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6E8203FB-7904-4041-B54D-9DDA2E94AB0B}</x14:id>
+          <x14:id>{06DD23CA-7483-4261-AE37-97971DF79C6E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3B96F22B-DB3D-4053-B132-8D1122FF78BF}</x14:id>
+          <x14:id>{D89AA3E7-EE74-4800-B626-9359780AE4A1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE0B1FA8-717F-403A-A146-D307A5D33918}">
+          <x14:cfRule type="dataBar" id="{6D0E7306-4F31-42CF-B91C-A08504E520B9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D76B48E-0E26-4335-BF3A-03489CC2EDFE}">
+          <x14:cfRule type="dataBar" id="{C1E2736A-0FEA-4504-B0AC-B476EA33BE8F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6E8203FB-7904-4041-B54D-9DDA2E94AB0B}">
+          <x14:cfRule type="dataBar" id="{06DD23CA-7483-4261-AE37-97971DF79C6E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3B96F22B-DB3D-4053-B132-8D1122FF78BF}">
+          <x14:cfRule type="dataBar" id="{D89AA3E7-EE74-4800-B626-9359780AE4A1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D711A45-BDDD-45C0-A33C-731AF4F4B456}</x14:id>
+          <x14:id>{E4EBDBC4-9C59-4580-940A-0142FFA88E2B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26760BFE-180D-46B9-A009-ECD58C13B04C}</x14:id>
+          <x14:id>{54047CFF-785A-4C74-928C-D701D3E05EC8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C36CD71-654E-4A9E-B16A-0EA6DBC2BED6}</x14:id>
+          <x14:id>{38D9826B-4343-4A7E-904F-B8CEC8D4745A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D10E4FA4-AB80-41DA-A541-4D06E39A5D95}</x14:id>
+          <x14:id>{F4DCFBF7-3CCB-4F7F-9FE4-018FC3C81D06}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D711A45-BDDD-45C0-A33C-731AF4F4B456}">
+          <x14:cfRule type="dataBar" id="{E4EBDBC4-9C59-4580-940A-0142FFA88E2B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26760BFE-180D-46B9-A009-ECD58C13B04C}">
+          <x14:cfRule type="dataBar" id="{54047CFF-785A-4C74-928C-D701D3E05EC8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C36CD71-654E-4A9E-B16A-0EA6DBC2BED6}">
+          <x14:cfRule type="dataBar" id="{38D9826B-4343-4A7E-904F-B8CEC8D4745A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D10E4FA4-AB80-41DA-A541-4D06E39A5D95}">
+          <x14:cfRule type="dataBar" id="{F4DCFBF7-3CCB-4F7F-9FE4-018FC3C81D06}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D0E7306-4F31-42CF-B91C-A08504E520B9}</x14:id>
+          <x14:id>{CBC90CB2-89FC-4AC4-B8E6-99D8DA7F6433}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C1E2736A-0FEA-4504-B0AC-B476EA33BE8F}</x14:id>
+          <x14:id>{2EC67EE7-6744-4447-9E31-17A7855EF455}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{06DD23CA-7483-4261-AE37-97971DF79C6E}</x14:id>
+          <x14:id>{41801D47-BDB7-4238-83C2-DBB2358A78A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D89AA3E7-EE74-4800-B626-9359780AE4A1}</x14:id>
+          <x14:id>{1DB8C621-5428-4FF7-9C49-9D89205B677C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D0E7306-4F31-42CF-B91C-A08504E520B9}">
+          <x14:cfRule type="dataBar" id="{CBC90CB2-89FC-4AC4-B8E6-99D8DA7F6433}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C1E2736A-0FEA-4504-B0AC-B476EA33BE8F}">
+          <x14:cfRule type="dataBar" id="{2EC67EE7-6744-4447-9E31-17A7855EF455}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{06DD23CA-7483-4261-AE37-97971DF79C6E}">
+          <x14:cfRule type="dataBar" id="{41801D47-BDB7-4238-83C2-DBB2358A78A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D89AA3E7-EE74-4800-B626-9359780AE4A1}">
+          <x14:cfRule type="dataBar" id="{1DB8C621-5428-4FF7-9C49-9D89205B677C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4EBDBC4-9C59-4580-940A-0142FFA88E2B}</x14:id>
+          <x14:id>{B28A04A6-FAB1-4292-9ECD-58AC6C62FE8A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{54047CFF-785A-4C74-928C-D701D3E05EC8}</x14:id>
+          <x14:id>{8CB88C6B-82E1-4AC6-BE58-84ED85E05AF8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38D9826B-4343-4A7E-904F-B8CEC8D4745A}</x14:id>
+          <x14:id>{CB73C978-2E42-40E8-9140-E2CA4625B1AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F4DCFBF7-3CCB-4F7F-9FE4-018FC3C81D06}</x14:id>
+          <x14:id>{38781DE4-5A38-4483-AF68-F1A53086C764}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4EBDBC4-9C59-4580-940A-0142FFA88E2B}">
+          <x14:cfRule type="dataBar" id="{B28A04A6-FAB1-4292-9ECD-58AC6C62FE8A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{54047CFF-785A-4C74-928C-D701D3E05EC8}">
+          <x14:cfRule type="dataBar" id="{8CB88C6B-82E1-4AC6-BE58-84ED85E05AF8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38D9826B-4343-4A7E-904F-B8CEC8D4745A}">
+          <x14:cfRule type="dataBar" id="{CB73C978-2E42-40E8-9140-E2CA4625B1AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F4DCFBF7-3CCB-4F7F-9FE4-018FC3C81D06}">
+          <x14:cfRule type="dataBar" id="{38781DE4-5A38-4483-AF68-F1A53086C764}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CBC90CB2-89FC-4AC4-B8E6-99D8DA7F6433}</x14:id>
+          <x14:id>{7C9A680A-AE16-4DB5-B77C-8856F3DA743A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2EC67EE7-6744-4447-9E31-17A7855EF455}</x14:id>
+          <x14:id>{0F3D70B4-FC8A-4F24-A413-6C7B4178CEC6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{41801D47-BDB7-4238-83C2-DBB2358A78A8}</x14:id>
+          <x14:id>{53D7060F-3B90-49A1-95A7-DF0E6E530C0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1DB8C621-5428-4FF7-9C49-9D89205B677C}</x14:id>
+          <x14:id>{C678A929-6080-40F4-82F9-D154F1A8E787}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CBC90CB2-89FC-4AC4-B8E6-99D8DA7F6433}">
+          <x14:cfRule type="dataBar" id="{7C9A680A-AE16-4DB5-B77C-8856F3DA743A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2EC67EE7-6744-4447-9E31-17A7855EF455}">
+          <x14:cfRule type="dataBar" id="{0F3D70B4-FC8A-4F24-A413-6C7B4178CEC6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{41801D47-BDB7-4238-83C2-DBB2358A78A8}">
+          <x14:cfRule type="dataBar" id="{53D7060F-3B90-49A1-95A7-DF0E6E530C0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1DB8C621-5428-4FF7-9C49-9D89205B677C}">
+          <x14:cfRule type="dataBar" id="{C678A929-6080-40F4-82F9-D154F1A8E787}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B28A04A6-FAB1-4292-9ECD-58AC6C62FE8A}</x14:id>
+          <x14:id>{CA355C00-F96C-4CAD-BAFC-E8A7B70FE5E1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8CB88C6B-82E1-4AC6-BE58-84ED85E05AF8}</x14:id>
+          <x14:id>{564D5BF5-F800-434B-8AC4-2E40105B148F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CB73C978-2E42-40E8-9140-E2CA4625B1AB}</x14:id>
+          <x14:id>{D33B0152-AB4B-4926-A766-128F7751485F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38781DE4-5A38-4483-AF68-F1A53086C764}</x14:id>
+          <x14:id>{F080F332-61C9-4ED4-BD9C-13933D891CC1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B28A04A6-FAB1-4292-9ECD-58AC6C62FE8A}">
+          <x14:cfRule type="dataBar" id="{CA355C00-F96C-4CAD-BAFC-E8A7B70FE5E1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8CB88C6B-82E1-4AC6-BE58-84ED85E05AF8}">
+          <x14:cfRule type="dataBar" id="{564D5BF5-F800-434B-8AC4-2E40105B148F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CB73C978-2E42-40E8-9140-E2CA4625B1AB}">
+          <x14:cfRule type="dataBar" id="{D33B0152-AB4B-4926-A766-128F7751485F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38781DE4-5A38-4483-AF68-F1A53086C764}">
+          <x14:cfRule type="dataBar" id="{F080F332-61C9-4ED4-BD9C-13933D891CC1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7C9A680A-AE16-4DB5-B77C-8856F3DA743A}</x14:id>
+          <x14:id>{8843ADCD-83C6-4050-96A3-392C39B2BF25}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F3D70B4-FC8A-4F24-A413-6C7B4178CEC6}</x14:id>
+          <x14:id>{73219CCB-1148-4AAA-A60C-3116450DB6E0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53D7060F-3B90-49A1-95A7-DF0E6E530C0B}</x14:id>
+          <x14:id>{0790123C-96C3-47CB-9FAF-6D460FC34BD2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C678A929-6080-40F4-82F9-D154F1A8E787}</x14:id>
+          <x14:id>{7FA384C6-5C0F-4B8F-AC4C-F7D2B8AE04DB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7C9A680A-AE16-4DB5-B77C-8856F3DA743A}">
+          <x14:cfRule type="dataBar" id="{8843ADCD-83C6-4050-96A3-392C39B2BF25}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0F3D70B4-FC8A-4F24-A413-6C7B4178CEC6}">
+          <x14:cfRule type="dataBar" id="{73219CCB-1148-4AAA-A60C-3116450DB6E0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53D7060F-3B90-49A1-95A7-DF0E6E530C0B}">
+          <x14:cfRule type="dataBar" id="{0790123C-96C3-47CB-9FAF-6D460FC34BD2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C678A929-6080-40F4-82F9-D154F1A8E787}">
+          <x14:cfRule type="dataBar" id="{7FA384C6-5C0F-4B8F-AC4C-F7D2B8AE04DB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CA355C00-F96C-4CAD-BAFC-E8A7B70FE5E1}</x14:id>
+          <x14:id>{F66AC452-2645-4DD9-96EF-189B5BEB43CC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{564D5BF5-F800-434B-8AC4-2E40105B148F}</x14:id>
+          <x14:id>{5EA769A3-EC14-4BB9-A466-2A385799FB85}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D33B0152-AB4B-4926-A766-128F7751485F}</x14:id>
+          <x14:id>{434EAABD-156E-41C1-AEBF-EFECF68F509F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F080F332-61C9-4ED4-BD9C-13933D891CC1}</x14:id>
+          <x14:id>{365FED74-A089-4B5D-AD82-9E649B1C5A2C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CA355C00-F96C-4CAD-BAFC-E8A7B70FE5E1}">
+          <x14:cfRule type="dataBar" id="{F66AC452-2645-4DD9-96EF-189B5BEB43CC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{564D5BF5-F800-434B-8AC4-2E40105B148F}">
+          <x14:cfRule type="dataBar" id="{5EA769A3-EC14-4BB9-A466-2A385799FB85}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D33B0152-AB4B-4926-A766-128F7751485F}">
+          <x14:cfRule type="dataBar" id="{434EAABD-156E-41C1-AEBF-EFECF68F509F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F080F332-61C9-4ED4-BD9C-13933D891CC1}">
+          <x14:cfRule type="dataBar" id="{365FED74-A089-4B5D-AD82-9E649B1C5A2C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8843ADCD-83C6-4050-96A3-392C39B2BF25}</x14:id>
+          <x14:id>{738A2B81-080A-430B-8372-B25632BEE66E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{73219CCB-1148-4AAA-A60C-3116450DB6E0}</x14:id>
+          <x14:id>{D906B1EC-ACA1-483B-95C7-648CC1C48490}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0790123C-96C3-47CB-9FAF-6D460FC34BD2}</x14:id>
+          <x14:id>{E71BEA37-6DF5-40AE-8681-1F7D1C7C9C5E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7FA384C6-5C0F-4B8F-AC4C-F7D2B8AE04DB}</x14:id>
+          <x14:id>{B280965C-11AE-48C2-B39D-423C199A26E4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8843ADCD-83C6-4050-96A3-392C39B2BF25}">
+          <x14:cfRule type="dataBar" id="{738A2B81-080A-430B-8372-B25632BEE66E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{73219CCB-1148-4AAA-A60C-3116450DB6E0}">
+          <x14:cfRule type="dataBar" id="{D906B1EC-ACA1-483B-95C7-648CC1C48490}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0790123C-96C3-47CB-9FAF-6D460FC34BD2}">
+          <x14:cfRule type="dataBar" id="{E71BEA37-6DF5-40AE-8681-1F7D1C7C9C5E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7FA384C6-5C0F-4B8F-AC4C-F7D2B8AE04DB}">
+          <x14:cfRule type="dataBar" id="{B280965C-11AE-48C2-B39D-423C199A26E4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F66AC452-2645-4DD9-96EF-189B5BEB43CC}</x14:id>
+          <x14:id>{8EDE1EB4-FB64-4C8C-A824-A64EDFF9ABF4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5EA769A3-EC14-4BB9-A466-2A385799FB85}</x14:id>
+          <x14:id>{3B0233B3-3BEC-403E-9E71-FBEDBEA3166C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{434EAABD-156E-41C1-AEBF-EFECF68F509F}</x14:id>
+          <x14:id>{CCAE69F8-4A15-4866-B152-0155D09FA683}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{365FED74-A089-4B5D-AD82-9E649B1C5A2C}</x14:id>
+          <x14:id>{24897473-75D5-4AB4-B107-BB968A0BA5A3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F66AC452-2645-4DD9-96EF-189B5BEB43CC}">
+          <x14:cfRule type="dataBar" id="{8EDE1EB4-FB64-4C8C-A824-A64EDFF9ABF4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5EA769A3-EC14-4BB9-A466-2A385799FB85}">
+          <x14:cfRule type="dataBar" id="{3B0233B3-3BEC-403E-9E71-FBEDBEA3166C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{434EAABD-156E-41C1-AEBF-EFECF68F509F}">
+          <x14:cfRule type="dataBar" id="{CCAE69F8-4A15-4866-B152-0155D09FA683}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{365FED74-A089-4B5D-AD82-9E649B1C5A2C}">
+          <x14:cfRule type="dataBar" id="{24897473-75D5-4AB4-B107-BB968A0BA5A3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{738A2B81-080A-430B-8372-B25632BEE66E}</x14:id>
+          <x14:id>{D0D52BB1-A845-46B9-B1C6-366EDAAAA210}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D906B1EC-ACA1-483B-95C7-648CC1C48490}</x14:id>
+          <x14:id>{E8D705E5-0614-4BCB-B847-59EF5F1F1A79}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E71BEA37-6DF5-40AE-8681-1F7D1C7C9C5E}</x14:id>
+          <x14:id>{8DACB61F-850D-455B-9744-DBCBB3053665}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B280965C-11AE-48C2-B39D-423C199A26E4}</x14:id>
+          <x14:id>{CE1FB512-AEF1-461D-A1CB-8E9CA84BAFAE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{738A2B81-080A-430B-8372-B25632BEE66E}">
+          <x14:cfRule type="dataBar" id="{D0D52BB1-A845-46B9-B1C6-366EDAAAA210}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D906B1EC-ACA1-483B-95C7-648CC1C48490}">
+          <x14:cfRule type="dataBar" id="{E8D705E5-0614-4BCB-B847-59EF5F1F1A79}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E71BEA37-6DF5-40AE-8681-1F7D1C7C9C5E}">
+          <x14:cfRule type="dataBar" id="{8DACB61F-850D-455B-9744-DBCBB3053665}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B280965C-11AE-48C2-B39D-423C199A26E4}">
+          <x14:cfRule type="dataBar" id="{CE1FB512-AEF1-461D-A1CB-8E9CA84BAFAE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8EDE1EB4-FB64-4C8C-A824-A64EDFF9ABF4}</x14:id>
+          <x14:id>{9DEE6D95-136F-450E-9BCB-00A476A41FD9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3B0233B3-3BEC-403E-9E71-FBEDBEA3166C}</x14:id>
+          <x14:id>{B8404811-418A-4B76-8C92-C55EC5DB8E2B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CCAE69F8-4A15-4866-B152-0155D09FA683}</x14:id>
+          <x14:id>{E372E9AD-9D3F-447B-B342-CA3DFA1C53CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24897473-75D5-4AB4-B107-BB968A0BA5A3}</x14:id>
+          <x14:id>{95B794F2-5669-4D2E-B684-CFCF17EE0605}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8EDE1EB4-FB64-4C8C-A824-A64EDFF9ABF4}">
+          <x14:cfRule type="dataBar" id="{9DEE6D95-136F-450E-9BCB-00A476A41FD9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3B0233B3-3BEC-403E-9E71-FBEDBEA3166C}">
+          <x14:cfRule type="dataBar" id="{B8404811-418A-4B76-8C92-C55EC5DB8E2B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CCAE69F8-4A15-4866-B152-0155D09FA683}">
+          <x14:cfRule type="dataBar" id="{E372E9AD-9D3F-447B-B342-CA3DFA1C53CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24897473-75D5-4AB4-B107-BB968A0BA5A3}">
+          <x14:cfRule type="dataBar" id="{95B794F2-5669-4D2E-B684-CFCF17EE0605}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0D52BB1-A845-46B9-B1C6-366EDAAAA210}</x14:id>
+          <x14:id>{26F072F8-6B69-4818-B5EE-464696AC0395}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E8D705E5-0614-4BCB-B847-59EF5F1F1A79}</x14:id>
+          <x14:id>{45A7298E-BC3A-463A-878B-2328D7DC4F09}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8DACB61F-850D-455B-9744-DBCBB3053665}</x14:id>
+          <x14:id>{CB05D413-D47F-48CD-9892-0C6A6E32CC7F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CE1FB512-AEF1-461D-A1CB-8E9CA84BAFAE}</x14:id>
+          <x14:id>{D7374CAB-2731-4501-A2FF-8812911CFB89}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0D52BB1-A845-46B9-B1C6-366EDAAAA210}">
+          <x14:cfRule type="dataBar" id="{26F072F8-6B69-4818-B5EE-464696AC0395}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E8D705E5-0614-4BCB-B847-59EF5F1F1A79}">
+          <x14:cfRule type="dataBar" id="{45A7298E-BC3A-463A-878B-2328D7DC4F09}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8DACB61F-850D-455B-9744-DBCBB3053665}">
+          <x14:cfRule type="dataBar" id="{CB05D413-D47F-48CD-9892-0C6A6E32CC7F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CE1FB512-AEF1-461D-A1CB-8E9CA84BAFAE}">
+          <x14:cfRule type="dataBar" id="{D7374CAB-2731-4501-A2FF-8812911CFB89}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9DEE6D95-136F-450E-9BCB-00A476A41FD9}</x14:id>
+          <x14:id>{74FD3970-2033-4DEF-9FF1-963BD349FF2F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B8404811-418A-4B76-8C92-C55EC5DB8E2B}</x14:id>
+          <x14:id>{B62F5B84-7446-417C-AC46-239D4E78996B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E372E9AD-9D3F-447B-B342-CA3DFA1C53CB}</x14:id>
+          <x14:id>{17875260-AE1D-4B12-9242-9A1EEA2DF5CC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95B794F2-5669-4D2E-B684-CFCF17EE0605}</x14:id>
+          <x14:id>{5AA2775B-4BCF-42F7-B12E-F0745084816B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9DEE6D95-136F-450E-9BCB-00A476A41FD9}">
+          <x14:cfRule type="dataBar" id="{74FD3970-2033-4DEF-9FF1-963BD349FF2F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B8404811-418A-4B76-8C92-C55EC5DB8E2B}">
+          <x14:cfRule type="dataBar" id="{B62F5B84-7446-417C-AC46-239D4E78996B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E372E9AD-9D3F-447B-B342-CA3DFA1C53CB}">
+          <x14:cfRule type="dataBar" id="{17875260-AE1D-4B12-9242-9A1EEA2DF5CC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95B794F2-5669-4D2E-B684-CFCF17EE0605}">
+          <x14:cfRule type="dataBar" id="{5AA2775B-4BCF-42F7-B12E-F0745084816B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26F072F8-6B69-4818-B5EE-464696AC0395}</x14:id>
+          <x14:id>{01697CA3-EA88-46F2-9D1E-86609BBE3562}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{45A7298E-BC3A-463A-878B-2328D7DC4F09}</x14:id>
+          <x14:id>{941A3B6B-2AC5-46E1-891C-F1E1221CAB4A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CB05D413-D47F-48CD-9892-0C6A6E32CC7F}</x14:id>
+          <x14:id>{808E1676-F882-4233-932C-AB681788E90F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D7374CAB-2731-4501-A2FF-8812911CFB89}</x14:id>
+          <x14:id>{42A1FD83-B5DB-4EFF-B7A9-B9F5C758A042}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26F072F8-6B69-4818-B5EE-464696AC0395}">
+          <x14:cfRule type="dataBar" id="{01697CA3-EA88-46F2-9D1E-86609BBE3562}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{45A7298E-BC3A-463A-878B-2328D7DC4F09}">
+          <x14:cfRule type="dataBar" id="{941A3B6B-2AC5-46E1-891C-F1E1221CAB4A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CB05D413-D47F-48CD-9892-0C6A6E32CC7F}">
+          <x14:cfRule type="dataBar" id="{808E1676-F882-4233-932C-AB681788E90F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D7374CAB-2731-4501-A2FF-8812911CFB89}">
+          <x14:cfRule type="dataBar" id="{42A1FD83-B5DB-4EFF-B7A9-B9F5C758A042}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74FD3970-2033-4DEF-9FF1-963BD349FF2F}</x14:id>
+          <x14:id>{74A8EBF2-BD1B-42E3-ACF7-B1D71E11E1C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B62F5B84-7446-417C-AC46-239D4E78996B}</x14:id>
+          <x14:id>{FCD4E522-4E96-4BEE-91F0-2EBCA0B88E0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17875260-AE1D-4B12-9242-9A1EEA2DF5CC}</x14:id>
+          <x14:id>{5D74F85D-78F5-43E6-9F60-2B2673AE2A63}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5AA2775B-4BCF-42F7-B12E-F0745084816B}</x14:id>
+          <x14:id>{4A34071D-EB39-4716-B3F5-C5470C41EF58}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74FD3970-2033-4DEF-9FF1-963BD349FF2F}">
+          <x14:cfRule type="dataBar" id="{74A8EBF2-BD1B-42E3-ACF7-B1D71E11E1C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B62F5B84-7446-417C-AC46-239D4E78996B}">
+          <x14:cfRule type="dataBar" id="{FCD4E522-4E96-4BEE-91F0-2EBCA0B88E0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17875260-AE1D-4B12-9242-9A1EEA2DF5CC}">
+          <x14:cfRule type="dataBar" id="{5D74F85D-78F5-43E6-9F60-2B2673AE2A63}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5AA2775B-4BCF-42F7-B12E-F0745084816B}">
+          <x14:cfRule type="dataBar" id="{4A34071D-EB39-4716-B3F5-C5470C41EF58}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{01697CA3-EA88-46F2-9D1E-86609BBE3562}</x14:id>
+          <x14:id>{22821C00-0188-45E7-9DBF-30CC489823A5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{941A3B6B-2AC5-46E1-891C-F1E1221CAB4A}</x14:id>
+          <x14:id>{970E8EEE-ADB0-4155-B8EE-F6A12D79D1B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{808E1676-F882-4233-932C-AB681788E90F}</x14:id>
+          <x14:id>{1A6465DF-D12B-4220-A088-370F4F903AA1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42A1FD83-B5DB-4EFF-B7A9-B9F5C758A042}</x14:id>
+          <x14:id>{73FFA8D4-004C-4BBA-87FE-D173F71E104B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{01697CA3-EA88-46F2-9D1E-86609BBE3562}">
+          <x14:cfRule type="dataBar" id="{22821C00-0188-45E7-9DBF-30CC489823A5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{941A3B6B-2AC5-46E1-891C-F1E1221CAB4A}">
+          <x14:cfRule type="dataBar" id="{970E8EEE-ADB0-4155-B8EE-F6A12D79D1B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{808E1676-F882-4233-932C-AB681788E90F}">
+          <x14:cfRule type="dataBar" id="{1A6465DF-D12B-4220-A088-370F4F903AA1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42A1FD83-B5DB-4EFF-B7A9-B9F5C758A042}">
+          <x14:cfRule type="dataBar" id="{73FFA8D4-004C-4BBA-87FE-D173F71E104B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74A8EBF2-BD1B-42E3-ACF7-B1D71E11E1C0}</x14:id>
+          <x14:id>{35E8C4F1-F965-4D0F-B3D4-5FB4E3E9856D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FCD4E522-4E96-4BEE-91F0-2EBCA0B88E0B}</x14:id>
+          <x14:id>{20A96AA8-E677-4141-B73E-AAB6D921B944}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5D74F85D-78F5-43E6-9F60-2B2673AE2A63}</x14:id>
+          <x14:id>{6D9A75C7-43DE-406D-BA7A-55F9F8A08B13}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4A34071D-EB39-4716-B3F5-C5470C41EF58}</x14:id>
+          <x14:id>{46CD683F-B6EA-4721-A54F-8AF0CD37850C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74A8EBF2-BD1B-42E3-ACF7-B1D71E11E1C0}">
+          <x14:cfRule type="dataBar" id="{35E8C4F1-F965-4D0F-B3D4-5FB4E3E9856D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FCD4E522-4E96-4BEE-91F0-2EBCA0B88E0B}">
+          <x14:cfRule type="dataBar" id="{20A96AA8-E677-4141-B73E-AAB6D921B944}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5D74F85D-78F5-43E6-9F60-2B2673AE2A63}">
+          <x14:cfRule type="dataBar" id="{6D9A75C7-43DE-406D-BA7A-55F9F8A08B13}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4A34071D-EB39-4716-B3F5-C5470C41EF58}">
+          <x14:cfRule type="dataBar" id="{46CD683F-B6EA-4721-A54F-8AF0CD37850C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22821C00-0188-45E7-9DBF-30CC489823A5}</x14:id>
+          <x14:id>{2372A400-4788-445F-9B97-FDE373FD25A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{970E8EEE-ADB0-4155-B8EE-F6A12D79D1B0}</x14:id>
+          <x14:id>{E9B5C7CD-9895-4B24-9FED-BF06726F2AB4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A6465DF-D12B-4220-A088-370F4F903AA1}</x14:id>
+          <x14:id>{3CF1BA1B-EF33-4BCE-AF6F-8D95BF2AD7EE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{73FFA8D4-004C-4BBA-87FE-D173F71E104B}</x14:id>
+          <x14:id>{A81CCAE7-1C7C-4AB7-BF2D-A179C07F7C8A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22821C00-0188-45E7-9DBF-30CC489823A5}">
+          <x14:cfRule type="dataBar" id="{2372A400-4788-445F-9B97-FDE373FD25A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{970E8EEE-ADB0-4155-B8EE-F6A12D79D1B0}">
+          <x14:cfRule type="dataBar" id="{E9B5C7CD-9895-4B24-9FED-BF06726F2AB4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A6465DF-D12B-4220-A088-370F4F903AA1}">
+          <x14:cfRule type="dataBar" id="{3CF1BA1B-EF33-4BCE-AF6F-8D95BF2AD7EE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{73FFA8D4-004C-4BBA-87FE-D173F71E104B}">
+          <x14:cfRule type="dataBar" id="{A81CCAE7-1C7C-4AB7-BF2D-A179C07F7C8A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-30 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -12867,7 +12867,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{35E8C4F1-F965-4D0F-B3D4-5FB4E3E9856D}</x14:id>
+          <x14:id>{F2CEE630-1C70-40DB-B413-D5E37C32867B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12881,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{20A96AA8-E677-4141-B73E-AAB6D921B944}</x14:id>
+          <x14:id>{488A91F4-5AC9-48C8-9FD0-D6B2104C1FCC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12895,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D9A75C7-43DE-406D-BA7A-55F9F8A08B13}</x14:id>
+          <x14:id>{72DB617C-240E-450E-886D-E358051ECA17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12909,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{46CD683F-B6EA-4721-A54F-8AF0CD37850C}</x14:id>
+          <x14:id>{7AE4C87B-EF67-425B-B120-7C44078A025A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12919,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{35E8C4F1-F965-4D0F-B3D4-5FB4E3E9856D}">
+          <x14:cfRule type="dataBar" id="{F2CEE630-1C70-40DB-B413-D5E37C32867B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12932,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{20A96AA8-E677-4141-B73E-AAB6D921B944}">
+          <x14:cfRule type="dataBar" id="{488A91F4-5AC9-48C8-9FD0-D6B2104C1FCC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12945,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D9A75C7-43DE-406D-BA7A-55F9F8A08B13}">
+          <x14:cfRule type="dataBar" id="{72DB617C-240E-450E-886D-E358051ECA17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12958,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{46CD683F-B6EA-4721-A54F-8AF0CD37850C}">
+          <x14:cfRule type="dataBar" id="{7AE4C87B-EF67-425B-B120-7C44078A025A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28313,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2372A400-4788-445F-9B97-FDE373FD25A0}</x14:id>
+          <x14:id>{512D1E3D-61E8-4E53-8E83-736058DDBE56}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28327,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E9B5C7CD-9895-4B24-9FED-BF06726F2AB4}</x14:id>
+          <x14:id>{934FFBA1-4E90-42C8-8F85-38051440FB7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28341,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CF1BA1B-EF33-4BCE-AF6F-8D95BF2AD7EE}</x14:id>
+          <x14:id>{CA4CA689-0D9C-4D51-8219-D949B8A96AE8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28355,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A81CCAE7-1C7C-4AB7-BF2D-A179C07F7C8A}</x14:id>
+          <x14:id>{EA741A53-6C74-4C8C-8FA7-086C8D042CF6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28365,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2372A400-4788-445F-9B97-FDE373FD25A0}">
+          <x14:cfRule type="dataBar" id="{512D1E3D-61E8-4E53-8E83-736058DDBE56}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28378,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E9B5C7CD-9895-4B24-9FED-BF06726F2AB4}">
+          <x14:cfRule type="dataBar" id="{934FFBA1-4E90-42C8-8F85-38051440FB7D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28391,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CF1BA1B-EF33-4BCE-AF6F-8D95BF2AD7EE}">
+          <x14:cfRule type="dataBar" id="{CA4CA689-0D9C-4D51-8219-D949B8A96AE8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28404,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A81CCAE7-1C7C-4AB7-BF2D-A179C07F7C8A}">
+          <x14:cfRule type="dataBar" id="{EA741A53-6C74-4C8C-8FA7-086C8D042CF6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-10-30 23:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-26.xlsx
+++ b/public/reports/weekly_briefing/2026-10-26.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="46545" yWindow="5250" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="주간 브리핑" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="신고가 근접" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="투자자별 순매수" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="공매도·대차" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="섹터x수급" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="업종별 수급 모멘텀" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="주간 브리핑" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="신고가 근접" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="투자자별 순매수" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공매도·대차" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="섹터x수급" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업종별 수급 모멘텀" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'신고가 근접'!$A$5:$L$22</definedName>
@@ -1071,7 +1071,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 10/23 → 10/29, %</t>
+          <t>미국 종가 기준 10/23 → 10/30, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1140,20 +1140,20 @@
       <c r="D8" s="29" t="n">
         <v>21430</v>
       </c>
-      <c r="E8" s="29" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="G8" s="29" t="n">
-        <v>0.88</v>
+      <c r="E8" s="28" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>-2</v>
       </c>
       <c r="H8" s="28" t="n">
-        <v>-11.57</v>
-      </c>
-      <c r="I8" s="29" t="n">
-        <v>6.85</v>
+        <v>-0.15</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>-0.84</v>
       </c>
     </row>
     <row r="9">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>반도체</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>6.54</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="13">
@@ -1228,11 +1228,11 @@
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>5.52</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="14">
@@ -1248,11 +1248,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>소재</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>3.35</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="15">
@@ -1268,11 +1268,11 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>에너지</t>
+          <t>기술</t>
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-0.89</v>
+        <v>-2.03</v>
       </c>
     </row>
     <row r="16">
@@ -1288,13 +1288,11 @@
       </c>
       <c r="C16" s="31" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>반도체</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>-0.89</v>
       </c>
     </row>
     <row r="17">
@@ -12867,7 +12865,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F2CEE630-1C70-40DB-B413-D5E37C32867B}</x14:id>
+          <x14:id>{24D30112-EF2A-49E3-A960-670FECD23138}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12881,7 +12879,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{488A91F4-5AC9-48C8-9FD0-D6B2104C1FCC}</x14:id>
+          <x14:id>{3586DE15-71EC-4436-A4AF-32C899428896}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12895,7 +12893,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{72DB617C-240E-450E-886D-E358051ECA17}</x14:id>
+          <x14:id>{14CE3994-859D-4028-9839-09861046ECCC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12909,7 +12907,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7AE4C87B-EF67-425B-B120-7C44078A025A}</x14:id>
+          <x14:id>{544C9E75-63CD-4108-A8EC-E2891C91D846}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12919,7 +12917,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F2CEE630-1C70-40DB-B413-D5E37C32867B}">
+          <x14:cfRule type="dataBar" id="{24D30112-EF2A-49E3-A960-670FECD23138}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12932,7 +12930,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{488A91F4-5AC9-48C8-9FD0-D6B2104C1FCC}">
+          <x14:cfRule type="dataBar" id="{3586DE15-71EC-4436-A4AF-32C899428896}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12945,7 +12943,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{72DB617C-240E-450E-886D-E358051ECA17}">
+          <x14:cfRule type="dataBar" id="{14CE3994-859D-4028-9839-09861046ECCC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12958,7 +12956,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7AE4C87B-EF67-425B-B120-7C44078A025A}">
+          <x14:cfRule type="dataBar" id="{544C9E75-63CD-4108-A8EC-E2891C91D846}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28313,7 +28311,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{512D1E3D-61E8-4E53-8E83-736058DDBE56}</x14:id>
+          <x14:id>{21A7E96D-E7BF-4A8C-BFEE-71AB719EFAC0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28327,7 +28325,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{934FFBA1-4E90-42C8-8F85-38051440FB7D}</x14:id>
+          <x14:id>{1539C275-AA46-49B4-AD71-D48F7A503AA2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28341,7 +28339,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CA4CA689-0D9C-4D51-8219-D949B8A96AE8}</x14:id>
+          <x14:id>{2D5FBD33-F305-4FCB-945A-9E853A1D7588}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28355,7 +28353,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EA741A53-6C74-4C8C-8FA7-086C8D042CF6}</x14:id>
+          <x14:id>{D1393B58-0E6F-42FD-B904-8E4407142693}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28365,7 +28363,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{512D1E3D-61E8-4E53-8E83-736058DDBE56}">
+          <x14:cfRule type="dataBar" id="{21A7E96D-E7BF-4A8C-BFEE-71AB719EFAC0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28378,7 +28376,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{934FFBA1-4E90-42C8-8F85-38051440FB7D}">
+          <x14:cfRule type="dataBar" id="{1539C275-AA46-49B4-AD71-D48F7A503AA2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28391,7 +28389,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CA4CA689-0D9C-4D51-8219-D949B8A96AE8}">
+          <x14:cfRule type="dataBar" id="{2D5FBD33-F305-4FCB-945A-9E853A1D7588}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -28404,7 +28402,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EA741A53-6C74-4C8C-8FA7-086C8D042CF6}">
+          <x14:cfRule type="dataBar" id="{D1393B58-0E6F-42FD-B904-8E4407142693}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>